<commit_message>
Scenariusze testowe: dodaj arkusz dla weryfikatora Niedobor normy okresu rozliczeniowego
Nowy arkusz "Niedobor normy okresu rozl." z 11 scenariuszami testowymi dla
weryfikatora DefWeryfKalend ID 40 (Rodzaj=Plan pracy), w tym samym formacie
kolumn co pozostale arkusze (Lp / Scenariusz / Dane wejsciowe / Oczekiwany
wynik / Oczekiwany komunikat / Zweryfikowano na zywo / Wynik testu / Uwagi
z testu). Zaktualizowano arkusz "Informacje" o piaty weryfikator i odnosnik
do dokumentacji.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017fSe2QNxttb6ma8QnXkfML
</commit_message>
<xml_diff>
--- a/Weryfikatory czasu pracy/Scenariusze testowe weryfikatorow czasu pracy.xlsx
+++ b/Weryfikatory czasu pracy/Scenariusze testowe weryfikatorow czasu pracy.xlsx
@@ -7,7 +7,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="Informacje" sheetId="1" r:id="rId1"/>
@@ -15,6 +15,7 @@
     <sheet name="Norma okresu rozliczeniowego" sheetId="3" r:id="rId3"/>
     <sheet name="Ilość dni wolnych" sheetId="4" r:id="rId4"/>
     <sheet name="Odpoczynek dobowy 11h" sheetId="6" r:id="rId5"/>
+    <sheet name="Niedobór normy okresu rozl." sheetId="8" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Okres zatrudnienia'!$A$4:$H$14</definedName>
@@ -32,12 +33,12 @@
     <t>Scenariusze testowe – weryfikatory czasu pracy</t>
   </si>
   <si>
-    <t>Zakres: cztery weryfikatory z folderu „Weryfikatory czasu pracy”, każdy na osobnym arkuszu.</t>
-  </si>
-  <si>
     <t/>
   </si>
   <si>
+    <t>Zakres: pięć weryfikatorów z folderu „Weryfikatory czasu pracy”, każdy na osobnym arkuszu.</t>
+  </si>
+  <si>
     <t>Arkusze:</t>
   </si>
   <si>
@@ -53,6 +54,9 @@
     <t>• Odpoczynek dobowy 11h – weryfikator dnia planu pracy; 11 h odpoczynku liczone w ramach JEDNEJ doby pracowniczej (24 h), + kontrola dnia poprzedniego.</t>
   </si>
   <si>
+    <t>• Niedobór normy okresu rozl. – weryfikator planu pracy (Rodzaj=Plan, ID 40 w bazie Claude); dopełnia wbudowany weryfikator normy okresu rozliczeniowego o wykrywanie NIEDOBORU godzin niemożliwego do nadrobienia w pozostałych miesiącach okresu. Uruchamia się przy KAŻDYM zapisie dnia planu. W bazie Claude jeszcze nie podpięty do żadnego kalendarza (nieaktywny).</t>
+  </si>
+  <si>
     <t>Kolumny na arkuszach scenariuszy:</t>
   </si>
   <si>
@@ -98,7 +102,10 @@
     <t>Weryfikatory czasu pracy/11-sto godzinny odpoczynek.md</t>
   </si>
   <si>
-    <t>Wygenerowano: 2026-09-10</t>
+    <t>Weryfikatory czasu pracy/Niedobór normy okresu rozliczeniowego.md (pkt 5)</t>
+  </si>
+  <si>
+    <t>Wygenerowano: 2026-09-10, zaktualizowano: 2026-09-28</t>
   </si>
   <si>
     <t>Weryfikator: Okres zatrudnienia</t>
@@ -593,6 +600,140 @@
   </si>
   <si>
     <t>Zgłoszone przez użytkownika jako brak komunikatu; usunięto znane ograniczenie - dodano dociąganie wczesnorannych stref dnia następnego do okna doby (patrz .md, commit fix) Zweryfikowano w GUI klienta 2026-09-11 - komunikat pojawia się poprawnie. Zadanie zamknięte.</t>
+  </si>
+  <si>
+    <t>Scenariusze testowe - Niedobór normy okresu rozliczeniowego (weryfikator planu pracy, ID 40 w bazie Claude)</t>
+  </si>
+  <si>
+    <t>Uzupełnia wbudowany weryfikator "Norma w okresie rozliczeniowym" (wykrywa tylko nadmiar) o wykrywanie NIEDOBORU godzin, którego nie da się już nadrobić w pozostałych miesiącach okresu rozliczeniowego. Rodzaj = Plan pracy - uruchamia się przy KAŻDYM zapisie dnia planu (nie tylko na koniec miesiąca), sprawdzając zakres od początku okresu do końca miesiąca edytowanego dnia. GUID 0015552D-B8E6-4609-8928-FC98CCC0F35B. W bazie Claude NIE jest jeszcze podpięty do żadnego kalendarza (WeryfKalend bez wiersza Definicja=40) - obecnie nieaktywny. Kolumny "Wynik testu / Uwagi z testu" - do wypełnienia po teście w GUI.</t>
+  </si>
+  <si>
+    <t>Okres jednomiesięczny, plan dokładnie równy normie kodeksowej</t>
+  </si>
+  <si>
+    <t>Okres rozliczeniowy = 1 miesiąc
+Zaplanowano dokładnie tyle godzin, ile wynosi norma kodeksowa miesiąca</t>
+  </si>
+  <si>
+    <t>- (deficyt &lt;= 0)</t>
+  </si>
+  <si>
+    <t>Nie - wynika z kodu</t>
+  </si>
+  <si>
+    <t>Okres jednomiesięczny (= ostatni miesiąc okresu), realny niedobór</t>
+  </si>
+  <si>
+    <t>Okres rozliczeniowy = 1 miesiąc
+Zaplanowano wyraźnie mniej niż norma kodeksowa</t>
+  </si>
+  <si>
+    <t>Zaplanowano za malo godzin do miesiaca {miesiąc} (brakuje {niedobór}); w pozostalych miesiacach okresu rozliczeniowego {} maksymalna mozliwa kompensacja to 0:00 - {pracownik}
+(brak kolejnego miesiąca -&gt; maxKompensacja = 0)</t>
+  </si>
+  <si>
+    <t>Okres 3-miesięczny, edycja miesiąca 1, duży niedobór, ale możliwy do odrobienia</t>
+  </si>
+  <si>
+    <t>Okres 3-mies. (np. system równoważny)
+Miesiąc 1: mocno niedoplanowany
+Miesiące 2-3: bez zmian (domyślny rozkład z kalendarza wzorcowego, pełne dni robocze)</t>
+  </si>
+  <si>
+    <t>- (niedobór &lt;= teoretyczna rezerwa miesięcy 2-3: dni robocze x norma dobowa etatu - norma kodeksowa tych miesięcy)</t>
+  </si>
+  <si>
+    <t>Okres 3-miesięczny, edycja miesiąca 1, niedobór niemożliwy do odrobienia</t>
+  </si>
+  <si>
+    <t>Jak w scen. 3, ale miesiąc 1 wyzerowany (0 godzin) lub prawie wyzerowany - niedobór przekracza teoretyczną rezerwę miesięcy 2-3</t>
+  </si>
+  <si>
+    <t>Zaplanowano za malo godzin do miesiaca {miesiąc 1} (brakuje {niedobór}); w pozostalych miesiacach okresu rozliczeniowego {miesiące 2-3} maksymalna mozliwa kompensacja to {rezerwa} - {pracownik}</t>
+  </si>
+  <si>
+    <t>Okres 3-miesięczny, edycja ostatniego miesiąca (3), skumulowany niedobór z całego okresu</t>
+  </si>
+  <si>
+    <t>Miesiące 1-2 niedoplanowane, edycja dowolnego dnia w miesiącu 3</t>
+  </si>
+  <si>
+    <t>Błąd (jeśli skumulowany niedobór okres.From -&gt; koniec miesiąca 3 &gt; 0)</t>
+  </si>
+  <si>
+    <t>jw. - maksymalna mozliwa kompensacja to 0:00 (startPo &gt; okres.To, brak kolejnych miesięcy)</t>
+  </si>
+  <si>
+    <t>Granica: niedobór dokładnie równy maksymalnej kompensacji</t>
+  </si>
+  <si>
+    <t>Okres wielomiesięczny; niedobór miesiąca bieżącego == maksymalna teoretyczna rezerwa pozostałych miesięcy (co do minuty)</t>
+  </si>
+  <si>
+    <t>- (warunek to deficyt &gt; maxKompensacja, ostry - równość nie generuje błędu)</t>
+  </si>
+  <si>
+    <t>Zwolnienie pracownika w trakcie pozostałych miesięcy okresu</t>
+  </si>
+  <si>
+    <t>Okres wielomiesięczny, niedobór w miesiącu bieżącym; etat pracownika kończy się w trakcie miesięcy 2-3 (przed końcem okresu)</t>
+  </si>
+  <si>
+    <t>Błąd przy mniejszym niedoborze niż w scen. 3</t>
+  </si>
+  <si>
+    <t>jw. - maksymalna kompensacja pomniejszona (dni po zwolnieniu nie liczą się do rezerwy: pracownik[d]==null lub .Etat==null)</t>
+  </si>
+  <si>
+    <t>Święto ustawowe w pozostałych miesiącach okresu</t>
+  </si>
+  <si>
+    <t>Okres wielomiesięczny z niedoborem; w pozostałych miesiącach dzień ustawowo wolny wypada w dzień roboczy</t>
+  </si>
+  <si>
+    <t>Rezerwa mniejsza o normę dobową za każde takie święto</t>
+  </si>
+  <si>
+    <t>- / Błąd zależnie od wielkości niedoboru (NormaTeoretycznaBezSwiat pomija dni świąteczne z Date.Holidays)</t>
+  </si>
+  <si>
+    <t>Miesiąc jeszcze nietknięty przez planistę</t>
+  </si>
+  <si>
+    <t>Okres wielomiesięczny; edycja dnia w miesiącu 1, miesiące 2-3 bez żadnej ręcznej ingerencji</t>
+  </si>
+  <si>
+    <t>"Zaplanowano" dla miesięcy 2-3 liczone z bieżącego stanu kalendarza planu (zwykle = domyślny rozkład z kalendarza wzorcowego), nie z zera</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>Edycja pojedynczego dnia w środku okresu (nie na końcu miesiąca)</t>
+  </si>
+  <si>
+    <t>Okres wielomiesięczny; zmiana jednego dnia roboczego w środku miesiąca 1</t>
+  </si>
+  <si>
+    <t>Weryfikator i tak się uruchamia i liczy zakres do końca CAŁEGO miesiąca edytowanego dnia (nie tylko do tego dnia)</t>
+  </si>
+  <si>
+    <t>zależnie od sumy narastająco od początku okresu</t>
+  </si>
+  <si>
+    <t>11</t>
+  </si>
+  <si>
+    <t>Definicja nie podpięta do kalendarza (stan bieżący w bazie Claude)</t>
+  </si>
+  <si>
+    <t>Dowolny zapis dnia planu na dowolnym kalendarzu</t>
+  </si>
+  <si>
+    <t>Brak jakiegokolwiek efektu</t>
+  </si>
+  <si>
+    <t>- (WeryfKalend nie ma wiersza z Definicja=40, GetWeryfikatory(Plan) nigdy jej nie zwróci)</t>
   </si>
 </sst>
 </file>
@@ -698,7 +839,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -735,6 +876,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1044,14 +1188,19 @@
         <v>0</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+    </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -1081,12 +1230,12 @@
     </row>
     <row r="10">
       <c r="A10" s="3" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
@@ -1121,12 +1270,12 @@
     </row>
     <row r="18">
       <c r="A18" s="3" t="s">
-        <v>2</v>
+        <v>15</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="s">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20">
@@ -1141,12 +1290,12 @@
     </row>
     <row r="22">
       <c r="A22" s="3" t="s">
-        <v>2</v>
+        <v>18</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="s">
-        <v>18</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24">
@@ -1171,12 +1320,22 @@
     </row>
     <row r="28">
       <c r="A28" s="3" t="s">
-        <v>2</v>
+        <v>23</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="s">
+        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -1199,298 +1358,298 @@
   <sheetData>
     <row r="1" ht="17.25">
       <c r="A1" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="6" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5" ht="30">
       <c r="A5" s="7" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="G5" s="11" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H5" s="11" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" ht="30">
       <c r="A6" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="E6" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="F6" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="C6" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="D6" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="E6" s="10" t="s">
-        <v>38</v>
-      </c>
-      <c r="F6" s="8" t="s">
-        <v>39</v>
-      </c>
       <c r="G6" s="11" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H6" s="11" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" ht="30">
       <c r="A7" s="7" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B7" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="D7" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="C7" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="D7" s="9" t="s">
-        <v>43</v>
-      </c>
       <c r="E7" s="10" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="G7" s="11" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H7" s="11" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" ht="30">
       <c r="A8" s="7" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="G8" s="11" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H8" s="11" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" ht="30">
       <c r="A9" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="D9" s="12" t="s">
         <v>52</v>
       </c>
-      <c r="B9" s="8" t="s">
+      <c r="E9" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="C9" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="D9" s="12" t="s">
-        <v>50</v>
-      </c>
-      <c r="E9" s="10" t="s">
-        <v>51</v>
-      </c>
       <c r="F9" s="8" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="G9" s="11" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H9" s="11" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10" ht="45">
       <c r="A10" s="7" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="G10" s="11" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H10" s="11" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11" ht="30">
       <c r="A11" s="7" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="G11" s="11" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H11" s="11" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12" ht="30">
       <c r="A12" s="7" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D12" s="12" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="G12" s="11" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H12" s="11" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13" ht="30">
       <c r="A13" s="7" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G13" s="11" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H13" s="11" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14" ht="45">
       <c r="A14" s="7" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="F14" s="8" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="G14" s="11" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H14" s="11" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1514,194 +1673,194 @@
   <sheetData>
     <row r="1" ht="17.25">
       <c r="A1" s="4" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="6" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5" ht="45">
       <c r="A5" s="7" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="G5" s="11" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H5" s="11" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" ht="75">
       <c r="A6" s="7" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B6" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="D6" s="12" t="s">
+        <v>87</v>
+      </c>
+      <c r="E6" s="10" t="s">
+        <v>88</v>
+      </c>
+      <c r="F6" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="C6" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="D6" s="12" t="s">
-        <v>85</v>
-      </c>
-      <c r="E6" s="10" t="s">
-        <v>86</v>
-      </c>
-      <c r="F6" s="8" t="s">
-        <v>81</v>
-      </c>
       <c r="G6" s="11" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H6" s="11" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" ht="60">
       <c r="A7" s="7" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B7" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="D7" s="12" t="s">
+        <v>92</v>
+      </c>
+      <c r="E7" s="10" t="s">
         <v>88</v>
       </c>
-      <c r="C7" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="D7" s="12" t="s">
-        <v>90</v>
-      </c>
-      <c r="E7" s="10" t="s">
-        <v>86</v>
-      </c>
       <c r="F7" s="8" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="G7" s="11" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H7" s="11" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" ht="45">
       <c r="A8" s="7" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="G8" s="11" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H8" s="11" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" ht="45">
       <c r="A9" s="7" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="G9" s="11" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H9" s="11" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10" ht="75">
       <c r="A10" s="7" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G10" s="11" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H10" s="11" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1726,244 +1885,244 @@
   <sheetData>
     <row r="1" ht="17.25">
       <c r="A1" s="4" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="6" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5" ht="45">
       <c r="A5" s="7" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H5" s="11" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I5" s="11" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" ht="45">
       <c r="A6" s="7" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B6" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>118</v>
+      </c>
+      <c r="E6" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="F6" s="8" t="s">
         <v>114</v>
       </c>
-      <c r="C6" s="8" t="s">
-        <v>115</v>
-      </c>
-      <c r="D6" s="9" t="s">
-        <v>116</v>
-      </c>
-      <c r="E6" s="10" t="s">
-        <v>38</v>
-      </c>
-      <c r="F6" s="8" t="s">
-        <v>112</v>
-      </c>
       <c r="G6" s="8" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H6" s="11" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I6" s="11" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" ht="36">
       <c r="A7" s="7" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H7" s="11" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I7" s="11" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" ht="45">
       <c r="A8" s="7" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H8" s="11" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I8" s="11" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" ht="75">
       <c r="A9" s="7" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H9" s="11" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I9" s="11" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10" ht="60">
       <c r="A10" s="7" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G10" s="8" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H10" s="11" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I10" s="11" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11" ht="48">
       <c r="A11" s="7" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="D11" s="12" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H11" s="11" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I11" s="11" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1988,7 +2147,7 @@
   <sheetData>
     <row r="1" ht="15.75">
       <c r="A1" s="13" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B1" s="13"/>
       <c r="C1" s="13"/>
@@ -2001,7 +2160,7 @@
     </row>
     <row r="2" ht="16.8" customHeight="1">
       <c r="A2" s="14" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B2" s="14"/>
       <c r="C2" s="14"/>
@@ -2014,292 +2173,292 @@
     </row>
     <row r="4" ht="7.2" customHeight="1">
       <c r="A4" s="15" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B4" s="15" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C4" s="15" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D4" s="15" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="E4" s="15" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F4" s="15" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="G4" s="15" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="H4" s="15" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="I4" s="15" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5" ht="45">
       <c r="A5" s="16" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="F5" s="16" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H5" s="16" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I5" s="16" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" ht="45">
       <c r="A6" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="B6" s="16" t="s">
+        <v>150</v>
+      </c>
+      <c r="C6" s="16" t="s">
+        <v>151</v>
+      </c>
+      <c r="D6" s="16" t="s">
+        <v>152</v>
+      </c>
+      <c r="E6" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="F6" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="B6" s="16" t="s">
-        <v>148</v>
-      </c>
-      <c r="C6" s="16" t="s">
-        <v>149</v>
-      </c>
-      <c r="D6" s="16" t="s">
-        <v>150</v>
-      </c>
-      <c r="E6" s="16" t="s">
-        <v>37</v>
-      </c>
-      <c r="F6" s="16" t="s">
-        <v>38</v>
-      </c>
       <c r="G6" s="16" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H6" s="16" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I6" s="16" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" ht="45">
       <c r="A7" s="16" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="C7" s="16" t="s">
+        <v>154</v>
+      </c>
+      <c r="D7" s="16" t="s">
         <v>152</v>
       </c>
-      <c r="D7" s="16" t="s">
-        <v>150</v>
-      </c>
       <c r="E7" s="16" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="F7" s="16" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H7" s="16" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I7" s="16" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" ht="45">
       <c r="A8" s="16" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B8" s="16" t="s">
+        <v>157</v>
+      </c>
+      <c r="C8" s="16" t="s">
+        <v>158</v>
+      </c>
+      <c r="D8" s="16" t="s">
+        <v>159</v>
+      </c>
+      <c r="E8" s="16" t="s">
         <v>155</v>
       </c>
-      <c r="C8" s="16" t="s">
-        <v>156</v>
-      </c>
-      <c r="D8" s="16" t="s">
-        <v>157</v>
-      </c>
-      <c r="E8" s="16" t="s">
-        <v>153</v>
-      </c>
       <c r="F8" s="16" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="G8" s="16" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H8" s="16" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I8" s="16" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" ht="45">
       <c r="A9" s="16" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="D9" s="16" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="E9" s="16" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="F9" s="16" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="G9" s="16" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="H9" s="16" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I9" s="16" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10" ht="45">
       <c r="A10" s="16" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="D10" s="16" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="E10" s="16" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="F10" s="16" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="G10" s="16" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="H10" s="16" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I10" s="16" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11" ht="30">
       <c r="A11" s="16" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="D11" s="16" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="E11" s="16" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="F11" s="16" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="G11" s="16" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="H11" s="16" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I11" s="16" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12" ht="30">
       <c r="A12" s="16" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="C12" s="16" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="D12" s="16" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="E12" s="16" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F12" s="16" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="G12" s="16" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="H12" s="16" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I12" s="16" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13" ht="30">
       <c r="A13" s="16" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B13" s="16" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="D13" s="16" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="E13" s="16" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="F13" s="16" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="G13" s="16" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="H13" s="16" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I13" s="16" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14" ht="30" customHeight="1">
@@ -2307,28 +2466,28 @@
         <v>10</v>
       </c>
       <c r="B14" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="C14" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="D14" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="E14" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="F14" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="G14" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="H14" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="I14" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
     </row>
   </sheetData>
@@ -2338,4 +2497,278 @@
     <mergeCell ref="A2:I2"/>
   </mergeCells>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="5.7109375" customWidth="1"/>
+    <col min="2" max="2" width="32.710938" customWidth="1"/>
+    <col min="3" max="3" width="40.710938" customWidth="1"/>
+    <col min="4" max="4" width="28.710938" customWidth="1"/>
+    <col min="5" max="5" width="45.710938" customWidth="1"/>
+    <col min="6" max="6" width="18.710938" customWidth="1"/>
+    <col min="7" max="7" width="15.7109375" customWidth="1"/>
+    <col min="8" max="8" width="20.710938" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="5" ht="45">
+      <c r="A5" t="s">
+        <v>36</v>
+      </c>
+      <c r="B5" t="s">
+        <v>189</v>
+      </c>
+      <c r="C5" s="17" t="s">
+        <v>190</v>
+      </c>
+      <c r="D5" t="s">
+        <v>39</v>
+      </c>
+      <c r="E5" s="17" t="s">
+        <v>191</v>
+      </c>
+      <c r="F5" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="6" ht="75">
+      <c r="A6" t="s">
+        <v>42</v>
+      </c>
+      <c r="B6" t="s">
+        <v>193</v>
+      </c>
+      <c r="C6" s="17" t="s">
+        <v>194</v>
+      </c>
+      <c r="D6" t="s">
+        <v>52</v>
+      </c>
+      <c r="E6" s="17" t="s">
+        <v>195</v>
+      </c>
+      <c r="F6" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="7" ht="60">
+      <c r="A7" t="s">
+        <v>46</v>
+      </c>
+      <c r="B7" t="s">
+        <v>196</v>
+      </c>
+      <c r="C7" s="17" t="s">
+        <v>197</v>
+      </c>
+      <c r="D7" t="s">
+        <v>39</v>
+      </c>
+      <c r="E7" s="17" t="s">
+        <v>198</v>
+      </c>
+      <c r="F7" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="8" ht="75">
+      <c r="A8" t="s">
+        <v>49</v>
+      </c>
+      <c r="B8" t="s">
+        <v>199</v>
+      </c>
+      <c r="C8" s="17" t="s">
+        <v>200</v>
+      </c>
+      <c r="D8" t="s">
+        <v>52</v>
+      </c>
+      <c r="E8" s="17" t="s">
+        <v>201</v>
+      </c>
+      <c r="F8" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="9" ht="30">
+      <c r="A9" t="s">
+        <v>54</v>
+      </c>
+      <c r="B9" t="s">
+        <v>202</v>
+      </c>
+      <c r="C9" s="17" t="s">
+        <v>203</v>
+      </c>
+      <c r="D9" t="s">
+        <v>204</v>
+      </c>
+      <c r="E9" s="17" t="s">
+        <v>205</v>
+      </c>
+      <c r="F9" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="10" ht="45">
+      <c r="A10" t="s">
+        <v>57</v>
+      </c>
+      <c r="B10" t="s">
+        <v>206</v>
+      </c>
+      <c r="C10" s="17" t="s">
+        <v>207</v>
+      </c>
+      <c r="D10" t="s">
+        <v>39</v>
+      </c>
+      <c r="E10" s="17" t="s">
+        <v>208</v>
+      </c>
+      <c r="F10" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="11" ht="45">
+      <c r="A11" t="s">
+        <v>61</v>
+      </c>
+      <c r="B11" t="s">
+        <v>209</v>
+      </c>
+      <c r="C11" s="17" t="s">
+        <v>210</v>
+      </c>
+      <c r="D11" t="s">
+        <v>211</v>
+      </c>
+      <c r="E11" s="17" t="s">
+        <v>212</v>
+      </c>
+      <c r="F11" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="12" ht="45">
+      <c r="A12" t="s">
+        <v>65</v>
+      </c>
+      <c r="B12" t="s">
+        <v>213</v>
+      </c>
+      <c r="C12" s="17" t="s">
+        <v>214</v>
+      </c>
+      <c r="D12" t="s">
+        <v>215</v>
+      </c>
+      <c r="E12" s="17" t="s">
+        <v>216</v>
+      </c>
+      <c r="F12" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="13" ht="45">
+      <c r="A13" t="s">
+        <v>68</v>
+      </c>
+      <c r="B13" t="s">
+        <v>217</v>
+      </c>
+      <c r="C13" s="17" t="s">
+        <v>218</v>
+      </c>
+      <c r="D13" t="s">
+        <v>219</v>
+      </c>
+      <c r="E13" s="17" t="s">
+        <v>220</v>
+      </c>
+      <c r="F13" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="14" ht="30">
+      <c r="A14" t="s">
+        <v>73</v>
+      </c>
+      <c r="B14" t="s">
+        <v>221</v>
+      </c>
+      <c r="C14" s="17" t="s">
+        <v>222</v>
+      </c>
+      <c r="D14" t="s">
+        <v>223</v>
+      </c>
+      <c r="E14" s="17" t="s">
+        <v>224</v>
+      </c>
+      <c r="F14" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="15" ht="30">
+      <c r="A15" t="s">
+        <v>225</v>
+      </c>
+      <c r="B15" t="s">
+        <v>226</v>
+      </c>
+      <c r="C15" s="17" t="s">
+        <v>227</v>
+      </c>
+      <c r="D15" t="s">
+        <v>228</v>
+      </c>
+      <c r="E15" s="17" t="s">
+        <v>229</v>
+      </c>
+      <c r="F15" t="s">
+        <v>192</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Scenariusze testowe: arkusze dla weryfikatorow 2048, 2044, 2049, 2051
Nowe arkusze: Norma dobowa, Norma sredniotygodniowa 48h, Praca w normie
wg planu, Magazyn nadgodzin - umowy; zaktualizowany arkusz Informacje.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XkLQcV8gkZA892VpAppynM
</commit_message>
<xml_diff>
--- a/Weryfikatory czasu pracy/Scenariusze testowe weryfikatorow czasu pracy.xlsx
+++ b/Weryfikatory czasu pracy/Scenariusze testowe weryfikatorow czasu pracy.xlsx
@@ -3,11 +3,11 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\enovaServer\Projekty\Enova\Weryfikatory czasu pracy\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin.vpn\AppData\Local\Temp\claude\C--enovaServer-Projekty-Enova\7d51e072-d333-4d2b-8052-c327b49e8093\scratchpad\out\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" activeTab="5"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0"/>
   </bookViews>
   <sheets>
     <sheet name="Informacje" sheetId="1" r:id="rId1"/>
@@ -16,12 +16,20 @@
     <sheet name="Ilość dni wolnych" sheetId="4" r:id="rId4"/>
     <sheet name="Odpoczynek dobowy 11h" sheetId="6" r:id="rId5"/>
     <sheet name="Niedobór normy okresu rozl." sheetId="8" r:id="rId6"/>
+    <sheet name="Norma dobowa" sheetId="9" r:id="rId7"/>
+    <sheet name="Norma średniotygodniowa 48h" sheetId="11" r:id="rId8"/>
+    <sheet name="Praca w normie wg planu" sheetId="13" r:id="rId9"/>
+    <sheet name="Magazyn nadgodzin - umowy" sheetId="15" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Okres zatrudnienia'!$A$4:$H$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Norma okresu rozliczeniowego'!$A$4:$H$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Ilość dni wolnych'!$A$4:$I$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Odpoczynek dobowy 11h'!$A$4:$I$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Norma dobowa'!$A$4:$H$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Norma średniotygodniowa 48h'!$A$4:$H$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Praca w normie wg planu'!$A$4:$H$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Magazyn nadgodzin - umowy'!$A$4:$H$14</definedName>
   </definedNames>
   <calcPr/>
 </workbook>
@@ -36,7 +44,7 @@
     <t/>
   </si>
   <si>
-    <t>Zakres: pięć weryfikatorów z folderu „Weryfikatory czasu pracy”, każdy na osobnym arkuszu.</t>
+    <t>Zakres: dziewięć weryfikatorów z folderu „Weryfikatory czasu pracy”, każdy na osobnym arkuszu.</t>
   </si>
   <si>
     <t>Arkusze:</t>
@@ -57,6 +65,18 @@
     <t>• Niedobór normy okresu rozl. – weryfikator planu pracy (Rodzaj=Plan, ID 40 w bazie Claude); dopełnia wbudowany weryfikator normy okresu rozliczeniowego o wykrywanie NIEDOBORU godzin niemożliwego do nadrobienia w pozostałych miesiącach okresu. Uruchamia się przy KAŻDYM zapisie dnia planu. W bazie Claude jeszcze nie podpięty do żadnego kalendarza (nieaktywny).</t>
   </si>
   <si>
+    <t>• Norma dobowa – weryfikator dnia planu pracy; plan dnia ≤ norma dobowa z etatu (w systemie równoważnym 12:00).</t>
+  </si>
+  <si>
+    <t>• Norma średniotygodniowa 48h – weryfikator planu pracy; przeciętnie 48h tygodniowo w okresie rozliczeniowym.</t>
+  </si>
+  <si>
+    <t>• Praca w normie wg planu – weryfikator dnia czasu pracy; strefa Praca w normie ≤ plan dnia.</t>
+  </si>
+  <si>
+    <t>• Magazyn nadgodzin - umowy – weryfikator dnia czasu pracy; czas z umowy cywilnoprawnej nie trafia do magazynu nadgodzin.</t>
+  </si>
+  <si>
     <t>Kolumny na arkuszach scenariuszy:</t>
   </si>
   <si>
@@ -105,7 +125,19 @@
     <t>Weryfikatory czasu pracy/Niedobór normy okresu rozliczeniowego.md (pkt 5)</t>
   </si>
   <si>
-    <t>Wygenerowano: 2026-09-10, zaktualizowano: 2026-09-28</t>
+    <t>Weryfikatory czasu pracy/KontrolePlanuZAlgorytmuKalendarza.md (Słabe miejsca, pkt 3)</t>
+  </si>
+  <si>
+    <t>Weryfikatory czasu pracy/KontrolePlanuZAlgorytmuKalendarza.md (Słabe miejsca, pkt 4)</t>
+  </si>
+  <si>
+    <t>Weryfikatory czasu pracy/Praca w normie nie ponad plan.md</t>
+  </si>
+  <si>
+    <t>Weryfikatory czasu pracy/Blokada magazynu nadgodzin - umowy cywilnoprawne.md</t>
+  </si>
+  <si>
+    <t>Wygenerowano: 2026-09-10, zaktualizowano: 2026-10-09</t>
   </si>
   <si>
     <t>Weryfikator: Okres zatrudnienia</t>
@@ -734,6 +766,350 @@
   </si>
   <si>
     <t>- (WeryfKalend nie ma wiersza z Definicja=40, GetWeryfikatory(Plan) nigdy jej nie zwróci)</t>
+  </si>
+  <si>
+    <t>Weryfikator: Norma dobowa</t>
+  </si>
+  <si>
+    <t>Weryfikator dnia planu pracy (Dzień planu). Plan dnia nie może przekroczyć normy dobowej z etatu (pole „Norma dobowa”, a gdy puste – wartość dobowa kalendarza, 8:00); w systemie równoważnym limit 12:00. Na bazie testowej: kalendarz 3 miesięczny – Ostrzeżenie, Podstawowy system_1_8:16 – Błąd.</t>
+  </si>
+  <si>
+    <t>System podstawowy, plan zgodny z normą</t>
+  </si>
+  <si>
+    <t>Kalendarz: Podstawowy system_1_8:16; pole „Norma dobowa” na etacie puste.
+Plan 13.10.2026: 8:00</t>
+  </si>
+  <si>
+    <t>brak błędu</t>
+  </si>
+  <si>
+    <t>System podstawowy, plan powyżej normy</t>
+  </si>
+  <si>
+    <t>Kalendarz: Podstawowy system_1_8:16; pole „Norma dobowa” na etacie puste.
+Plan 13.10.2026: 9:00</t>
+  </si>
+  <si>
+    <t>Błąd – zapis zablokowany (limit 8:00 z kalendarza)</t>
+  </si>
+  <si>
+    <t>Dla dnia (13.10.2026) zaplanowano czas (9:00) przekraczający dopuszczalną normę dobową (8:00) - (pracownik)</t>
+  </si>
+  <si>
+    <t>Norma dobowa wpisana na etacie, plan powyżej</t>
+  </si>
+  <si>
+    <t>Kalendarz: Podstawowy system_1_8:16; pole „Norma dobowa” na etacie = 7:00.
+Plan 13.10.2026: 7:30</t>
+  </si>
+  <si>
+    <t>Błąd – limit 7:00 z etatu, nie 8:00 z kalendarza</t>
+  </si>
+  <si>
+    <t>Dla dnia (13.10.2026) zaplanowano czas (7:30) przekraczający dopuszczalną normę dobową (7:00) - (pracownik)</t>
+  </si>
+  <si>
+    <t>Norma dobowa wpisana na etacie, plan równy</t>
+  </si>
+  <si>
+    <t>Jak w pkt 3, plan 13.10.2026: 7:00</t>
+  </si>
+  <si>
+    <t>Brak błędu (granica dozwolona)</t>
+  </si>
+  <si>
+    <t>System równoważny, plan 12h</t>
+  </si>
+  <si>
+    <t>Kalendarz: 3 miesięczny (równoważny).
+Plan 13.10.2026: 12:00</t>
+  </si>
+  <si>
+    <t>Brak błędu (limit 12:00)</t>
+  </si>
+  <si>
+    <t>System równoważny, plan 10h</t>
+  </si>
+  <si>
+    <t>Kalendarz: 3 miesięczny (równoważny).
+Plan 13.10.2026: 10:00</t>
+  </si>
+  <si>
+    <t>Brak błędu – wbudowana „Norma dobowa” zgłosiłaby przekroczenie 8:00, ten weryfikator nie</t>
+  </si>
+  <si>
+    <t>System równoważny, plan ponad 12h</t>
+  </si>
+  <si>
+    <t>Kalendarz: 3 miesięczny (równoważny).
+Plan 13.10.2026: 12:30</t>
+  </si>
+  <si>
+    <t>Ostrzeżenie – zapis możliwy (na tym kalendarzu podpięty jako Ostrzeżenie)</t>
+  </si>
+  <si>
+    <t>Dla dnia (13.10.2026) zaplanowano czas (12:30) przekraczający dopuszczalną normę dobową w równoważnym systemie czasu pracy (12:00) - (pracownik)</t>
+  </si>
+  <si>
+    <t>Dzień wolny w planie</t>
+  </si>
+  <si>
+    <t>Dowolny kalendarz.
+Plan soboty 17.10.2026: 0:00</t>
+  </si>
+  <si>
+    <t>Brak błędu – dni z planem 0:00 nie są sprawdzane</t>
+  </si>
+  <si>
+    <t>Zmiana kalendarza etatu w trakcie miesiąca</t>
+  </si>
+  <si>
+    <t>Etat do 15.10.2026 na kalendarzu 3 miesięczny, od 16.10.2026 na kalendarzu Podstawowy system_1_8:16 (nowy zapis historii etatu).
+Plan 10:00 w dniach 14.10.2026 i 20.10.2026</t>
+  </si>
+  <si>
+    <t>14.10 – brak błędu (limit 12:00); 20.10 – Błąd (limit 8:00). Limit liczony z etatu obowiązującego w danym dniu.</t>
+  </si>
+  <si>
+    <t>Dla dnia (20.10.2026) zaplanowano czas (10:00) przekraczający dopuszczalną normę dobową (8:00) - (pracownik)</t>
+  </si>
+  <si>
+    <t>Weryfikator: Norma średniotygodniowa 48h</t>
+  </si>
+  <si>
+    <t>Weryfikator planu pracy (Plan pracy). Plan okresu rozliczeniowego (przyciętego do zatrudnienia) nie może przekroczyć przeciętnie 48h tygodniowo: 48:00 za pełny tydzień + 12:00 za dzień niepełnego tygodnia (bez niedziel i świąt), maks. 48:00. Na bazie testowej: kalendarz 3 miesięczny – Ostrzeżenie, Podstawowy system_1_8:16 – Błąd.</t>
+  </si>
+  <si>
+    <t>Plan wprost z kalendarza</t>
+  </si>
+  <si>
+    <t>Kalendarz: Podstawowy system_1_8:16 (okres 1-miesięczny), październik 2026 bez zmian: 22 dni robocze × 8:00 = 176:00. Limit 48h: 228:00</t>
+  </si>
+  <si>
+    <t>Plan ponad normę, ale poniżej limitu 48h</t>
+  </si>
+  <si>
+    <t>Jak w pkt 1, dni robocze października po 10:00: 22 × 10:00 = 220:00</t>
+  </si>
+  <si>
+    <t>Brak komunikatu 48h. Pojawi się tylko przekroczenie normy z weryfikatora A1_Norma w okresie rozliczeniowym.</t>
+  </si>
+  <si>
+    <t>brak komunikatu 48h; A1_Norma w okresie rozliczeniowym: Przekroczono limit godzin (…) o (…)</t>
+  </si>
+  <si>
+    <t>Plan równy limitowi 48h</t>
+  </si>
+  <si>
+    <t>Jak w pkt 1, dni robocze po 10:00 (220:00) + sobota 17.10.2026: 8:00 = 228:00</t>
+  </si>
+  <si>
+    <t>Brak komunikatu 48h (granica dozwolona). A1_Norma w okresie rozliczeniowym zgłosi przekroczenie normy.</t>
+  </si>
+  <si>
+    <t>brak komunikatu 48h</t>
+  </si>
+  <si>
+    <t>Przekroczenie 48h w okresie 1-miesięcznym</t>
+  </si>
+  <si>
+    <t>Jak w pkt 1, wszystkie 31 dni października po 8:00 = 248:00</t>
+  </si>
+  <si>
+    <t>Błąd – zapis zablokowany; dodatkowo komunikat A1_Norma w okresie rozliczeniowym</t>
+  </si>
+  <si>
+    <t>Zaplanowany czas pracy (248:00) przekracza przeciętnie 48h tygodniowo (228:00) o (20:00) w okresie rozliczeniowym (…) - (pracownik)</t>
+  </si>
+  <si>
+    <t>Zatrudnienie w trakcie okresu</t>
+  </si>
+  <si>
+    <t>Kalendarz: Podstawowy system_1_8:16. Przyjęcie 15.10.2026, plan 15–31.10 codziennie 8:00 = 136:00. Limit: 2 pełne tygodnie (15–28.10) = 96:00 + 29, 30, 31.10 = 36:00 → 132:00</t>
+  </si>
+  <si>
+    <t>Błąd – nadwyżka 4:00 (okres przycięty do zatrudnienia)</t>
+  </si>
+  <si>
+    <t>Zaplanowany czas pracy (136:00) przekracza przeciętnie 48h tygodniowo (132:00) o (4:00) w okresie rozliczeniowym (…) - (pracownik)</t>
+  </si>
+  <si>
+    <t>System równoważny, plan zgodny z kalendarzem</t>
+  </si>
+  <si>
+    <t>Kalendarz: 3 miesięczny, okres październik–grudzień 2026 (92 dni = 13 pełnych tygodni + 31.12), limit 13 × 48:00 + 12:00 = 636:00. Plan bez zmian.</t>
+  </si>
+  <si>
+    <t>System równoważny, przekroczenie 48h</t>
+  </si>
+  <si>
+    <t>Kalendarz: 3 miesięczny. Październik i listopad 2026 codziennie po 12:00 (61 × 12:00 = 732:00), grudzień bez zmian → plan okresu &gt; 636:00</t>
+  </si>
+  <si>
+    <t>Ostrzeżenie (na tym kalendarzu podpięty jako Ostrzeżenie). Zapis i tak zablokuje błąd A1_Norma w okresie rozliczeniowym.</t>
+  </si>
+  <si>
+    <t>Zaplanowany czas pracy (…) przekracza przeciętnie 48h tygodniowo (636:00) o (…) w okresie rozliczeniowym (…) - (pracownik)</t>
+  </si>
+  <si>
+    <t>Weryfikator: Praca w normie wg planu</t>
+  </si>
+  <si>
+    <t>Weryfikator dnia czasu pracy (Dzień pracy). Suma stref „Praca w normie” w dniu nie może przekroczyć planu dnia; nadwyżkę trzeba wpisać jako „Praca poza normą” + „Nadgodziny do przeniesienia”. Na bazie testowej: kalendarze 3 miesięczny i Podstawowy system_1_8:16 – Błąd (bez kalendarza Standard).</t>
+  </si>
+  <si>
+    <t>Praca w normie równa planowi</t>
+  </si>
+  <si>
+    <t>Kalendarz: Podstawowy system_1_8:16. Plan 13.10.2026: 8:00 (8:00–16:00).
+Czas pracy: Praca w normie 8:00</t>
+  </si>
+  <si>
+    <t>Praca w normie mniejsza niż plan</t>
+  </si>
+  <si>
+    <t>Plan 13.10.2026: 8:00.
+Czas pracy: Praca w normie 6:00</t>
+  </si>
+  <si>
+    <t>Brak błędu – kontrolowana jest tylko górna granica</t>
+  </si>
+  <si>
+    <t>Praca w normie ponad plan</t>
+  </si>
+  <si>
+    <t>Plan 13.10.2026: 8:00.
+Czas pracy: Praca w normie 8:00–18:00 (10:00)</t>
+  </si>
+  <si>
+    <t>Błąd – zapis zablokowany</t>
+  </si>
+  <si>
+    <t>Dla dnia (13.10.2026) w strefie Praca w normie wpisano (10:00), a plan przewiduje (8:00). Nadwyżkę (2:00) wpisz jako Praca poza normą i Nadgodziny do przeniesienia - (pracownik)</t>
+  </si>
+  <si>
+    <t>Nadwyżka poprawnie rozpisana</t>
+  </si>
+  <si>
+    <t>Plan 13.10.2026: 8:00.
+Czas pracy: Praca w normie 8:00–16:00 (8:00), Praca poza normą 16:00–18:00 (2:00), Nadgodziny do przeniesienia 2:00</t>
+  </si>
+  <si>
+    <t>Kilka stref Praca w normie w dniu</t>
+  </si>
+  <si>
+    <t>Plan 13.10.2026: 8:00.
+Czas pracy: Praca w normie 6:00–10:00 (4:00) i 11:00–16:00 (5:00)</t>
+  </si>
+  <si>
+    <t>Błąd – strefy są sumowane (9:00), nadwyżka 1:00</t>
+  </si>
+  <si>
+    <t>Dla dnia (13.10.2026) w strefie Praca w normie wpisano (9:00), a plan przewiduje (8:00). Nadwyżkę (1:00) wpisz jako (…)</t>
+  </si>
+  <si>
+    <t>Praca w normie w dniu wolnym wg planu</t>
+  </si>
+  <si>
+    <t>Sobota 17.10.2026, plan 0:00.
+Czas pracy: Praca w normie 8:00</t>
+  </si>
+  <si>
+    <t>Błąd – cała praca to nadwyżka</t>
+  </si>
+  <si>
+    <t>Dla dnia (17.10.2026) w strefie Praca w normie wpisano (8:00), a plan przewiduje (0:00). Nadwyżkę (8:00) wpisz jako (…)</t>
+  </si>
+  <si>
+    <t>Dzień wolny bez strefy Praca w normie</t>
+  </si>
+  <si>
+    <t>Sobota 17.10.2026, plan 0:00.
+Czas pracy: Praca poza normą 8:00 + Nadgodziny do przeniesienia 8:00</t>
+  </si>
+  <si>
+    <t>Kalendarz bez podpiętego weryfikatora</t>
+  </si>
+  <si>
+    <t>Pracownik na kalendarzu Standard. Plan 13.10.2026: 8:00.
+Czas pracy: Praca w normie 10:00</t>
+  </si>
+  <si>
+    <t>Brak błędu – na bazie testowej weryfikator nie jest podpięty do kalendarza Standard</t>
+  </si>
+  <si>
+    <t>Weryfikator: Magazyn nadgodzin - umowy</t>
+  </si>
+  <si>
+    <t>Weryfikator dnia czasu pracy (Dzień pracy). W dniu, w którym pracownik nie ma umowy o pracę, a ma umowę cywilnoprawną, blokuje strefy zasilające magazyn nadgodzin (rozliczenie „W kolejnych miesiącach”). Na bazie testowej: kalendarze Standard, 3 miesięczny i Podstawowy system_1_8:16 – Błąd.</t>
+  </si>
+  <si>
+    <t>Zleceniobiorca, Nadgodziny do przeniesienia</t>
+  </si>
+  <si>
+    <t>Pracownik tylko z umową zlecenia (bez umowy o pracę).
+Czas pracy 13.10.2026: Praca poza normą 8:00 + Nadgodziny do przeniesienia 8:00</t>
+  </si>
+  <si>
+    <t>Dnia (13.10.2026) pracownik pracuje na umowie cywilnoprawnej - czasu (8:00) nie można przenieść do magazynu nadgodzin (strefa Nadgodziny do przeniesienia) - (pracownik)</t>
+  </si>
+  <si>
+    <t>Zleceniobiorca, bez stref magazynu</t>
+  </si>
+  <si>
+    <t>Jak w pkt 1, czas pracy: tylko Praca poza normą 8:00</t>
+  </si>
+  <si>
+    <t>Zleceniobiorca, Rozliczenie wyjścia prywatnego</t>
+  </si>
+  <si>
+    <t>Jak w pkt 1, czas pracy: strefa Rozliczenie wyjścia prywatnego 1:00</t>
+  </si>
+  <si>
+    <t>Błąd – strefa również zasila magazyn</t>
+  </si>
+  <si>
+    <t>Dnia (13.10.2026) pracownik pracuje na umowie cywilnoprawnej - czasu (1:00) nie można przenieść do magazynu nadgodzin (strefa Rozliczenie wyjścia prywatnego) - (pracownik)</t>
+  </si>
+  <si>
+    <t>Pracownik na umowie o pracę</t>
+  </si>
+  <si>
+    <t>Pracownik z umową o pracę.
+Czas pracy 13.10.2026: Praca w normie 8:00, Praca poza normą 2:00 + Nadgodziny do przeniesienia 2:00</t>
+  </si>
+  <si>
+    <t>Umowa o pracę i zlecenie równocześnie</t>
+  </si>
+  <si>
+    <t>Pracownik ma w tym samym okresie umowę o pracę i umowę zlecenia.
+Czas pracy 13.10.2026: Nadgodziny do przeniesienia 2:00</t>
+  </si>
+  <si>
+    <t>Brak błędu – czas traktowany jak czas z etatu (ograniczenie weryfikatora)</t>
+  </si>
+  <si>
+    <t>Zmiana formy zatrudnienia</t>
+  </si>
+  <si>
+    <t>Umowa o pracę do 30.09.2026, umowa zlecenia od 01.10.2026.
+Nadgodziny do przeniesienia 2:00 w dniach 30.09.2026 i 01.10.2026</t>
+  </si>
+  <si>
+    <t>30.09 – brak błędu; 01.10 – Błąd</t>
+  </si>
+  <si>
+    <t>Dnia (01.10.2026) pracownik pracuje na umowie cywilnoprawnej - czasu (2:00) nie można przenieść do magazynu nadgodzin (strefa Nadgodziny do przeniesienia) - (pracownik)</t>
+  </si>
+  <si>
+    <t>Zleceniobiorca, strefa odbioru nadgodzin</t>
+  </si>
+  <si>
+    <t>Jak w pkt 1, czas pracy: strefa odbioru nadgodzin (rozliczenie „Z poprzednich miesięcy”)</t>
+  </si>
+  <si>
+    <t>Brak błędu – kontrolowane jest tylko zasilanie magazynu</t>
   </si>
 </sst>
 </file>
@@ -1234,28 +1610,28 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="s">
-        <v>1</v>
+      <c r="A11" s="3" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="s">
-        <v>12</v>
+      <c r="A15" s="2" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="16">
@@ -1275,47 +1651,47 @@
     </row>
     <row r="19">
       <c r="A19" s="3" t="s">
-        <v>1</v>
+        <v>16</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="s">
+      <c r="A23" s="3" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="s">
-        <v>22</v>
+      <c r="A27" s="2" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="28">
@@ -1329,16 +1705,265 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="s">
-        <v>1</v>
+      <c r="A30" s="3" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>25</v>
+        <v>26</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="s">
+        <v>33</v>
       </c>
     </row>
   </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="5.7109375" customWidth="1"/>
+    <col min="2" max="2" width="34.710938" customWidth="1"/>
+    <col min="3" max="3" width="40.710938" customWidth="1"/>
+    <col min="4" max="4" width="44.710938" customWidth="1"/>
+    <col min="5" max="5" width="46.710938" customWidth="1"/>
+    <col min="6" max="6" width="16.710938" customWidth="1"/>
+    <col min="7" max="7" width="18.710938" customWidth="1"/>
+    <col min="8" max="8" width="26.710938" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="17.25">
+      <c r="A1" s="4" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="G4" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="H4" s="6" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="5" ht="60">
+      <c r="A5" s="7">
+        <v>1</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>325</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>326</v>
+      </c>
+      <c r="D5" s="12" t="s">
+        <v>306</v>
+      </c>
+      <c r="E5" s="10" t="s">
+        <v>327</v>
+      </c>
+      <c r="F5" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="G5" s="11"/>
+      <c r="H5" s="11"/>
+    </row>
+    <row r="6" ht="30">
+      <c r="A6" s="7">
+        <v>2</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>328</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>329</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="E6" s="10" t="s">
+        <v>242</v>
+      </c>
+      <c r="F6" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="G6" s="11"/>
+      <c r="H6" s="11"/>
+    </row>
+    <row r="7" ht="48">
+      <c r="A7" s="7">
+        <v>3</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>330</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>331</v>
+      </c>
+      <c r="D7" s="12" t="s">
+        <v>332</v>
+      </c>
+      <c r="E7" s="10" t="s">
+        <v>333</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="G7" s="11"/>
+      <c r="H7" s="11"/>
+    </row>
+    <row r="8" ht="60">
+      <c r="A8" s="7">
+        <v>4</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>334</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>335</v>
+      </c>
+      <c r="D8" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="E8" s="10" t="s">
+        <v>242</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="G8" s="11"/>
+      <c r="H8" s="11"/>
+    </row>
+    <row r="9" ht="60">
+      <c r="A9" s="7">
+        <v>5</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>336</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>337</v>
+      </c>
+      <c r="D9" s="9" t="s">
+        <v>338</v>
+      </c>
+      <c r="E9" s="10" t="s">
+        <v>242</v>
+      </c>
+      <c r="F9" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="G9" s="11"/>
+      <c r="H9" s="11"/>
+    </row>
+    <row r="10" ht="60">
+      <c r="A10" s="7">
+        <v>6</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>339</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>340</v>
+      </c>
+      <c r="D10" s="12" t="s">
+        <v>341</v>
+      </c>
+      <c r="E10" s="10" t="s">
+        <v>342</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="G10" s="11"/>
+      <c r="H10" s="11"/>
+    </row>
+    <row r="11" ht="45">
+      <c r="A11" s="7">
+        <v>7</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>343</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>344</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>345</v>
+      </c>
+      <c r="E11" s="10" t="s">
+        <v>242</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="G11" s="11"/>
+      <c r="H11" s="11"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:H14"/>
 </worksheet>
 </file>
 
@@ -1358,58 +1983,58 @@
   <sheetData>
     <row r="1" ht="17.25">
       <c r="A1" s="4" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="6" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
     </row>
     <row r="5" ht="30">
       <c r="A5" s="7" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="G5" s="11" t="s">
         <v>1</v>
@@ -1420,22 +2045,22 @@
     </row>
     <row r="6" ht="30">
       <c r="A6" s="7" t="s">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>45</v>
+        <v>53</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="G6" s="11" t="s">
         <v>1</v>
@@ -1446,22 +2071,22 @@
     </row>
     <row r="7" ht="30">
       <c r="A7" s="7" t="s">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="C7" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="E7" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="D7" s="9" t="s">
-        <v>45</v>
-      </c>
-      <c r="E7" s="10" t="s">
-        <v>40</v>
-      </c>
       <c r="F7" s="8" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="G7" s="11" t="s">
         <v>1</v>
@@ -1472,22 +2097,22 @@
     </row>
     <row r="8" ht="30">
       <c r="A8" s="7" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="G8" s="11" t="s">
         <v>1</v>
@@ -1498,22 +2123,22 @@
     </row>
     <row r="9" ht="30">
       <c r="A9" s="7" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="G9" s="11" t="s">
         <v>1</v>
@@ -1524,22 +2149,22 @@
     </row>
     <row r="10" ht="45">
       <c r="A10" s="7" t="s">
-        <v>57</v>
+        <v>65</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="G10" s="11" t="s">
         <v>1</v>
@@ -1550,22 +2175,22 @@
     </row>
     <row r="11" ht="30">
       <c r="A11" s="7" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>63</v>
+        <v>71</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>64</v>
+        <v>72</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="G11" s="11" t="s">
         <v>1</v>
@@ -1576,22 +2201,22 @@
     </row>
     <row r="12" ht="30">
       <c r="A12" s="7" t="s">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>67</v>
+        <v>75</v>
       </c>
       <c r="D12" s="12" t="s">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="G12" s="11" t="s">
         <v>1</v>
@@ -1602,22 +2227,22 @@
     </row>
     <row r="13" ht="30">
       <c r="A13" s="7" t="s">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>69</v>
+        <v>77</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="G13" s="11" t="s">
         <v>1</v>
@@ -1628,22 +2253,22 @@
     </row>
     <row r="14" ht="45">
       <c r="A14" s="7" t="s">
-        <v>73</v>
+        <v>81</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="F14" s="8" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="G14" s="11" t="s">
         <v>1</v>
@@ -1673,58 +2298,58 @@
   <sheetData>
     <row r="1" ht="17.25">
       <c r="A1" s="4" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>78</v>
+        <v>86</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="6" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
     </row>
     <row r="5" ht="45">
       <c r="A5" s="7" t="s">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="G5" s="11" t="s">
         <v>1</v>
@@ -1735,22 +2360,22 @@
     </row>
     <row r="6" ht="75">
       <c r="A6" s="7" t="s">
-        <v>84</v>
+        <v>92</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>87</v>
+        <v>95</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="G6" s="11" t="s">
         <v>1</v>
@@ -1761,22 +2386,22 @@
     </row>
     <row r="7" ht="60">
       <c r="A7" s="7" t="s">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>90</v>
+        <v>98</v>
       </c>
       <c r="C7" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="D7" s="12" t="s">
+        <v>100</v>
+      </c>
+      <c r="E7" s="10" t="s">
+        <v>96</v>
+      </c>
+      <c r="F7" s="8" t="s">
         <v>91</v>
-      </c>
-      <c r="D7" s="12" t="s">
-        <v>92</v>
-      </c>
-      <c r="E7" s="10" t="s">
-        <v>88</v>
-      </c>
-      <c r="F7" s="8" t="s">
-        <v>83</v>
       </c>
       <c r="G7" s="11" t="s">
         <v>1</v>
@@ -1787,22 +2412,22 @@
     </row>
     <row r="8" ht="45">
       <c r="A8" s="7" t="s">
-        <v>93</v>
+        <v>101</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>95</v>
+        <v>103</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>96</v>
+        <v>104</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="G8" s="11" t="s">
         <v>1</v>
@@ -1813,22 +2438,22 @@
     </row>
     <row r="9" ht="45">
       <c r="A9" s="7" t="s">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>99</v>
+        <v>107</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>101</v>
+        <v>109</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="G9" s="11" t="s">
         <v>1</v>
@@ -1839,22 +2464,22 @@
     </row>
     <row r="10" ht="75">
       <c r="A10" s="7" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="G10" s="11" t="s">
         <v>1</v>
@@ -1885,64 +2510,64 @@
   <sheetData>
     <row r="1" ht="17.25">
       <c r="A1" s="4" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>107</v>
+        <v>115</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="6" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
     </row>
     <row r="5" ht="45">
       <c r="A5" s="7" t="s">
-        <v>109</v>
+        <v>117</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>110</v>
+        <v>118</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="H5" s="11" t="s">
         <v>1</v>
@@ -1953,25 +2578,25 @@
     </row>
     <row r="6" ht="45">
       <c r="A6" s="7" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="H6" s="11" t="s">
         <v>1</v>
@@ -1982,25 +2607,25 @@
     </row>
     <row r="7" ht="36">
       <c r="A7" s="7" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>121</v>
+        <v>129</v>
       </c>
       <c r="D7" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="E7" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="F7" s="8" t="s">
         <v>122</v>
       </c>
-      <c r="E7" s="10" t="s">
-        <v>123</v>
-      </c>
-      <c r="F7" s="8" t="s">
-        <v>114</v>
-      </c>
       <c r="G7" s="8" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="H7" s="11" t="s">
         <v>1</v>
@@ -2011,25 +2636,25 @@
     </row>
     <row r="8" ht="45">
       <c r="A8" s="7" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>125</v>
+        <v>133</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>128</v>
+        <v>136</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="H8" s="11" t="s">
         <v>1</v>
@@ -2040,25 +2665,25 @@
     </row>
     <row r="9" ht="75">
       <c r="A9" s="7" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>130</v>
+        <v>138</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="H9" s="11" t="s">
         <v>1</v>
@@ -2069,25 +2694,25 @@
     </row>
     <row r="10" ht="60">
       <c r="A10" s="7" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>134</v>
+        <v>142</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>137</v>
+        <v>145</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="G10" s="8" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="H10" s="11" t="s">
         <v>1</v>
@@ -2098,25 +2723,25 @@
     </row>
     <row r="11" ht="48">
       <c r="A11" s="7" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>139</v>
+        <v>147</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>140</v>
+        <v>148</v>
       </c>
       <c r="D11" s="12" t="s">
-        <v>141</v>
+        <v>149</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>142</v>
+        <v>150</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>128</v>
+        <v>136</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="H11" s="11" t="s">
         <v>1</v>
@@ -2147,7 +2772,7 @@
   <sheetData>
     <row r="1" ht="15.75">
       <c r="A1" s="13" t="s">
-        <v>143</v>
+        <v>151</v>
       </c>
       <c r="B1" s="13"/>
       <c r="C1" s="13"/>
@@ -2160,7 +2785,7 @@
     </row>
     <row r="2" ht="16.8" customHeight="1">
       <c r="A2" s="14" t="s">
-        <v>144</v>
+        <v>152</v>
       </c>
       <c r="B2" s="14"/>
       <c r="C2" s="14"/>
@@ -2173,54 +2798,54 @@
     </row>
     <row r="4" ht="7.2" customHeight="1">
       <c r="A4" s="15" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="B4" s="15" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="C4" s="15" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="D4" s="15" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="E4" s="15" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="F4" s="15" t="s">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="G4" s="15" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="H4" s="15" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="I4" s="15" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
     </row>
     <row r="5" ht="45">
       <c r="A5" s="16" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>147</v>
+        <v>155</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>149</v>
+        <v>157</v>
       </c>
       <c r="F5" s="16" t="s">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="H5" s="16" t="s">
         <v>1</v>
@@ -2231,25 +2856,25 @@
     </row>
     <row r="6" ht="45">
       <c r="A6" s="16" t="s">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>151</v>
+        <v>159</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>152</v>
+        <v>160</v>
       </c>
       <c r="E6" s="16" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="F6" s="16" t="s">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="G6" s="16" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="H6" s="16" t="s">
         <v>1</v>
@@ -2260,25 +2885,25 @@
     </row>
     <row r="7" ht="45">
       <c r="A7" s="16" t="s">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>153</v>
+        <v>161</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>154</v>
+        <v>162</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>152</v>
+        <v>160</v>
       </c>
       <c r="E7" s="16" t="s">
-        <v>155</v>
+        <v>163</v>
       </c>
       <c r="F7" s="16" t="s">
-        <v>156</v>
+        <v>164</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="H7" s="16" t="s">
         <v>1</v>
@@ -2289,25 +2914,25 @@
     </row>
     <row r="8" ht="45">
       <c r="A8" s="16" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>158</v>
+        <v>166</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>159</v>
+        <v>167</v>
       </c>
       <c r="E8" s="16" t="s">
-        <v>155</v>
+        <v>163</v>
       </c>
       <c r="F8" s="16" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="G8" s="16" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="H8" s="16" t="s">
         <v>1</v>
@@ -2318,25 +2943,25 @@
     </row>
     <row r="9" ht="45">
       <c r="A9" s="16" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>161</v>
+        <v>169</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>162</v>
+        <v>170</v>
       </c>
       <c r="D9" s="16" t="s">
-        <v>163</v>
+        <v>171</v>
       </c>
       <c r="E9" s="16" t="s">
-        <v>164</v>
+        <v>172</v>
       </c>
       <c r="F9" s="16" t="s">
-        <v>165</v>
+        <v>173</v>
       </c>
       <c r="G9" s="16" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="H9" s="16" t="s">
         <v>1</v>
@@ -2347,25 +2972,25 @@
     </row>
     <row r="10" ht="45">
       <c r="A10" s="16" t="s">
-        <v>57</v>
+        <v>65</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>167</v>
+        <v>175</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>168</v>
+        <v>176</v>
       </c>
       <c r="D10" s="16" t="s">
-        <v>152</v>
+        <v>160</v>
       </c>
       <c r="E10" s="16" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="F10" s="16" t="s">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="G10" s="16" t="s">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="H10" s="16" t="s">
         <v>1</v>
@@ -2376,25 +3001,25 @@
     </row>
     <row r="11" ht="30">
       <c r="A11" s="16" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>170</v>
+        <v>178</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>171</v>
+        <v>179</v>
       </c>
       <c r="D11" s="16" t="s">
-        <v>172</v>
+        <v>180</v>
       </c>
       <c r="E11" s="16" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="F11" s="16" t="s">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="G11" s="16" t="s">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="H11" s="16" t="s">
         <v>1</v>
@@ -2405,25 +3030,25 @@
     </row>
     <row r="12" ht="30">
       <c r="A12" s="16" t="s">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="C12" s="16" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="D12" s="16" t="s">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="E12" s="16" t="s">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="F12" s="16" t="s">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="G12" s="16" t="s">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="H12" s="16" t="s">
         <v>1</v>
@@ -2434,25 +3059,25 @@
     </row>
     <row r="13" ht="30">
       <c r="A13" s="16" t="s">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="B13" s="16" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>176</v>
+        <v>184</v>
       </c>
       <c r="D13" s="16" t="s">
-        <v>177</v>
+        <v>185</v>
       </c>
       <c r="E13" s="16" t="s">
-        <v>178</v>
+        <v>186</v>
       </c>
       <c r="F13" s="16" t="s">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="G13" s="16" t="s">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="H13" s="16" t="s">
         <v>1</v>
@@ -2466,28 +3091,28 @@
         <v>10</v>
       </c>
       <c r="B14" t="s">
-        <v>179</v>
+        <v>187</v>
       </c>
       <c r="C14" t="s">
-        <v>180</v>
+        <v>188</v>
       </c>
       <c r="D14" t="s">
-        <v>181</v>
+        <v>189</v>
       </c>
       <c r="E14" t="s">
-        <v>182</v>
+        <v>190</v>
       </c>
       <c r="F14" t="s">
-        <v>183</v>
+        <v>191</v>
       </c>
       <c r="G14" t="s">
-        <v>184</v>
+        <v>192</v>
       </c>
       <c r="H14" t="s">
-        <v>185</v>
+        <v>193</v>
       </c>
       <c r="I14" t="s">
-        <v>186</v>
+        <v>194</v>
       </c>
     </row>
   </sheetData>
@@ -2515,260 +3140,953 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>187</v>
+        <v>195</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>188</v>
+        <v>196</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
     </row>
     <row r="5" ht="45">
       <c r="A5" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="B5" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>190</v>
+        <v>198</v>
       </c>
       <c r="D5" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>191</v>
+        <v>199</v>
       </c>
       <c r="F5" t="s">
-        <v>192</v>
+        <v>200</v>
       </c>
     </row>
     <row r="6" ht="75">
       <c r="A6" t="s">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="B6" t="s">
-        <v>193</v>
+        <v>201</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>194</v>
+        <v>202</v>
       </c>
       <c r="D6" t="s">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="E6" s="17" t="s">
-        <v>195</v>
+        <v>203</v>
       </c>
       <c r="F6" t="s">
-        <v>192</v>
+        <v>200</v>
       </c>
     </row>
     <row r="7" ht="60">
       <c r="A7" t="s">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="B7" t="s">
-        <v>196</v>
+        <v>204</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>197</v>
+        <v>205</v>
       </c>
       <c r="D7" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="E7" s="17" t="s">
-        <v>198</v>
+        <v>206</v>
       </c>
       <c r="F7" t="s">
-        <v>192</v>
+        <v>200</v>
       </c>
     </row>
     <row r="8" ht="75">
       <c r="A8" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="B8" t="s">
-        <v>199</v>
+        <v>207</v>
       </c>
       <c r="C8" s="17" t="s">
+        <v>208</v>
+      </c>
+      <c r="D8" t="s">
+        <v>60</v>
+      </c>
+      <c r="E8" s="17" t="s">
+        <v>209</v>
+      </c>
+      <c r="F8" t="s">
         <v>200</v>
-      </c>
-      <c r="D8" t="s">
-        <v>52</v>
-      </c>
-      <c r="E8" s="17" t="s">
-        <v>201</v>
-      </c>
-      <c r="F8" t="s">
-        <v>192</v>
       </c>
     </row>
     <row r="9" ht="30">
       <c r="A9" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="B9" t="s">
-        <v>202</v>
+        <v>210</v>
       </c>
       <c r="C9" s="17" t="s">
-        <v>203</v>
+        <v>211</v>
       </c>
       <c r="D9" t="s">
-        <v>204</v>
+        <v>212</v>
       </c>
       <c r="E9" s="17" t="s">
-        <v>205</v>
+        <v>213</v>
       </c>
       <c r="F9" t="s">
-        <v>192</v>
+        <v>200</v>
       </c>
     </row>
     <row r="10" ht="45">
       <c r="A10" t="s">
-        <v>57</v>
+        <v>65</v>
       </c>
       <c r="B10" t="s">
-        <v>206</v>
+        <v>214</v>
       </c>
       <c r="C10" s="17" t="s">
-        <v>207</v>
+        <v>215</v>
       </c>
       <c r="D10" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="E10" s="17" t="s">
-        <v>208</v>
+        <v>216</v>
       </c>
       <c r="F10" t="s">
-        <v>192</v>
+        <v>200</v>
       </c>
     </row>
     <row r="11" ht="45">
       <c r="A11" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="B11" t="s">
-        <v>209</v>
+        <v>217</v>
       </c>
       <c r="C11" s="17" t="s">
-        <v>210</v>
+        <v>218</v>
       </c>
       <c r="D11" t="s">
-        <v>211</v>
+        <v>219</v>
       </c>
       <c r="E11" s="17" t="s">
-        <v>212</v>
+        <v>220</v>
       </c>
       <c r="F11" t="s">
-        <v>192</v>
+        <v>200</v>
       </c>
     </row>
     <row r="12" ht="45">
       <c r="A12" t="s">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="B12" t="s">
-        <v>213</v>
+        <v>221</v>
       </c>
       <c r="C12" s="17" t="s">
-        <v>214</v>
+        <v>222</v>
       </c>
       <c r="D12" t="s">
-        <v>215</v>
+        <v>223</v>
       </c>
       <c r="E12" s="17" t="s">
-        <v>216</v>
+        <v>224</v>
       </c>
       <c r="F12" t="s">
-        <v>192</v>
+        <v>200</v>
       </c>
     </row>
     <row r="13" ht="45">
       <c r="A13" t="s">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="B13" t="s">
-        <v>217</v>
+        <v>225</v>
       </c>
       <c r="C13" s="17" t="s">
-        <v>218</v>
+        <v>226</v>
       </c>
       <c r="D13" t="s">
-        <v>219</v>
+        <v>227</v>
       </c>
       <c r="E13" s="17" t="s">
-        <v>220</v>
+        <v>228</v>
       </c>
       <c r="F13" t="s">
-        <v>192</v>
+        <v>200</v>
       </c>
     </row>
     <row r="14" ht="30">
       <c r="A14" t="s">
-        <v>73</v>
+        <v>81</v>
       </c>
       <c r="B14" t="s">
-        <v>221</v>
+        <v>229</v>
       </c>
       <c r="C14" s="17" t="s">
-        <v>222</v>
+        <v>230</v>
       </c>
       <c r="D14" t="s">
-        <v>223</v>
+        <v>231</v>
       </c>
       <c r="E14" s="17" t="s">
-        <v>224</v>
+        <v>232</v>
       </c>
       <c r="F14" t="s">
-        <v>192</v>
+        <v>200</v>
       </c>
     </row>
     <row r="15" ht="30">
       <c r="A15" t="s">
-        <v>225</v>
+        <v>233</v>
       </c>
       <c r="B15" t="s">
-        <v>226</v>
+        <v>234</v>
       </c>
       <c r="C15" s="17" t="s">
-        <v>227</v>
+        <v>235</v>
       </c>
       <c r="D15" t="s">
-        <v>228</v>
+        <v>236</v>
       </c>
       <c r="E15" s="17" t="s">
-        <v>229</v>
+        <v>237</v>
       </c>
       <c r="F15" t="s">
-        <v>192</v>
+        <v>200</v>
       </c>
     </row>
   </sheetData>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="5.7109375" customWidth="1"/>
+    <col min="2" max="2" width="34.710938" customWidth="1"/>
+    <col min="3" max="3" width="40.710938" customWidth="1"/>
+    <col min="4" max="4" width="44.710938" customWidth="1"/>
+    <col min="5" max="5" width="46.710938" customWidth="1"/>
+    <col min="6" max="6" width="16.710938" customWidth="1"/>
+    <col min="7" max="7" width="18.710938" customWidth="1"/>
+    <col min="8" max="8" width="26.710938" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="17.25">
+      <c r="A1" s="4" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="G4" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="H4" s="6" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="5" ht="45">
+      <c r="A5" s="7">
+        <v>1</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>240</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>241</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="E5" s="10" t="s">
+        <v>242</v>
+      </c>
+      <c r="F5" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="G5" s="11"/>
+      <c r="H5" s="11"/>
+    </row>
+    <row r="6" ht="45">
+      <c r="A6" s="7">
+        <v>2</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>243</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>244</v>
+      </c>
+      <c r="D6" s="12" t="s">
+        <v>245</v>
+      </c>
+      <c r="E6" s="10" t="s">
+        <v>246</v>
+      </c>
+      <c r="F6" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="G6" s="11"/>
+      <c r="H6" s="11"/>
+    </row>
+    <row r="7" ht="45">
+      <c r="A7" s="7">
+        <v>3</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>247</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>248</v>
+      </c>
+      <c r="D7" s="12" t="s">
+        <v>249</v>
+      </c>
+      <c r="E7" s="10" t="s">
+        <v>250</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="G7" s="11"/>
+      <c r="H7" s="11"/>
+    </row>
+    <row r="8" ht="30">
+      <c r="A8" s="7">
+        <v>4</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>251</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>252</v>
+      </c>
+      <c r="D8" s="9" t="s">
+        <v>253</v>
+      </c>
+      <c r="E8" s="10" t="s">
+        <v>242</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="G8" s="11"/>
+      <c r="H8" s="11"/>
+    </row>
+    <row r="9" ht="30">
+      <c r="A9" s="7">
+        <v>5</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>254</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>255</v>
+      </c>
+      <c r="D9" s="9" t="s">
+        <v>256</v>
+      </c>
+      <c r="E9" s="10" t="s">
+        <v>242</v>
+      </c>
+      <c r="F9" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="G9" s="11"/>
+      <c r="H9" s="11"/>
+    </row>
+    <row r="10" ht="30">
+      <c r="A10" s="7">
+        <v>6</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>257</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>258</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>259</v>
+      </c>
+      <c r="E10" s="10" t="s">
+        <v>242</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="G10" s="11"/>
+      <c r="H10" s="11"/>
+    </row>
+    <row r="11" ht="36">
+      <c r="A11" s="7">
+        <v>7</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>260</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>261</v>
+      </c>
+      <c r="D11" s="12" t="s">
+        <v>262</v>
+      </c>
+      <c r="E11" s="10" t="s">
+        <v>263</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="G11" s="11"/>
+      <c r="H11" s="11"/>
+    </row>
+    <row r="12" ht="30">
+      <c r="A12" s="7">
+        <v>8</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>264</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>265</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>266</v>
+      </c>
+      <c r="E12" s="10" t="s">
+        <v>242</v>
+      </c>
+      <c r="F12" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="G12" s="11"/>
+      <c r="H12" s="11"/>
+    </row>
+    <row r="13" ht="75">
+      <c r="A13" s="7">
+        <v>9</v>
+      </c>
+      <c r="B13" s="8" t="s">
+        <v>267</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>268</v>
+      </c>
+      <c r="D13" s="12" t="s">
+        <v>269</v>
+      </c>
+      <c r="E13" s="10" t="s">
+        <v>270</v>
+      </c>
+      <c r="F13" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="G13" s="11"/>
+      <c r="H13" s="11"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:H14"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="5.7109375" customWidth="1"/>
+    <col min="2" max="2" width="34.710938" customWidth="1"/>
+    <col min="3" max="3" width="40.710938" customWidth="1"/>
+    <col min="4" max="4" width="44.710938" customWidth="1"/>
+    <col min="5" max="5" width="46.710938" customWidth="1"/>
+    <col min="6" max="6" width="16.710938" customWidth="1"/>
+    <col min="7" max="7" width="18.710938" customWidth="1"/>
+    <col min="8" max="8" width="26.710938" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="17.25">
+      <c r="A1" s="4" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="G4" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="H4" s="6" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="5" ht="60">
+      <c r="A5" s="7">
+        <v>1</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>273</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>274</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="E5" s="10" t="s">
+        <v>242</v>
+      </c>
+      <c r="F5" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="G5" s="11"/>
+      <c r="H5" s="11"/>
+    </row>
+    <row r="6" ht="45">
+      <c r="A6" s="7">
+        <v>2</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>275</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>276</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>277</v>
+      </c>
+      <c r="E6" s="10" t="s">
+        <v>278</v>
+      </c>
+      <c r="F6" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="G6" s="11"/>
+      <c r="H6" s="11"/>
+    </row>
+    <row r="7" ht="45">
+      <c r="A7" s="7">
+        <v>3</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>279</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>280</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>281</v>
+      </c>
+      <c r="E7" s="10" t="s">
+        <v>282</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="G7" s="11"/>
+      <c r="H7" s="11"/>
+    </row>
+    <row r="8" ht="36">
+      <c r="A8" s="7">
+        <v>4</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>283</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>284</v>
+      </c>
+      <c r="D8" s="12" t="s">
+        <v>285</v>
+      </c>
+      <c r="E8" s="10" t="s">
+        <v>286</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="G8" s="11"/>
+      <c r="H8" s="11"/>
+    </row>
+    <row r="9" ht="75">
+      <c r="A9" s="7">
+        <v>5</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>287</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>288</v>
+      </c>
+      <c r="D9" s="12" t="s">
+        <v>289</v>
+      </c>
+      <c r="E9" s="10" t="s">
+        <v>290</v>
+      </c>
+      <c r="F9" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="G9" s="11"/>
+      <c r="H9" s="11"/>
+    </row>
+    <row r="10" ht="60">
+      <c r="A10" s="7">
+        <v>6</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>291</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>292</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="E10" s="10" t="s">
+        <v>242</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="G10" s="11"/>
+      <c r="H10" s="11"/>
+    </row>
+    <row r="11" ht="60">
+      <c r="A11" s="7">
+        <v>7</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>293</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>294</v>
+      </c>
+      <c r="D11" s="12" t="s">
+        <v>295</v>
+      </c>
+      <c r="E11" s="10" t="s">
+        <v>296</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="G11" s="11"/>
+      <c r="H11" s="11"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:H14"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="5.7109375" customWidth="1"/>
+    <col min="2" max="2" width="34.710938" customWidth="1"/>
+    <col min="3" max="3" width="40.710938" customWidth="1"/>
+    <col min="4" max="4" width="44.710938" customWidth="1"/>
+    <col min="5" max="5" width="46.710938" customWidth="1"/>
+    <col min="6" max="6" width="16.710938" customWidth="1"/>
+    <col min="7" max="7" width="18.710938" customWidth="1"/>
+    <col min="8" max="8" width="26.710938" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="17.25">
+      <c r="A1" s="4" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="G4" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="H4" s="6" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="5" ht="45">
+      <c r="A5" s="7">
+        <v>1</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>299</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>300</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="E5" s="10" t="s">
+        <v>242</v>
+      </c>
+      <c r="F5" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="G5" s="11"/>
+      <c r="H5" s="11"/>
+    </row>
+    <row r="6" ht="30">
+      <c r="A6" s="7">
+        <v>2</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>301</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>302</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>303</v>
+      </c>
+      <c r="E6" s="10" t="s">
+        <v>242</v>
+      </c>
+      <c r="F6" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="G6" s="11"/>
+      <c r="H6" s="11"/>
+    </row>
+    <row r="7" ht="48">
+      <c r="A7" s="7">
+        <v>3</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>304</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>305</v>
+      </c>
+      <c r="D7" s="12" t="s">
+        <v>306</v>
+      </c>
+      <c r="E7" s="10" t="s">
+        <v>307</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="G7" s="11"/>
+      <c r="H7" s="11"/>
+    </row>
+    <row r="8" ht="60">
+      <c r="A8" s="7">
+        <v>4</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>308</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>309</v>
+      </c>
+      <c r="D8" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="E8" s="10" t="s">
+        <v>242</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="G8" s="11"/>
+      <c r="H8" s="11"/>
+    </row>
+    <row r="9" ht="45">
+      <c r="A9" s="7">
+        <v>5</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>310</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>311</v>
+      </c>
+      <c r="D9" s="12" t="s">
+        <v>312</v>
+      </c>
+      <c r="E9" s="10" t="s">
+        <v>313</v>
+      </c>
+      <c r="F9" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="G9" s="11"/>
+      <c r="H9" s="11"/>
+    </row>
+    <row r="10" ht="36">
+      <c r="A10" s="7">
+        <v>6</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>314</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>315</v>
+      </c>
+      <c r="D10" s="12" t="s">
+        <v>316</v>
+      </c>
+      <c r="E10" s="10" t="s">
+        <v>317</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="G10" s="11"/>
+      <c r="H10" s="11"/>
+    </row>
+    <row r="11" ht="45">
+      <c r="A11" s="7">
+        <v>7</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>318</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>319</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="E11" s="10" t="s">
+        <v>242</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="G11" s="11"/>
+      <c r="H11" s="11"/>
+    </row>
+    <row r="12" ht="45">
+      <c r="A12" s="7">
+        <v>8</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>320</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>321</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>322</v>
+      </c>
+      <c r="E12" s="10" t="s">
+        <v>242</v>
+      </c>
+      <c r="F12" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="G12" s="11"/>
+      <c r="H12" s="11"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:H14"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Scenariusze testowe: Okres zatrudnienia - umowy cywilnoprawne
Scenariusze 10-12: pracownik tylko z umowa cywilnoprawna, zmiana etatu
na zlecenie, etat i zlecenie rownoczesnie.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XkLQcV8gkZA892VpAppynM
</commit_message>
<xml_diff>
--- a/Weryfikatory czasu pracy/Scenariusze testowe weryfikatorow czasu pracy.xlsx
+++ b/Weryfikatory czasu pracy/Scenariusze testowe weryfikatorow czasu pracy.xlsx
@@ -143,7 +143,7 @@
     <t>Weryfikator: Okres zatrudnienia</t>
   </si>
   <si>
-    <t>Weryfikator okresu zatrudnienia – weryfikator dnia planu pracy (DzienPlanu). Blokuje zakładanie/zmianę dni planu poza okresem zatrudnienia pracownika.</t>
+    <t>Weryfikator okresu zatrudnienia – weryfikator dnia planu pracy (DzienPlanu). Blokuje zakładanie/zmianę dni planu poza okresem zatrudnienia pracownika, także pracownika zatrudnionego wyłącznie na umowie cywilnoprawnej.</t>
   </si>
   <si>
     <t>Lp</t>
@@ -304,6 +304,42 @@
     <t>Brak błędu – weryfikacja liczona względem etatu aktywnego w tym dniu (Etat 2)</t>
   </si>
   <si>
+    <t>Pracownik tylko z umową cywilnoprawną</t>
+  </si>
+  <si>
+    <t>Brak etatu, umowa zlecenia od 01.01.2026 (kalendarz Standard).
+Dzień planu: 13.10.2026 zmieniony na 8:00</t>
+  </si>
+  <si>
+    <t>Błąd – plan zleceniobiorcy nie może być uzupełniany</t>
+  </si>
+  <si>
+    <t>Nie można modyfikować planu pracy w dniach poza okresem zatrudnienia: Okres zatrudnienia (…)</t>
+  </si>
+  <si>
+    <t>Zmiana etatu na umowę cywilnoprawną</t>
+  </si>
+  <si>
+    <t>Etat do 30.09.2026, od 01.10.2026 tylko umowa zlecenia.
+Dzień planu: 05.10.2026</t>
+  </si>
+  <si>
+    <t>Błąd – dzień po zakończeniu etatu, mimo trwającej umowy zlecenia</t>
+  </si>
+  <si>
+    <t>Etat i umowa cywilnoprawna równocześnie</t>
+  </si>
+  <si>
+    <t>Etat: 01.01.2026–31.12.2026 oraz umowa zlecenia w tym samym okresie.
+Dzień planu: 13.10.2026</t>
+  </si>
+  <si>
+    <t>Brak błędu – dzień w okresie etatu</t>
+  </si>
+  <si>
+    <t>brak błędu</t>
+  </si>
+  <si>
     <t>Weryfikator: Norma okresu rozliczeniowego</t>
   </si>
   <si>
@@ -779,9 +815,6 @@
   <si>
     <t>Kalendarz: Podstawowy system_1_8:16; pole „Norma dobowa” na etacie puste.
 Plan 13.10.2026: 8:00</t>
-  </si>
-  <si>
-    <t>brak błędu</t>
   </si>
   <si>
     <t>System podstawowy, plan powyżej normy</t>
@@ -1774,12 +1807,12 @@
   <sheetData>
     <row r="1" ht="17.25">
       <c r="A1" s="4" t="s">
-        <v>323</v>
+        <v>333</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>324</v>
+        <v>334</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
@@ -1813,16 +1846,16 @@
         <v>1</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>325</v>
+        <v>335</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>326</v>
+        <v>336</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>306</v>
+        <v>316</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>327</v>
+        <v>337</v>
       </c>
       <c r="F5" s="8" t="s">
         <v>49</v>
@@ -1835,16 +1868,16 @@
         <v>2</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>328</v>
+        <v>338</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>329</v>
+        <v>339</v>
       </c>
       <c r="D6" s="9" t="s">
         <v>47</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>242</v>
+        <v>95</v>
       </c>
       <c r="F6" s="8" t="s">
         <v>49</v>
@@ -1857,16 +1890,16 @@
         <v>3</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>330</v>
+        <v>340</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>331</v>
+        <v>341</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>332</v>
+        <v>342</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="F7" s="8" t="s">
         <v>49</v>
@@ -1879,16 +1912,16 @@
         <v>4</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>334</v>
+        <v>344</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>335</v>
+        <v>345</v>
       </c>
       <c r="D8" s="9" t="s">
         <v>47</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>242</v>
+        <v>95</v>
       </c>
       <c r="F8" s="8" t="s">
         <v>49</v>
@@ -1901,16 +1934,16 @@
         <v>5</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>336</v>
+        <v>346</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>337</v>
+        <v>347</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>338</v>
+        <v>348</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>242</v>
+        <v>95</v>
       </c>
       <c r="F9" s="8" t="s">
         <v>49</v>
@@ -1923,16 +1956,16 @@
         <v>6</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>339</v>
+        <v>349</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>340</v>
+        <v>350</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>341</v>
+        <v>351</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>342</v>
+        <v>352</v>
       </c>
       <c r="F10" s="8" t="s">
         <v>49</v>
@@ -1945,16 +1978,16 @@
         <v>7</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>343</v>
+        <v>353</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>344</v>
+        <v>354</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>345</v>
+        <v>355</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>242</v>
+        <v>95</v>
       </c>
       <c r="F11" s="8" t="s">
         <v>49</v>
@@ -2277,6 +2310,84 @@
         <v>1</v>
       </c>
     </row>
+    <row r="15" ht="45">
+      <c r="A15" s="7">
+        <v>10</v>
+      </c>
+      <c r="B15" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="C15" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="D15" s="12" t="s">
+        <v>87</v>
+      </c>
+      <c r="E15" s="10" t="s">
+        <v>88</v>
+      </c>
+      <c r="F15" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="G15" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="H15" s="11" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" ht="45">
+      <c r="A16" s="7">
+        <v>11</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="C16" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="D16" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="E16" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="F16" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="G16" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="H16" s="11" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" ht="45">
+      <c r="A17" s="7">
+        <v>12</v>
+      </c>
+      <c r="B17" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="C17" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="D17" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="E17" s="10" t="s">
+        <v>95</v>
+      </c>
+      <c r="F17" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="G17" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="H17" s="11" t="s">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A4:H14"/>
 </worksheet>
@@ -2298,12 +2409,12 @@
   <sheetData>
     <row r="1" ht="17.25">
       <c r="A1" s="4" t="s">
-        <v>85</v>
+        <v>96</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>86</v>
+        <v>97</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
@@ -2334,22 +2445,22 @@
     </row>
     <row r="5" ht="45">
       <c r="A5" s="7" t="s">
-        <v>87</v>
+        <v>98</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>88</v>
+        <v>99</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>89</v>
+        <v>100</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="E5" s="10" t="s">
         <v>48</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>91</v>
+        <v>102</v>
       </c>
       <c r="G5" s="11" t="s">
         <v>1</v>
@@ -2360,22 +2471,22 @@
     </row>
     <row r="6" ht="75">
       <c r="A6" s="7" t="s">
-        <v>92</v>
+        <v>103</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>93</v>
+        <v>104</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>94</v>
+        <v>105</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>95</v>
+        <v>106</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>96</v>
+        <v>107</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>91</v>
+        <v>102</v>
       </c>
       <c r="G6" s="11" t="s">
         <v>1</v>
@@ -2386,22 +2497,22 @@
     </row>
     <row r="7" ht="60">
       <c r="A7" s="7" t="s">
-        <v>97</v>
+        <v>108</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>98</v>
+        <v>109</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>99</v>
+        <v>110</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>100</v>
+        <v>111</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>96</v>
+        <v>107</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>91</v>
+        <v>102</v>
       </c>
       <c r="G7" s="11" t="s">
         <v>1</v>
@@ -2412,22 +2523,22 @@
     </row>
     <row r="8" ht="45">
       <c r="A8" s="7" t="s">
-        <v>101</v>
+        <v>112</v>
       </c>
       <c r="B8" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="D8" s="12" t="s">
+        <v>115</v>
+      </c>
+      <c r="E8" s="10" t="s">
+        <v>116</v>
+      </c>
+      <c r="F8" s="8" t="s">
         <v>102</v>
-      </c>
-      <c r="C8" s="8" t="s">
-        <v>103</v>
-      </c>
-      <c r="D8" s="12" t="s">
-        <v>104</v>
-      </c>
-      <c r="E8" s="10" t="s">
-        <v>105</v>
-      </c>
-      <c r="F8" s="8" t="s">
-        <v>91</v>
       </c>
       <c r="G8" s="11" t="s">
         <v>1</v>
@@ -2438,16 +2549,16 @@
     </row>
     <row r="9" ht="45">
       <c r="A9" s="7" t="s">
-        <v>106</v>
+        <v>117</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>107</v>
+        <v>118</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>108</v>
+        <v>119</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>109</v>
+        <v>120</v>
       </c>
       <c r="E9" s="10" t="s">
         <v>48</v>
@@ -2464,16 +2575,16 @@
     </row>
     <row r="10" ht="75">
       <c r="A10" s="7" t="s">
-        <v>110</v>
+        <v>121</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>111</v>
+        <v>122</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>112</v>
+        <v>123</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>113</v>
+        <v>124</v>
       </c>
       <c r="E10" s="10" t="s">
         <v>48</v>
@@ -2510,12 +2621,12 @@
   <sheetData>
     <row r="1" ht="17.25">
       <c r="A1" s="4" t="s">
-        <v>114</v>
+        <v>125</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
@@ -2535,7 +2646,7 @@
         <v>40</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>116</v>
+        <v>127</v>
       </c>
       <c r="G4" s="6" t="s">
         <v>41</v>
@@ -2549,22 +2660,22 @@
     </row>
     <row r="5" ht="45">
       <c r="A5" s="7" t="s">
-        <v>117</v>
+        <v>128</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>119</v>
+        <v>130</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>120</v>
+        <v>131</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>121</v>
+        <v>132</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>122</v>
+        <v>133</v>
       </c>
       <c r="G5" s="8" t="s">
         <v>49</v>
@@ -2578,22 +2689,22 @@
     </row>
     <row r="6" ht="45">
       <c r="A6" s="7" t="s">
-        <v>123</v>
+        <v>134</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>124</v>
+        <v>135</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>125</v>
+        <v>136</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>126</v>
+        <v>137</v>
       </c>
       <c r="E6" s="10" t="s">
         <v>48</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>122</v>
+        <v>133</v>
       </c>
       <c r="G6" s="8" t="s">
         <v>49</v>
@@ -2607,22 +2718,22 @@
     </row>
     <row r="7" ht="36">
       <c r="A7" s="7" t="s">
-        <v>127</v>
+        <v>138</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>128</v>
+        <v>139</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>129</v>
+        <v>140</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>130</v>
+        <v>141</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>131</v>
+        <v>142</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>122</v>
+        <v>133</v>
       </c>
       <c r="G7" s="8" t="s">
         <v>49</v>
@@ -2636,22 +2747,22 @@
     </row>
     <row r="8" ht="45">
       <c r="A8" s="7" t="s">
-        <v>132</v>
+        <v>143</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>133</v>
+        <v>144</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>134</v>
+        <v>145</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>135</v>
+        <v>146</v>
       </c>
       <c r="E8" s="10" t="s">
         <v>48</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>136</v>
+        <v>147</v>
       </c>
       <c r="G8" s="8" t="s">
         <v>49</v>
@@ -2665,22 +2776,22 @@
     </row>
     <row r="9" ht="75">
       <c r="A9" s="7" t="s">
-        <v>137</v>
+        <v>148</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>138</v>
+        <v>149</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>139</v>
+        <v>150</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>140</v>
+        <v>151</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>121</v>
+        <v>132</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>122</v>
+        <v>133</v>
       </c>
       <c r="G9" s="8" t="s">
         <v>49</v>
@@ -2694,22 +2805,22 @@
     </row>
     <row r="10" ht="60">
       <c r="A10" s="7" t="s">
-        <v>141</v>
+        <v>152</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>142</v>
+        <v>153</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>143</v>
+        <v>154</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>144</v>
+        <v>155</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>145</v>
+        <v>156</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>122</v>
+        <v>133</v>
       </c>
       <c r="G10" s="8" t="s">
         <v>49</v>
@@ -2723,22 +2834,22 @@
     </row>
     <row r="11" ht="48">
       <c r="A11" s="7" t="s">
-        <v>146</v>
+        <v>157</v>
       </c>
       <c r="B11" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>159</v>
+      </c>
+      <c r="D11" s="12" t="s">
+        <v>160</v>
+      </c>
+      <c r="E11" s="10" t="s">
+        <v>161</v>
+      </c>
+      <c r="F11" s="8" t="s">
         <v>147</v>
-      </c>
-      <c r="C11" s="8" t="s">
-        <v>148</v>
-      </c>
-      <c r="D11" s="12" t="s">
-        <v>149</v>
-      </c>
-      <c r="E11" s="10" t="s">
-        <v>150</v>
-      </c>
-      <c r="F11" s="8" t="s">
-        <v>136</v>
       </c>
       <c r="G11" s="8" t="s">
         <v>49</v>
@@ -2772,7 +2883,7 @@
   <sheetData>
     <row r="1" ht="15.75">
       <c r="A1" s="13" t="s">
-        <v>151</v>
+        <v>162</v>
       </c>
       <c r="B1" s="13"/>
       <c r="C1" s="13"/>
@@ -2785,7 +2896,7 @@
     </row>
     <row r="2" ht="16.8" customHeight="1">
       <c r="A2" s="14" t="s">
-        <v>152</v>
+        <v>163</v>
       </c>
       <c r="B2" s="14"/>
       <c r="C2" s="14"/>
@@ -2807,7 +2918,7 @@
         <v>38</v>
       </c>
       <c r="D4" s="15" t="s">
-        <v>153</v>
+        <v>164</v>
       </c>
       <c r="E4" s="15" t="s">
         <v>39</v>
@@ -2830,16 +2941,16 @@
         <v>44</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>154</v>
+        <v>165</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>155</v>
+        <v>166</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>156</v>
+        <v>167</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>157</v>
+        <v>168</v>
       </c>
       <c r="F5" s="16" t="s">
         <v>48</v>
@@ -2859,13 +2970,13 @@
         <v>50</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>158</v>
+        <v>169</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>159</v>
+        <v>170</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>160</v>
+        <v>171</v>
       </c>
       <c r="E6" s="16" t="s">
         <v>47</v>
@@ -2888,19 +2999,19 @@
         <v>54</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>161</v>
+        <v>172</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>162</v>
+        <v>173</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>160</v>
+        <v>171</v>
       </c>
       <c r="E7" s="16" t="s">
-        <v>163</v>
+        <v>174</v>
       </c>
       <c r="F7" s="16" t="s">
-        <v>164</v>
+        <v>175</v>
       </c>
       <c r="G7" s="16" t="s">
         <v>49</v>
@@ -2917,19 +3028,19 @@
         <v>57</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>165</v>
+        <v>176</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>166</v>
+        <v>177</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>167</v>
+        <v>178</v>
       </c>
       <c r="E8" s="16" t="s">
-        <v>163</v>
+        <v>174</v>
       </c>
       <c r="F8" s="16" t="s">
-        <v>168</v>
+        <v>179</v>
       </c>
       <c r="G8" s="16" t="s">
         <v>49</v>
@@ -2946,22 +3057,22 @@
         <v>62</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>169</v>
+        <v>180</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>170</v>
+        <v>181</v>
       </c>
       <c r="D9" s="16" t="s">
-        <v>171</v>
+        <v>182</v>
       </c>
       <c r="E9" s="16" t="s">
-        <v>172</v>
+        <v>183</v>
       </c>
       <c r="F9" s="16" t="s">
-        <v>173</v>
+        <v>184</v>
       </c>
       <c r="G9" s="16" t="s">
-        <v>174</v>
+        <v>185</v>
       </c>
       <c r="H9" s="16" t="s">
         <v>1</v>
@@ -2975,16 +3086,16 @@
         <v>65</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>175</v>
+        <v>186</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>176</v>
+        <v>187</v>
       </c>
       <c r="D10" s="16" t="s">
-        <v>160</v>
+        <v>171</v>
       </c>
       <c r="E10" s="16" t="s">
-        <v>177</v>
+        <v>188</v>
       </c>
       <c r="F10" s="16" t="s">
         <v>48</v>
@@ -3004,13 +3115,13 @@
         <v>69</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>178</v>
+        <v>189</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>179</v>
+        <v>190</v>
       </c>
       <c r="D11" s="16" t="s">
-        <v>180</v>
+        <v>191</v>
       </c>
       <c r="E11" s="16" t="s">
         <v>47</v>
@@ -3033,10 +3144,10 @@
         <v>73</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>181</v>
+        <v>192</v>
       </c>
       <c r="C12" s="16" t="s">
-        <v>182</v>
+        <v>193</v>
       </c>
       <c r="D12" s="16" t="s">
         <v>48</v>
@@ -3062,16 +3173,16 @@
         <v>76</v>
       </c>
       <c r="B13" s="16" t="s">
-        <v>183</v>
+        <v>194</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>184</v>
+        <v>195</v>
       </c>
       <c r="D13" s="16" t="s">
-        <v>185</v>
+        <v>196</v>
       </c>
       <c r="E13" s="16" t="s">
-        <v>186</v>
+        <v>197</v>
       </c>
       <c r="F13" s="16" t="s">
         <v>48</v>
@@ -3091,28 +3202,28 @@
         <v>10</v>
       </c>
       <c r="B14" t="s">
-        <v>187</v>
+        <v>198</v>
       </c>
       <c r="C14" t="s">
-        <v>188</v>
+        <v>199</v>
       </c>
       <c r="D14" t="s">
-        <v>189</v>
+        <v>200</v>
       </c>
       <c r="E14" t="s">
-        <v>190</v>
+        <v>201</v>
       </c>
       <c r="F14" t="s">
-        <v>191</v>
+        <v>202</v>
       </c>
       <c r="G14" t="s">
-        <v>192</v>
+        <v>203</v>
       </c>
       <c r="H14" t="s">
-        <v>193</v>
+        <v>204</v>
       </c>
       <c r="I14" t="s">
-        <v>194</v>
+        <v>205</v>
       </c>
     </row>
   </sheetData>
@@ -3140,12 +3251,12 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>195</v>
+        <v>206</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>196</v>
+        <v>207</v>
       </c>
     </row>
     <row r="4">
@@ -3179,19 +3290,19 @@
         <v>44</v>
       </c>
       <c r="B5" t="s">
-        <v>197</v>
+        <v>208</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>198</v>
+        <v>209</v>
       </c>
       <c r="D5" t="s">
         <v>47</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>199</v>
+        <v>210</v>
       </c>
       <c r="F5" t="s">
-        <v>200</v>
+        <v>211</v>
       </c>
     </row>
     <row r="6" ht="75">
@@ -3199,19 +3310,19 @@
         <v>50</v>
       </c>
       <c r="B6" t="s">
-        <v>201</v>
+        <v>212</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>202</v>
+        <v>213</v>
       </c>
       <c r="D6" t="s">
         <v>60</v>
       </c>
       <c r="E6" s="17" t="s">
-        <v>203</v>
+        <v>214</v>
       </c>
       <c r="F6" t="s">
-        <v>200</v>
+        <v>211</v>
       </c>
     </row>
     <row r="7" ht="60">
@@ -3219,19 +3330,19 @@
         <v>54</v>
       </c>
       <c r="B7" t="s">
-        <v>204</v>
+        <v>215</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>205</v>
+        <v>216</v>
       </c>
       <c r="D7" t="s">
         <v>47</v>
       </c>
       <c r="E7" s="17" t="s">
-        <v>206</v>
+        <v>217</v>
       </c>
       <c r="F7" t="s">
-        <v>200</v>
+        <v>211</v>
       </c>
     </row>
     <row r="8" ht="75">
@@ -3239,19 +3350,19 @@
         <v>57</v>
       </c>
       <c r="B8" t="s">
-        <v>207</v>
+        <v>218</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>208</v>
+        <v>219</v>
       </c>
       <c r="D8" t="s">
         <v>60</v>
       </c>
       <c r="E8" s="17" t="s">
-        <v>209</v>
+        <v>220</v>
       </c>
       <c r="F8" t="s">
-        <v>200</v>
+        <v>211</v>
       </c>
     </row>
     <row r="9" ht="30">
@@ -3259,19 +3370,19 @@
         <v>62</v>
       </c>
       <c r="B9" t="s">
-        <v>210</v>
+        <v>221</v>
       </c>
       <c r="C9" s="17" t="s">
+        <v>222</v>
+      </c>
+      <c r="D9" t="s">
+        <v>223</v>
+      </c>
+      <c r="E9" s="17" t="s">
+        <v>224</v>
+      </c>
+      <c r="F9" t="s">
         <v>211</v>
-      </c>
-      <c r="D9" t="s">
-        <v>212</v>
-      </c>
-      <c r="E9" s="17" t="s">
-        <v>213</v>
-      </c>
-      <c r="F9" t="s">
-        <v>200</v>
       </c>
     </row>
     <row r="10" ht="45">
@@ -3279,19 +3390,19 @@
         <v>65</v>
       </c>
       <c r="B10" t="s">
-        <v>214</v>
+        <v>225</v>
       </c>
       <c r="C10" s="17" t="s">
-        <v>215</v>
+        <v>226</v>
       </c>
       <c r="D10" t="s">
         <v>47</v>
       </c>
       <c r="E10" s="17" t="s">
-        <v>216</v>
+        <v>227</v>
       </c>
       <c r="F10" t="s">
-        <v>200</v>
+        <v>211</v>
       </c>
     </row>
     <row r="11" ht="45">
@@ -3299,19 +3410,19 @@
         <v>69</v>
       </c>
       <c r="B11" t="s">
-        <v>217</v>
+        <v>228</v>
       </c>
       <c r="C11" s="17" t="s">
-        <v>218</v>
+        <v>229</v>
       </c>
       <c r="D11" t="s">
-        <v>219</v>
+        <v>230</v>
       </c>
       <c r="E11" s="17" t="s">
-        <v>220</v>
+        <v>231</v>
       </c>
       <c r="F11" t="s">
-        <v>200</v>
+        <v>211</v>
       </c>
     </row>
     <row r="12" ht="45">
@@ -3319,19 +3430,19 @@
         <v>73</v>
       </c>
       <c r="B12" t="s">
-        <v>221</v>
+        <v>232</v>
       </c>
       <c r="C12" s="17" t="s">
-        <v>222</v>
+        <v>233</v>
       </c>
       <c r="D12" t="s">
-        <v>223</v>
+        <v>234</v>
       </c>
       <c r="E12" s="17" t="s">
-        <v>224</v>
+        <v>235</v>
       </c>
       <c r="F12" t="s">
-        <v>200</v>
+        <v>211</v>
       </c>
     </row>
     <row r="13" ht="45">
@@ -3339,19 +3450,19 @@
         <v>76</v>
       </c>
       <c r="B13" t="s">
-        <v>225</v>
+        <v>236</v>
       </c>
       <c r="C13" s="17" t="s">
-        <v>226</v>
+        <v>237</v>
       </c>
       <c r="D13" t="s">
-        <v>227</v>
+        <v>238</v>
       </c>
       <c r="E13" s="17" t="s">
-        <v>228</v>
+        <v>239</v>
       </c>
       <c r="F13" t="s">
-        <v>200</v>
+        <v>211</v>
       </c>
     </row>
     <row r="14" ht="30">
@@ -3359,39 +3470,39 @@
         <v>81</v>
       </c>
       <c r="B14" t="s">
-        <v>229</v>
+        <v>240</v>
       </c>
       <c r="C14" s="17" t="s">
-        <v>230</v>
+        <v>241</v>
       </c>
       <c r="D14" t="s">
-        <v>231</v>
+        <v>242</v>
       </c>
       <c r="E14" s="17" t="s">
-        <v>232</v>
+        <v>243</v>
       </c>
       <c r="F14" t="s">
-        <v>200</v>
+        <v>211</v>
       </c>
     </row>
     <row r="15" ht="30">
       <c r="A15" t="s">
-        <v>233</v>
+        <v>244</v>
       </c>
       <c r="B15" t="s">
-        <v>234</v>
+        <v>245</v>
       </c>
       <c r="C15" s="17" t="s">
-        <v>235</v>
+        <v>246</v>
       </c>
       <c r="D15" t="s">
-        <v>236</v>
+        <v>247</v>
       </c>
       <c r="E15" s="17" t="s">
-        <v>237</v>
+        <v>248</v>
       </c>
       <c r="F15" t="s">
-        <v>200</v>
+        <v>211</v>
       </c>
     </row>
   </sheetData>
@@ -3414,12 +3525,12 @@
   <sheetData>
     <row r="1" ht="17.25">
       <c r="A1" s="4" t="s">
-        <v>238</v>
+        <v>249</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>239</v>
+        <v>250</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
@@ -3453,16 +3564,16 @@
         <v>1</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>240</v>
+        <v>251</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>241</v>
+        <v>252</v>
       </c>
       <c r="D5" s="9" t="s">
         <v>47</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>242</v>
+        <v>95</v>
       </c>
       <c r="F5" s="8" t="s">
         <v>49</v>
@@ -3475,16 +3586,16 @@
         <v>2</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>243</v>
+        <v>253</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>244</v>
+        <v>254</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>245</v>
+        <v>255</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>246</v>
+        <v>256</v>
       </c>
       <c r="F6" s="8" t="s">
         <v>49</v>
@@ -3497,16 +3608,16 @@
         <v>3</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>247</v>
+        <v>257</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>248</v>
+        <v>258</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>249</v>
+        <v>259</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>250</v>
+        <v>260</v>
       </c>
       <c r="F7" s="8" t="s">
         <v>49</v>
@@ -3519,16 +3630,16 @@
         <v>4</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>251</v>
+        <v>261</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>252</v>
+        <v>262</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>253</v>
+        <v>263</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>242</v>
+        <v>95</v>
       </c>
       <c r="F8" s="8" t="s">
         <v>49</v>
@@ -3541,16 +3652,16 @@
         <v>5</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>254</v>
+        <v>264</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>255</v>
+        <v>265</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>256</v>
+        <v>266</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>242</v>
+        <v>95</v>
       </c>
       <c r="F9" s="8" t="s">
         <v>49</v>
@@ -3563,16 +3674,16 @@
         <v>6</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>257</v>
+        <v>267</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>258</v>
+        <v>268</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>259</v>
+        <v>269</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>242</v>
+        <v>95</v>
       </c>
       <c r="F10" s="8" t="s">
         <v>49</v>
@@ -3585,16 +3696,16 @@
         <v>7</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>260</v>
+        <v>270</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>261</v>
+        <v>271</v>
       </c>
       <c r="D11" s="12" t="s">
-        <v>262</v>
+        <v>272</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>263</v>
+        <v>273</v>
       </c>
       <c r="F11" s="8" t="s">
         <v>49</v>
@@ -3607,16 +3718,16 @@
         <v>8</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>264</v>
+        <v>274</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>265</v>
+        <v>275</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>266</v>
+        <v>276</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>242</v>
+        <v>95</v>
       </c>
       <c r="F12" s="8" t="s">
         <v>49</v>
@@ -3629,16 +3740,16 @@
         <v>9</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>267</v>
+        <v>277</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>268</v>
+        <v>278</v>
       </c>
       <c r="D13" s="12" t="s">
-        <v>269</v>
+        <v>279</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>270</v>
+        <v>280</v>
       </c>
       <c r="F13" s="8" t="s">
         <v>49</v>
@@ -3667,12 +3778,12 @@
   <sheetData>
     <row r="1" ht="17.25">
       <c r="A1" s="4" t="s">
-        <v>271</v>
+        <v>281</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>272</v>
+        <v>282</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
@@ -3706,16 +3817,16 @@
         <v>1</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>273</v>
+        <v>283</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>274</v>
+        <v>284</v>
       </c>
       <c r="D5" s="9" t="s">
         <v>47</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>242</v>
+        <v>95</v>
       </c>
       <c r="F5" s="8" t="s">
         <v>49</v>
@@ -3728,16 +3839,16 @@
         <v>2</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>275</v>
+        <v>285</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>276</v>
+        <v>286</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>277</v>
+        <v>287</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>278</v>
+        <v>288</v>
       </c>
       <c r="F6" s="8" t="s">
         <v>49</v>
@@ -3750,16 +3861,16 @@
         <v>3</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>279</v>
+        <v>289</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>280</v>
+        <v>290</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>281</v>
+        <v>291</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>282</v>
+        <v>292</v>
       </c>
       <c r="F7" s="8" t="s">
         <v>49</v>
@@ -3772,16 +3883,16 @@
         <v>4</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>283</v>
+        <v>293</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>284</v>
+        <v>294</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>285</v>
+        <v>295</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>286</v>
+        <v>296</v>
       </c>
       <c r="F8" s="8" t="s">
         <v>49</v>
@@ -3794,16 +3905,16 @@
         <v>5</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>287</v>
+        <v>297</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>288</v>
+        <v>298</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>289</v>
+        <v>299</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>290</v>
+        <v>300</v>
       </c>
       <c r="F9" s="8" t="s">
         <v>49</v>
@@ -3816,16 +3927,16 @@
         <v>6</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>291</v>
+        <v>301</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>292</v>
+        <v>302</v>
       </c>
       <c r="D10" s="9" t="s">
         <v>47</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>242</v>
+        <v>95</v>
       </c>
       <c r="F10" s="8" t="s">
         <v>49</v>
@@ -3838,16 +3949,16 @@
         <v>7</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>293</v>
+        <v>303</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>294</v>
+        <v>304</v>
       </c>
       <c r="D11" s="12" t="s">
-        <v>295</v>
+        <v>305</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>296</v>
+        <v>306</v>
       </c>
       <c r="F11" s="8" t="s">
         <v>49</v>
@@ -3876,12 +3987,12 @@
   <sheetData>
     <row r="1" ht="17.25">
       <c r="A1" s="4" t="s">
-        <v>297</v>
+        <v>307</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>298</v>
+        <v>308</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
@@ -3915,16 +4026,16 @@
         <v>1</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>299</v>
+        <v>309</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>300</v>
+        <v>310</v>
       </c>
       <c r="D5" s="9" t="s">
         <v>47</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>242</v>
+        <v>95</v>
       </c>
       <c r="F5" s="8" t="s">
         <v>49</v>
@@ -3937,16 +4048,16 @@
         <v>2</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>301</v>
+        <v>311</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>302</v>
+        <v>312</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>303</v>
+        <v>313</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>242</v>
+        <v>95</v>
       </c>
       <c r="F6" s="8" t="s">
         <v>49</v>
@@ -3959,19 +4070,19 @@
         <v>3</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>304</v>
+        <v>314</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>305</v>
+        <v>315</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>306</v>
+        <v>316</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>307</v>
+        <v>317</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>91</v>
+        <v>102</v>
       </c>
       <c r="G7" s="11"/>
       <c r="H7" s="11"/>
@@ -3981,16 +4092,16 @@
         <v>4</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>308</v>
+        <v>318</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>309</v>
+        <v>319</v>
       </c>
       <c r="D8" s="9" t="s">
         <v>47</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>242</v>
+        <v>95</v>
       </c>
       <c r="F8" s="8" t="s">
         <v>49</v>
@@ -4003,16 +4114,16 @@
         <v>5</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>310</v>
+        <v>320</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>311</v>
+        <v>321</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>312</v>
+        <v>322</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>313</v>
+        <v>323</v>
       </c>
       <c r="F9" s="8" t="s">
         <v>49</v>
@@ -4025,16 +4136,16 @@
         <v>6</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>314</v>
+        <v>324</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>315</v>
+        <v>325</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>316</v>
+        <v>326</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>317</v>
+        <v>327</v>
       </c>
       <c r="F10" s="8" t="s">
         <v>49</v>
@@ -4047,16 +4158,16 @@
         <v>7</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>318</v>
+        <v>328</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>319</v>
+        <v>329</v>
       </c>
       <c r="D11" s="9" t="s">
         <v>47</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>242</v>
+        <v>95</v>
       </c>
       <c r="F11" s="8" t="s">
         <v>49</v>
@@ -4069,16 +4180,16 @@
         <v>8</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>320</v>
+        <v>330</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>321</v>
+        <v>331</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>322</v>
+        <v>332</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>242</v>
+        <v>95</v>
       </c>
       <c r="F12" s="8" t="s">
         <v>49</v>

</xml_diff>

<commit_message>
Weryfikator brak zgody 8h (Al): scenariusze testowe przejscie na zywo 9/10, pracownicy testowi NP1-NP9, blad przy zmianie stopnia w trakcie zapisu historii
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LteDBT3rxDXGxoKYPGaKbf
</commit_message>
<xml_diff>
--- a/Weryfikatory czasu pracy/Scenariusze testowe weryfikatorow czasu pracy.xlsx
+++ b/Weryfikatory czasu pracy/Scenariusze testowe weryfikatorow czasu pracy.xlsx
@@ -1,16 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
-  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="M:\Klienci\Aldi\Rozwiązania A1\Weryfikatory\Nowe\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\enovaServer\Projekty\Enova\Weryfikatory czasu pracy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFC167F0-1B32-4353-8CF0-61168F70494C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" firstSheet="2" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" firstSheet="2" activeTab="7"/>
   </bookViews>
   <sheets>
     <sheet name="Informacje" sheetId="1" r:id="rId1"/>
@@ -20,25 +18,30 @@
     <sheet name="Norma dobowa" sheetId="5" r:id="rId5"/>
     <sheet name="Praca w normie wg planu" sheetId="9" r:id="rId6"/>
     <sheet name="Magazyn nadgodzin - umowy" sheetId="11" r:id="rId7"/>
+    <sheet name="Brak zgody 8h" sheetId="12" r:id="rId8"/>
   </sheets>
   <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Okres zatrudnienia'!$A$4:$G$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Norma okresu rozliczeniowego'!$A$4:$G$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Ilość dni wolnych'!$A$4:$G$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Norma dobowa'!$A$4:$G$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Praca w normie wg planu'!$A$4:$G$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Magazyn nadgodzin - umowy'!$A$4:$G$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Norma dobowa'!$A$4:$G$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Norma okresu rozliczeniowego'!$A$4:$G$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Okres zatrudnienia'!$A$4:$G$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Praca w normie wg planu'!$A$4:$G$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Brak zgody 8h'!$A$4:$G$14</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="198">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <si>
     <t>Scenariusze testowe – weryfikatory czasu pracy</t>
   </si>
   <si>
+    <t>Zakres: siedem weryfikatorów z folderu „Weryfikatory czasu pracy”, każdy na osobnym arkuszu.</t>
+  </si>
+  <si>
     <t/>
   </si>
   <si>
@@ -61,6 +64,9 @@
   </si>
   <si>
     <t>• Magazyn nadgodzin - umowy – weryfikator dnia czasu pracy; czas z umowy cywilnoprawnej nie trafia do magazynu nadgodzin.</t>
+  </si>
+  <si>
+    <t>• Brak zgody na pracę 8h – weryfikator dnia planu pracy; osoba ze stopniem umiarkowanym/znacznym bez zgody na pracę 8h – plan dnia ≤ 7:00.</t>
   </si>
   <si>
     <t>Kolumny na arkuszach scenariuszy:</t>
@@ -392,7 +398,7 @@
     <t>Okres 3-miesięczny. Miesiące 1–2 mocno przeplanowane pracą, bieżący miesiąc = miesiąc 3 (ostatni). Nawet cały wolny miesiąc 3 nie nadrobi deficytu.</t>
   </si>
   <si>
-    <t>Błąd –  brak dni wolnych do domknięcia normy.</t>
+    <t xml:space="preserve">Błąd –  brak dni wolnych do domknięcia normy.</t>
   </si>
   <si>
     <t>Za mało dni wolnych (X) wobec wymaganej liczby (Y) w okresie rozliczeniowym (…)</t>
@@ -661,14 +667,138 @@
     <t>Brak błędu – kontrolowane jest tylko zasilanie magazynu</t>
   </si>
   <si>
-    <t>Zakres: sześć weryfikatorów z folderu „Weryfikatory czasu pracy”, każdy na osobnym arkuszu.</t>
+    <t>Weryfikator: Brak zgody na pracę 8h</t>
+  </si>
+  <si>
+    <t>Weryfikator dnia planu pracy (Dzień planu), definicja „A1_Brak zgody na pracę 8h”. Pracownik ze stopniem umiarkowanym lub znacznym (orzeczenie PFRON albo ZUS), bez zaznaczonego na etacie pola „Zgoda na pracę 8h”, nie może mieć zaplanowanych więcej niż 7:00 na dobę. Na bazie testowej: kalendarze 3 miesięczny i Podstawowy system_1_8:16 – Błąd. Test 15.10.2026 na bazie Al, pracownicy NP1–NP9 (ImportyXML/Weryfikator brak zgody 8h - pracownicy i plan.xml; orzeczenia dodane w programie).</t>
+  </si>
+  <si>
+    <t>Umiarkowany, bez zgody, plan 8:00</t>
+  </si>
+  <si>
+    <t>NP1: orzeczenie PFRON – umiarkowany 01.01–31.12.2026; „Zgoda na pracę 8h” niezaznaczona; kal. Podstawowy system_1_8:16.
+Plan 02.11.2026: 8:00</t>
+  </si>
+  <si>
+    <t>Dla dnia (2.11.2026) zaplanowano czas (8:00), a pracownik bez zgody na pracę 8h (stopień niepełnosprawności Umiarkowany) może pracować maksymalnie 7:00 - (pracownik)</t>
+  </si>
+  <si>
+    <t>Komunikat pojawia się już przy zmianie czasu strefy, przed zapisem.</t>
+  </si>
+  <si>
+    <t>Umiarkowany, bez zgody, plan 7:00 (granica)</t>
+  </si>
+  <si>
+    <t>NP2: jak NP1.
+Plan 02.11.2026: 7:00 (dodatkowo sobota 07.11: 1:00, żeby nie wywołać niedoboru normy okresu)</t>
+  </si>
+  <si>
+    <t>Odezwał się tylko weryfikator dni wolnych – skutek pomocniczej soboty, nie tego weryfikatora.</t>
+  </si>
+  <si>
+    <t>Znaczny, bez zgody, plan 7:30</t>
+  </si>
+  <si>
+    <t>NP3: orzeczenie PFRON – znaczny 01.01–31.12.2026; zgoda niezaznaczona; kal. Podstawowy system_1_8:16.
+Plan 02.11.2026: 7:30</t>
+  </si>
+  <si>
+    <t>Dla dnia (2.11.2026) zaplanowano czas (7:30), a pracownik bez zgody na pracę 8h (stopień niepełnosprawności Znaczny) może pracować maksymalnie 7:00 - (pracownik)</t>
+  </si>
+  <si>
+    <t>Jednocześnie norma okresu rozliczeniowego żąda 160:00 i podpowiada „Wydłuż plan dni: 02.11 (+0:30)” – patrz uwaga pod tabelą.</t>
+  </si>
+  <si>
+    <t>Umiarkowany, ze zgodą na pracę 8h</t>
+  </si>
+  <si>
+    <t>NP4: orzeczenie PFRON – umiarkowany; „Zgoda na pracę 8h” zaznaczona; kal. Podstawowy system_1_8:16.
+Plan 02.11.2026: 8:00</t>
+  </si>
+  <si>
+    <t>Dzień zapisany.</t>
+  </si>
+  <si>
+    <t>Stopień lekki, bez zgody</t>
+  </si>
+  <si>
+    <t>NP5: orzeczenie PFRON – lekki; zgoda niezaznaczona; kal. Podstawowy system_1_8:16.
+Plan 02.11.2026: 8:00</t>
+  </si>
+  <si>
+    <t>Brak błędu – stopień lekki nie jest objęty limitem 7h</t>
+  </si>
+  <si>
+    <t>Bez orzeczenia</t>
+  </si>
+  <si>
+    <t>NP6: brak orzeczeń; zgoda niezaznaczona (pole jest puste także u osób bez niepełnosprawności); kal. Podstawowy system_1_8:16.
+Plan 02.11.2026: 8:00</t>
+  </si>
+  <si>
+    <t>Orzeczenie ZUS zamiast PFRON</t>
+  </si>
+  <si>
+    <t>NP7: orzeczenie ZUS – całkowita niezdolność do pracy 01.01–31.12.2026 (odpowiadający stopień: umiarkowany), brak orzeczenia PFRON; zgoda niezaznaczona; kal. Podstawowy system_1_8:16.
+Plan 02.11.2026: 8:00</t>
+  </si>
+  <si>
+    <t>Błąd – stopień z orzeczenia ZUS też się liczy</t>
+  </si>
+  <si>
+    <t>Zmiana stopnia w miesiącu – dzień przed zmianą</t>
+  </si>
+  <si>
+    <t>NP8: orzeczenia PFRON – umiarkowany 01.01–15.11.2026, lekki 16.11–31.12.2026; zgoda niezaznaczona; kal. Podstawowy system_1_8:16.
+Plan 13.11.2026: 8:00</t>
+  </si>
+  <si>
+    <t>Błąd – 13.11 obowiązuje stopień umiarkowany</t>
+  </si>
+  <si>
+    <t>Dla dnia (13.11.2026) zaplanowano czas (8:00), a pracownik bez zgody na pracę 8h (stopień niepełnosprawności Umiarkowany) może pracować maksymalnie 7:00 - (pracownik)</t>
+  </si>
+  <si>
+    <t>negatywny</t>
+  </si>
+  <si>
+    <t>Brak komunikatu. Przyczyna: weryfikator czyta stopień z historii pracownika (StopienNiepelnosp / PFRON), które w enova 2610 zwracają JEDNO orzeczenie obowiązujące w okresie zapisu historii – to z najpóźniejszą datą „Obowiązuje od” (tu lekki od 16.11). Okres tego orzeczenia nie obejmuje 13.11 → stopień „Brak”. Do poprawy: szukać orzeczenia obejmującego dany dzień w orzeczeniach PFRON i ZUS pracownika. (Ostrzeżenie o dobie pracowniczej i niedobór normy okresu – skutki danych testowych.)</t>
+  </si>
+  <si>
+    <t>Zmiana stopnia w miesiącu – dzień po zmianie</t>
+  </si>
+  <si>
+    <t>NP8: jak wyżej.
+Plan 16.11.2026: 8:00</t>
+  </si>
+  <si>
+    <t>Brak błędu – od 16.11 stopień lekki</t>
+  </si>
+  <si>
+    <t>Niedobór normy okresu – skutek drugiego dnia testowego z planem 6:00.</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>System równoważny</t>
+  </si>
+  <si>
+    <t>NP9: orzeczenie PFRON – umiarkowany; zgoda niezaznaczona; kal. 3 miesięczny (równoważny).
+Plan 02.11.2026: 8:00</t>
+  </si>
+  <si>
+    <t>Błąd – weryfikator podpięty także do kalendarza 3 miesięczny</t>
+  </si>
+  <si>
+    <t>Uwaga z testu (poza zakresem tego weryfikatora): weryfikator normy okresu rozliczeniowego liczy normę ogólną (np. 160:00 w 11.2026) także dla osób ze stopniem umiarkowanym/znacznym bez zgody, którym przysługuje norma 7h/dobę i 35h/tydzień. Dla takiej osoby oba weryfikatory wykluczają się: niedobór normy okresu podpowiada wydłużenie dnia do 8:00, a ten weryfikator blokuje więcej niż 7:00.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -742,13 +872,7 @@
     </fill>
   </fills>
   <borders count="2">
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
+    <border/>
     <border>
       <left style="thin">
         <color rgb="FFBFBFBF"/>
@@ -762,13 +886,12 @@
       <bottom style="thin">
         <color rgb="FFBFBFBF"/>
       </bottom>
-      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -798,20 +921,15 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normalny" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
@@ -820,10 +938,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
+        <a:sysClr val="windowText"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
+        <a:sysClr val="window"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="1F497D"/>
@@ -1099,1489 +1217,1767 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A20"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="110.7109375" customWidth="1"/>
+    <col min="1" max="1" width="110.71094" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="19.5" x14ac:dyDescent="0.3">
+    <row r="1" ht="19.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3">
       <c r="A3" s="2" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
       <c r="A4" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5">
       <c r="A5" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6">
       <c r="A6" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7">
       <c r="A7" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8">
       <c r="A8" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9">
       <c r="A9" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10">
       <c r="A10" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11">
       <c r="A11" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12">
       <c r="A12" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="13">
+      <c r="A13" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="15">
       <c r="A15" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="16">
       <c r="A16" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="17">
       <c r="A17" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="18">
       <c r="A18" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="19">
       <c r="A19" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="20">
       <c r="A20" t="s">
-        <v>1</v>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s">
+        <v>2</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:G16"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="5.7109375" customWidth="1"/>
-    <col min="2" max="2" width="34.7109375" customWidth="1"/>
-    <col min="3" max="3" width="40.7109375" customWidth="1"/>
-    <col min="4" max="4" width="44.7109375" customWidth="1"/>
-    <col min="5" max="5" width="46.7109375" customWidth="1"/>
-    <col min="6" max="6" width="18.7109375" customWidth="1"/>
-    <col min="7" max="7" width="26.7109375" customWidth="1"/>
+    <col min="2" max="2" width="34.710938" customWidth="1"/>
+    <col min="3" max="3" width="40.710938" customWidth="1"/>
+    <col min="4" max="4" width="44.710938" customWidth="1"/>
+    <col min="5" max="5" width="46.710938" customWidth="1"/>
+    <col min="6" max="6" width="18.710938" customWidth="1"/>
+    <col min="7" max="7" width="26.710938" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="1" ht="17.25">
       <c r="A1" s="3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" s="4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
       <c r="A4" s="5" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" ht="30">
       <c r="A5" s="6" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G5" s="10" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" ht="30">
       <c r="A6" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="E6" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="B6" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="C6" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="D6" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="E6" s="9" t="s">
-        <v>28</v>
-      </c>
       <c r="F6" s="10" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" ht="30">
       <c r="A7" s="6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B7" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="D7" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="C7" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="D7" s="8" t="s">
-        <v>33</v>
-      </c>
       <c r="E7" s="9" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F7" s="10" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G7" s="10" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" ht="30">
       <c r="A8" s="6" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F8" s="10" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9" ht="30">
       <c r="A9" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="D9" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="E9" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="C9" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="D9" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="E9" s="9" t="s">
-        <v>41</v>
-      </c>
       <c r="F9" s="10" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G9" s="10" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" ht="45">
       <c r="A10" s="6" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="F10" s="10" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" ht="30">
       <c r="A11" s="6" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F11" s="10" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G11" s="10" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" ht="30">
       <c r="A12" s="6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F12" s="10" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" ht="45">
       <c r="A13" s="6" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F13" s="10" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G13" s="10" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" ht="45">
       <c r="A14" s="6">
         <v>10</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D14" s="11" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="F14" s="10" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" ht="45">
       <c r="A15" s="6">
         <v>11</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D15" s="11" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F15" s="10" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G15" s="10" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16" ht="45">
       <c r="A16" s="6">
         <v>12</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="E16" s="9" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F16" s="10" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:G13" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <autoFilter ref="A4:G13"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:G10"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="5.7109375" customWidth="1"/>
-    <col min="2" max="2" width="34.7109375" customWidth="1"/>
-    <col min="3" max="3" width="40.7109375" customWidth="1"/>
-    <col min="4" max="4" width="44.7109375" customWidth="1"/>
-    <col min="5" max="5" width="46.7109375" customWidth="1"/>
-    <col min="6" max="6" width="18.7109375" customWidth="1"/>
-    <col min="7" max="7" width="26.7109375" customWidth="1"/>
+    <col min="2" max="2" width="34.710938" customWidth="1"/>
+    <col min="3" max="3" width="40.710938" customWidth="1"/>
+    <col min="4" max="4" width="44.710938" customWidth="1"/>
+    <col min="5" max="5" width="46.710938" customWidth="1"/>
+    <col min="6" max="6" width="18.710938" customWidth="1"/>
+    <col min="7" max="7" width="26.710938" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="1" ht="17.25">
       <c r="A1" s="3" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" s="4" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
       <c r="A4" s="5" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" ht="45">
       <c r="A5" s="6">
         <v>1</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G5" s="10" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="90" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" ht="90">
       <c r="A6" s="6">
         <v>2</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="F6" s="10" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" ht="60">
       <c r="A7" s="6">
         <v>3</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C7" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="D7" s="11" t="s">
+        <v>83</v>
+      </c>
+      <c r="E7" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="D7" s="11" t="s">
-        <v>81</v>
-      </c>
-      <c r="E7" s="9" t="s">
-        <v>78</v>
-      </c>
       <c r="F7" s="10" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G7" s="10" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" ht="60">
       <c r="A8" s="6">
         <v>4</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="F8" s="10" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9" ht="45">
       <c r="A9" s="6">
         <v>5</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F9" s="10" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G9" s="10" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" ht="90" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" ht="90">
       <c r="A10" s="6">
         <v>6</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F10" s="10" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:G10" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <autoFilter ref="A4:G10"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:G10"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="5.7109375" customWidth="1"/>
-    <col min="2" max="2" width="34.7109375" customWidth="1"/>
-    <col min="3" max="3" width="40.7109375" customWidth="1"/>
-    <col min="4" max="4" width="44.7109375" customWidth="1"/>
-    <col min="5" max="5" width="46.7109375" customWidth="1"/>
-    <col min="6" max="6" width="18.7109375" customWidth="1"/>
-    <col min="7" max="7" width="26.7109375" customWidth="1"/>
+    <col min="2" max="2" width="34.710938" customWidth="1"/>
+    <col min="3" max="3" width="40.710938" customWidth="1"/>
+    <col min="4" max="4" width="44.710938" customWidth="1"/>
+    <col min="5" max="5" width="46.710938" customWidth="1"/>
+    <col min="6" max="6" width="18.710938" customWidth="1"/>
+    <col min="7" max="7" width="26.710938" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="1" ht="17.25">
       <c r="A1" s="3" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" s="4" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
       <c r="A4" s="5" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" ht="45">
       <c r="A5" s="6">
         <v>1</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="G5" s="10" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" ht="45">
       <c r="A6" s="6">
         <v>2</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C6" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="E6" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="F6" s="10" t="s">
         <v>100</v>
       </c>
-      <c r="D6" s="8" t="s">
-        <v>101</v>
-      </c>
-      <c r="E6" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="F6" s="10" t="s">
-        <v>98</v>
-      </c>
       <c r="G6" s="10" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="36" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" ht="36">
       <c r="A7" s="6">
         <v>3</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="F7" s="10" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="G7" s="10" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" ht="45">
       <c r="A8" s="6">
         <v>4</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F8" s="10" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" ht="75" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9" ht="75">
       <c r="A9" s="6">
         <v>5</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="F9" s="10" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="G9" s="10" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" ht="60">
       <c r="A10" s="6">
         <v>6</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F10" s="10" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:G10" xr:uid="{00000000-0009-0000-0000-000003000000}"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <autoFilter ref="A4:G10"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:G13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="5.7109375" customWidth="1"/>
-    <col min="2" max="2" width="34.7109375" customWidth="1"/>
-    <col min="3" max="3" width="40.7109375" customWidth="1"/>
-    <col min="4" max="4" width="44.7109375" customWidth="1"/>
-    <col min="5" max="5" width="46.7109375" customWidth="1"/>
-    <col min="6" max="6" width="18.7109375" customWidth="1"/>
-    <col min="7" max="7" width="26.7109375" customWidth="1"/>
+    <col min="2" max="2" width="34.710938" customWidth="1"/>
+    <col min="3" max="3" width="40.710938" customWidth="1"/>
+    <col min="4" max="4" width="44.710938" customWidth="1"/>
+    <col min="5" max="5" width="46.710938" customWidth="1"/>
+    <col min="6" max="6" width="18.710938" customWidth="1"/>
+    <col min="7" max="7" width="26.710938" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="1" ht="17.25">
       <c r="A1" s="3" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" s="4" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
       <c r="A4" s="5" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" ht="45">
       <c r="A5" s="6">
         <v>1</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F5" s="12" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G5" s="10"/>
     </row>
-    <row r="6" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="6" ht="45">
       <c r="A6" s="6">
         <v>2</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="F6" s="12" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G6" s="10"/>
     </row>
-    <row r="7" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="7" ht="45">
       <c r="A7" s="6">
         <v>3</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="F7" s="12" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G7" s="10"/>
     </row>
-    <row r="8" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="8" ht="30">
       <c r="A8" s="6">
         <v>4</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F8" s="12" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G8" s="10"/>
     </row>
-    <row r="9" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="9" ht="30">
       <c r="A9" s="6">
         <v>5</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F9" s="12" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G9" s="10"/>
     </row>
-    <row r="10" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="10" ht="45">
       <c r="A10" s="6">
         <v>6</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F10" s="12" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G10" s="10"/>
     </row>
-    <row r="11" spans="1:7" ht="36" x14ac:dyDescent="0.25">
+    <row r="11" ht="36">
       <c r="A11" s="6">
         <v>7</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="F11" s="12" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G11" s="10"/>
     </row>
-    <row r="12" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="12" ht="30">
       <c r="A12" s="6">
         <v>8</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F12" s="12" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G12" s="10"/>
     </row>
-    <row r="13" spans="1:7" ht="75" x14ac:dyDescent="0.25">
+    <row r="13" ht="75">
       <c r="A13" s="6">
         <v>9</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="F13" s="12" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G13" s="10"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:G13" xr:uid="{00000000-0009-0000-0000-000004000000}"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <autoFilter ref="A4:G13"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:G12"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="5.7109375" customWidth="1"/>
-    <col min="2" max="2" width="34.7109375" customWidth="1"/>
-    <col min="3" max="3" width="40.7109375" customWidth="1"/>
-    <col min="4" max="4" width="44.7109375" customWidth="1"/>
-    <col min="5" max="5" width="46.7109375" customWidth="1"/>
-    <col min="6" max="6" width="18.7109375" customWidth="1"/>
-    <col min="7" max="7" width="26.7109375" customWidth="1"/>
+    <col min="2" max="2" width="34.710938" customWidth="1"/>
+    <col min="3" max="3" width="40.710938" customWidth="1"/>
+    <col min="4" max="4" width="44.710938" customWidth="1"/>
+    <col min="5" max="5" width="46.710938" customWidth="1"/>
+    <col min="6" max="6" width="18.710938" customWidth="1"/>
+    <col min="7" max="7" width="26.710938" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="1" ht="17.25">
       <c r="A1" s="3" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" s="4" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
       <c r="A4" s="5" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" ht="45">
       <c r="A5" s="6">
         <v>1</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F5" s="12" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G5" s="10"/>
     </row>
-    <row r="6" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="6" ht="30">
       <c r="A6" s="6">
         <v>2</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F6" s="12" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G6" s="10"/>
     </row>
-    <row r="7" spans="1:7" ht="48" x14ac:dyDescent="0.25">
+    <row r="7" ht="48">
       <c r="A7" s="6">
         <v>3</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="F7" s="12" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G7" s="10"/>
     </row>
-    <row r="8" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+    <row r="8" ht="60">
       <c r="A8" s="6">
         <v>4</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F8" s="12" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G8" s="10"/>
     </row>
-    <row r="9" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="9" ht="45">
       <c r="A9" s="6">
         <v>5</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="F9" s="12" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G9" s="10"/>
     </row>
-    <row r="10" spans="1:7" ht="36" x14ac:dyDescent="0.25">
+    <row r="10" ht="36">
       <c r="A10" s="6">
         <v>6</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="F10" s="12" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G10" s="10"/>
     </row>
-    <row r="11" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="11" ht="45">
       <c r="A11" s="6">
         <v>7</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F11" s="12" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G11" s="10"/>
     </row>
-    <row r="12" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="12" ht="45">
       <c r="A12" s="6">
         <v>8</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F12" s="12" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G12" s="10"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:G13" xr:uid="{00000000-0009-0000-0000-000006000000}"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <autoFilter ref="A4:G13"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:G11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="5.7109375" customWidth="1"/>
-    <col min="2" max="2" width="34.7109375" customWidth="1"/>
-    <col min="3" max="3" width="40.7109375" customWidth="1"/>
-    <col min="4" max="4" width="44.7109375" customWidth="1"/>
-    <col min="5" max="5" width="46.7109375" customWidth="1"/>
-    <col min="6" max="6" width="18.7109375" customWidth="1"/>
-    <col min="7" max="7" width="26.7109375" customWidth="1"/>
+    <col min="2" max="2" width="34.710938" customWidth="1"/>
+    <col min="3" max="3" width="40.710938" customWidth="1"/>
+    <col min="4" max="4" width="44.710938" customWidth="1"/>
+    <col min="5" max="5" width="46.710938" customWidth="1"/>
+    <col min="6" max="6" width="18.710938" customWidth="1"/>
+    <col min="7" max="7" width="26.710938" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="1" ht="17.25">
       <c r="A1" s="3" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" s="4" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
       <c r="A4" s="5" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" ht="60">
       <c r="A5" s="6">
         <v>1</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="F5" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="G5" s="10"/>
+    </row>
+    <row r="6" ht="30">
+      <c r="A6" s="6">
+        <v>2</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>181</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>182</v>
+      </c>
+      <c r="D6" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="G5" s="10"/>
-    </row>
-    <row r="6" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A6" s="6">
-        <v>2</v>
-      </c>
-      <c r="B6" s="7" t="s">
-        <v>179</v>
-      </c>
-      <c r="C6" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="D6" s="8" t="s">
-        <v>27</v>
-      </c>
       <c r="E6" s="9" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F6" s="12" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G6" s="10"/>
     </row>
-    <row r="7" spans="1:7" ht="48" x14ac:dyDescent="0.25">
+    <row r="7" ht="48">
       <c r="A7" s="6">
         <v>3</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="F7" s="12" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G7" s="10"/>
     </row>
-    <row r="8" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+    <row r="8" ht="60">
       <c r="A8" s="6">
         <v>4</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F8" s="12" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G8" s="10"/>
     </row>
-    <row r="9" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+    <row r="9" ht="60">
       <c r="A9" s="6">
         <v>5</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F9" s="12" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G9" s="10"/>
     </row>
-    <row r="10" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+    <row r="10" ht="60">
       <c r="A10" s="6">
         <v>6</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="F10" s="12" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G10" s="10"/>
     </row>
-    <row r="11" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="11" ht="45">
       <c r="A11" s="6">
         <v>7</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F11" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="G11" s="10"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:G13"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="5.7109375" customWidth="1"/>
+    <col min="2" max="2" width="34.710938" customWidth="1"/>
+    <col min="3" max="3" width="40.710938" customWidth="1"/>
+    <col min="4" max="4" width="44.710938" customWidth="1"/>
+    <col min="5" max="5" width="46.710938" customWidth="1"/>
+    <col min="6" max="6" width="18.710938" customWidth="1"/>
+    <col min="7" max="7" width="26.710938" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="17.25">
+      <c r="A1" s="3" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" ht="75">
+      <c r="A5" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>201</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>202</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>159</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>203</v>
+      </c>
+      <c r="F5" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="G5" s="10" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="6" ht="60">
+      <c r="A6" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>205</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>206</v>
+      </c>
+      <c r="D6" s="11" t="s">
+        <v>132</v>
+      </c>
+      <c r="E6" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="F6" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="G6" s="10" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="7" ht="75">
+      <c r="A7" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>208</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="D7" s="11" t="s">
+        <v>159</v>
+      </c>
+      <c r="E7" s="9" t="s">
+        <v>210</v>
+      </c>
+      <c r="F7" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="G7" s="10" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="8" ht="60">
+      <c r="A8" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>213</v>
+      </c>
+      <c r="D8" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="G11" s="10"/>
+      <c r="E8" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="F8" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="G8" s="10" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="9" ht="60">
+      <c r="A9" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>215</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>216</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>217</v>
+      </c>
+      <c r="E9" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="F9" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="G9" s="10" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="10" ht="75">
+      <c r="A10" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>218</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>219</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="E10" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="F10" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="G10" s="10" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="11" ht="90">
+      <c r="A11" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="D11" s="11" t="s">
+        <v>222</v>
+      </c>
+      <c r="E11" s="9" t="s">
+        <v>203</v>
+      </c>
+      <c r="F11" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="G11" s="10" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" ht="300">
+      <c r="A12" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>223</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="D12" s="8" t="s">
+        <v>225</v>
+      </c>
+      <c r="E12" s="9" t="s">
+        <v>226</v>
+      </c>
+      <c r="F12" s="12" t="s">
+        <v>227</v>
+      </c>
+      <c r="G12" s="10" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="13" ht="45">
+      <c r="A13" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>230</v>
+      </c>
+      <c r="D13" s="11" t="s">
+        <v>231</v>
+      </c>
+      <c r="E13" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="F13" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="G13" s="10" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="14" ht="75" customHeight="1">
+      <c r="A14" s="6" t="s">
+        <v>233</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>234</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>235</v>
+      </c>
+      <c r="D14" s="8" t="s">
+        <v>236</v>
+      </c>
+      <c r="E14" s="9" t="s">
+        <v>203</v>
+      </c>
+      <c r="F14" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="G14" s="10" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16" ht="45" customHeight="1">
+      <c r="B16" s="13" t="s">
+        <v>237</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:G13" xr:uid="{00000000-0009-0000-0000-000007000000}"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <autoFilter ref="A4:G14"/>
+  <mergeCells count="1">
+    <mergeCell ref="B16:G16"/>
+  </mergeCells>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Weryfikator ilosci dni wolnych (1036): test na zywo w bazie Al OK (DW1-DW3), scenariusze 7-9 w arkuszu, dokumentacja nowej reguly nadmiaru
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0182ohJ4QbL8h7nxDhghZj3k
</commit_message>
<xml_diff>
--- a/Weryfikatory czasu pracy/Scenariusze testowe weryfikatorow czasu pracy.xlsx
+++ b/Weryfikatory czasu pracy/Scenariusze testowe weryfikatorow czasu pracy.xlsx
@@ -23,7 +23,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Okres zatrudnienia'!$A$4:$G$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Norma okresu rozliczeniowego'!$A$4:$G$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Ilość dni wolnych'!$A$4:$G$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Ilość dni wolnych'!$A$4:$G$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Norma dobowa'!$A$4:$G$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Praca w normie wg planu'!$A$4:$G$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Magazyn nadgodzin - umowy'!$A$4:$G$13</definedName>
@@ -335,7 +335,7 @@
     <t>Weryfikator: Ilość dni wolnych</t>
   </si>
   <si>
-    <t>Weryfikator ilości dni okresu rozliczeniowego – na zapisie całego kalendarza. Sprawdza liczbę dni wolnych: wymagana = dni kalendarzowe okresu − dni robocze normy kodeksowej (CzasDni.Dni). Tryb ścisły vs tolerancyjny zależy od bieżącej daty zapisu.</t>
+    <t>Weryfikator ilości dni okresu rozliczeniowego – na zapisie całego kalendarza. Sprawdza liczbę dni wolnych: wymagana = dni kalendarzowe okresu − dni robocze normy kodeksowej (CzasDni.Dni). Tryb ścisły vs tolerancyjny zależy od bieżącej daty zapisu. Od 15.10.2026: za mało dni wolnych = zawsze błąd; zbyt dużo dni wolnych = błąd tylko, gdy godziny planu w okresie przekraczają normę (np. system równoważny po 12h może mieć więcej dni wolnych).</t>
   </si>
   <si>
     <t>Okres miesięczny, sobota + niedziela zamienione na pracę, nic więcej</t>
@@ -362,16 +362,22 @@
     <t>Brak błędu – liczba dni wolnych = wymagana.</t>
   </si>
   <si>
-    <t>Okres miesięczny, jeden dzień roboczy jawnie oznaczony jako wolny</t>
+    <t>Okres miesięczny, jeden dzień roboczy jawnie oznaczony jako wolny (godziny poniżej normy)</t>
   </si>
   <si>
     <t>Okres 1-miesięczny. Jeden dzień roboczy jawnie oznaczony jako wolny, nic więcej.</t>
   </si>
   <si>
-    <t>Błąd „zbyt dużo dni wolnych” o 1 – trzeba dodać dzień pracy.</t>
-  </si>
-  <si>
-    <t>Zaplanowano zbyt dużo dni wolnych (X) wobec wymaganej liczby (Y) w okresie rozliczeniowym (…). Trzeba dodać dni pracy: (X−Y).</t>
+    <t>Brak błędu weryfikatora dni wolnych – godziny planu (norma − 8h) nie przekraczają normy. Niedobór godzin zgłasza weryfikator normy okresu (37). [Przed 15.10.2026: błąd „zbyt dużo dni wolnych”.]</t>
+  </si>
+  <si>
+    <t>brak błędu (weryfikator 37: „Nie da się już osiągnąć normy godzin…”)</t>
+  </si>
+  <si>
+    <t>Do powtórki</t>
+  </si>
+  <si>
+    <t>Wcześniej Pozytywny przy starej regule (błąd nadmiaru). Ten sam przypadek godzinowy pokrywa scenariusz 7.</t>
   </si>
   <si>
     <t>Okres 3-miesięczny, jesteśmy w miesiącu 1, dodatkowy dzień pracy w mies. 1</t>
@@ -402,6 +408,48 @@
   </si>
   <si>
     <t>Za mało dni wolnych (X) wobec wymaganej liczby (Y) w okresie rozliczeniowym (…)</t>
+  </si>
+  <si>
+    <t>System równoważny, więcej dni wolnych, godziny w normie</t>
+  </si>
+  <si>
+    <t>Pracownik DW1 (TEST-DW1), kal. 1075 „Równoważny system_1_8:16” (okres 1-mies.), 11.2026: 13 dni × 12:00 + 30.11 × 4:00 = 160:00, 6 dni roboczych jawnie wolnych → 16 dni wolnych (wymagane 10). W programie 30.11 zmienione z 5:00 na 4:00.</t>
+  </si>
+  <si>
+    <t>Brak błędu – nadmiar dni wolnych dopuszczalny, bo godziny = norma.</t>
+  </si>
+  <si>
+    <t>15.10.2026, baza Al, MCP: brak komunikatów, zapis przeszedł.</t>
+  </si>
+  <si>
+    <t>System równoważny, więcej dni wolnych, godziny ponad normę</t>
+  </si>
+  <si>
+    <t>Pracownik DW2 (TEST-DW2), kal. 1075, 11.2026: 14 dni × 12:00 = 168:00, 16 dni wolnych. W programie 30.11 zmienione z 11:00 na 12:00.</t>
+  </si>
+  <si>
+    <t>Błąd „zbyt dużo dni wolnych … przy przekroczonej normie godzin” (+ weryfikator 37 „Przekroczono limit godzin”).</t>
+  </si>
+  <si>
+    <t>Zaplanowano zbyt dużo dni wolnych (16) wobec wymaganej liczby (10) przy przekroczonej normie godzin (zaplanowano 168:00, norma 160:00) w okresie rozliczeniowym (…). Trzeba dodać dni pracy: 6.</t>
+  </si>
+  <si>
+    <t>15.10.2026, baza Al, MCP: komunikat zgodny co do liczb; zmiana wycofana.</t>
+  </si>
+  <si>
+    <t>Za mało dni wolnych przy godzinach w normie</t>
+  </si>
+  <si>
+    <t>Pracownik DW3 (TEST-DW3), kal. 1075, 11.2026: 18 dni × 8:00 + 2 dni × 4:00 + sobota 07.11 × 8:00 = 160:00, 21 dni pracy → 9 dni wolnych. W programie 07.11 zmienione z 7:00 na 8:00.</t>
+  </si>
+  <si>
+    <t>Błąd „za mało dni wolnych” – mimo że godziny = norma.</t>
+  </si>
+  <si>
+    <t>Za mało dni wolnych (9) wobec wymaganej liczby (10) w okresie rozliczeniowym (…). Trzeba jeszcze zamienić na wolne dni robocze: 1 (dostępnych dni roboczych bez jawnego wpisu: 0).</t>
+  </si>
+  <si>
+    <t>15.10.2026, baza Al, MCP: komunikat zgodny; zmiana wycofana.</t>
   </si>
   <si>
     <t>Weryfikator: Norma dobowa</t>
@@ -1939,7 +1987,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" ht="36">
+    <row r="7" ht="75">
       <c r="A7" s="6">
         <v>3</v>
       </c>
@@ -1956,10 +2004,10 @@
         <v>107</v>
       </c>
       <c r="F7" s="10" t="s">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="G7" s="10" t="s">
-        <v>2</v>
+        <v>109</v>
       </c>
     </row>
     <row r="8" ht="45">
@@ -1967,13 +2015,13 @@
         <v>4</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E8" s="9" t="s">
         <v>30</v>
@@ -1990,13 +2038,13 @@
         <v>5</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="E9" s="9" t="s">
         <v>99</v>
@@ -2013,16 +2061,16 @@
         <v>6</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="F10" s="10" t="s">
         <v>100</v>
@@ -2031,8 +2079,77 @@
         <v>2</v>
       </c>
     </row>
+    <row r="11" ht="90">
+      <c r="A11" s="6">
+        <v>7</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="D11" s="11" t="s">
+        <v>122</v>
+      </c>
+      <c r="E11" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="F11" s="10" t="s">
+        <v>100</v>
+      </c>
+      <c r="G11" s="10" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="12" ht="60">
+      <c r="A12" s="6">
+        <v>8</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="D12" s="11" t="s">
+        <v>126</v>
+      </c>
+      <c r="E12" s="9" t="s">
+        <v>127</v>
+      </c>
+      <c r="F12" s="10" t="s">
+        <v>100</v>
+      </c>
+      <c r="G12" s="10" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="13" ht="75">
+      <c r="A13" s="6">
+        <v>9</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="D13" s="11" t="s">
+        <v>131</v>
+      </c>
+      <c r="E13" s="9" t="s">
+        <v>132</v>
+      </c>
+      <c r="F13" s="10" t="s">
+        <v>100</v>
+      </c>
+      <c r="G13" s="10" t="s">
+        <v>133</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:G10"/>
+  <autoFilter ref="A4:G13"/>
 </worksheet>
 </file>
 
@@ -2051,12 +2168,12 @@
   <sheetData>
     <row r="1" ht="17.25">
       <c r="A1" s="3" t="s">
-        <v>118</v>
+        <v>134</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="s">
-        <v>119</v>
+        <v>135</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
@@ -2087,10 +2204,10 @@
         <v>1</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>120</v>
+        <v>136</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>121</v>
+        <v>137</v>
       </c>
       <c r="D5" s="8" t="s">
         <v>29</v>
@@ -2108,16 +2225,16 @@
         <v>2</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>122</v>
+        <v>138</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>123</v>
+        <v>139</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>124</v>
+        <v>140</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>125</v>
+        <v>141</v>
       </c>
       <c r="F6" s="12" t="s">
         <v>31</v>
@@ -2129,16 +2246,16 @@
         <v>3</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>126</v>
+        <v>142</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>127</v>
+        <v>143</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>128</v>
+        <v>144</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>129</v>
+        <v>145</v>
       </c>
       <c r="F7" s="12" t="s">
         <v>31</v>
@@ -2150,13 +2267,13 @@
         <v>4</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>130</v>
+        <v>146</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>131</v>
+        <v>147</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>132</v>
+        <v>148</v>
       </c>
       <c r="E8" s="9" t="s">
         <v>30</v>
@@ -2171,13 +2288,13 @@
         <v>5</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>133</v>
+        <v>149</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>134</v>
+        <v>150</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>135</v>
+        <v>151</v>
       </c>
       <c r="E9" s="9" t="s">
         <v>30</v>
@@ -2192,13 +2309,13 @@
         <v>6</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>136</v>
+        <v>152</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>137</v>
+        <v>153</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>138</v>
+        <v>154</v>
       </c>
       <c r="E10" s="9" t="s">
         <v>30</v>
@@ -2213,16 +2330,16 @@
         <v>7</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>139</v>
+        <v>155</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>140</v>
+        <v>156</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>141</v>
+        <v>157</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>142</v>
+        <v>158</v>
       </c>
       <c r="F11" s="12" t="s">
         <v>31</v>
@@ -2234,13 +2351,13 @@
         <v>8</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>143</v>
+        <v>159</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>144</v>
+        <v>160</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>145</v>
+        <v>161</v>
       </c>
       <c r="E12" s="9" t="s">
         <v>30</v>
@@ -2255,16 +2372,16 @@
         <v>9</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>146</v>
+        <v>162</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>147</v>
+        <v>163</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>148</v>
+        <v>164</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>149</v>
+        <v>165</v>
       </c>
       <c r="F13" s="12" t="s">
         <v>31</v>
@@ -2291,12 +2408,12 @@
   <sheetData>
     <row r="1" ht="17.25">
       <c r="A1" s="3" t="s">
-        <v>150</v>
+        <v>166</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="s">
-        <v>151</v>
+        <v>167</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
@@ -2327,10 +2444,10 @@
         <v>1</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>152</v>
+        <v>168</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>153</v>
+        <v>169</v>
       </c>
       <c r="D5" s="8" t="s">
         <v>29</v>
@@ -2348,13 +2465,13 @@
         <v>2</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>154</v>
+        <v>170</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>155</v>
+        <v>171</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>156</v>
+        <v>172</v>
       </c>
       <c r="E6" s="9" t="s">
         <v>30</v>
@@ -2369,16 +2486,16 @@
         <v>3</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>157</v>
+        <v>173</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>158</v>
+        <v>174</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>159</v>
+        <v>175</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>160</v>
+        <v>176</v>
       </c>
       <c r="F7" s="12" t="s">
         <v>31</v>
@@ -2390,10 +2507,10 @@
         <v>4</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>161</v>
+        <v>177</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>162</v>
+        <v>178</v>
       </c>
       <c r="D8" s="8" t="s">
         <v>29</v>
@@ -2411,16 +2528,16 @@
         <v>5</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>163</v>
+        <v>179</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>164</v>
+        <v>180</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>165</v>
+        <v>181</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>166</v>
+        <v>182</v>
       </c>
       <c r="F9" s="12" t="s">
         <v>31</v>
@@ -2432,16 +2549,16 @@
         <v>6</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>167</v>
+        <v>183</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>168</v>
+        <v>184</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>169</v>
+        <v>185</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>170</v>
+        <v>186</v>
       </c>
       <c r="F10" s="12" t="s">
         <v>31</v>
@@ -2453,10 +2570,10 @@
         <v>7</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>171</v>
+        <v>187</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>172</v>
+        <v>188</v>
       </c>
       <c r="D11" s="8" t="s">
         <v>29</v>
@@ -2474,13 +2591,13 @@
         <v>8</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>173</v>
+        <v>189</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>174</v>
+        <v>190</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>175</v>
+        <v>191</v>
       </c>
       <c r="E12" s="9" t="s">
         <v>30</v>
@@ -2510,12 +2627,12 @@
   <sheetData>
     <row r="1" ht="17.25">
       <c r="A1" s="3" t="s">
-        <v>176</v>
+        <v>192</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="s">
-        <v>177</v>
+        <v>193</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
@@ -2546,16 +2663,16 @@
         <v>1</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>178</v>
+        <v>194</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>179</v>
+        <v>195</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>159</v>
+        <v>175</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>180</v>
+        <v>196</v>
       </c>
       <c r="F5" s="12" t="s">
         <v>31</v>
@@ -2567,10 +2684,10 @@
         <v>2</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>181</v>
+        <v>197</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>182</v>
+        <v>198</v>
       </c>
       <c r="D6" s="8" t="s">
         <v>29</v>
@@ -2588,16 +2705,16 @@
         <v>3</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>183</v>
+        <v>199</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>184</v>
+        <v>200</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>185</v>
+        <v>201</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>186</v>
+        <v>202</v>
       </c>
       <c r="F7" s="12" t="s">
         <v>31</v>
@@ -2609,10 +2726,10 @@
         <v>4</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>187</v>
+        <v>203</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>188</v>
+        <v>204</v>
       </c>
       <c r="D8" s="8" t="s">
         <v>29</v>
@@ -2630,13 +2747,13 @@
         <v>5</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>189</v>
+        <v>205</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>190</v>
+        <v>206</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>191</v>
+        <v>207</v>
       </c>
       <c r="E9" s="9" t="s">
         <v>30</v>
@@ -2651,16 +2768,16 @@
         <v>6</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>192</v>
+        <v>208</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>193</v>
+        <v>209</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>194</v>
+        <v>210</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>195</v>
+        <v>211</v>
       </c>
       <c r="F10" s="12" t="s">
         <v>31</v>
@@ -2672,13 +2789,13 @@
         <v>7</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>196</v>
+        <v>212</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>197</v>
+        <v>213</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>198</v>
+        <v>214</v>
       </c>
       <c r="E11" s="9" t="s">
         <v>30</v>
@@ -2708,12 +2825,12 @@
   <sheetData>
     <row r="1" ht="17.25">
       <c r="A1" s="3" t="s">
-        <v>199</v>
+        <v>215</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="s">
-        <v>200</v>
+        <v>216</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
@@ -2744,22 +2861,22 @@
         <v>26</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>201</v>
+        <v>217</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>202</v>
+        <v>218</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>159</v>
+        <v>175</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>203</v>
+        <v>219</v>
       </c>
       <c r="F5" s="12" t="s">
         <v>31</v>
       </c>
       <c r="G5" s="10" t="s">
-        <v>204</v>
+        <v>220</v>
       </c>
     </row>
     <row r="6" ht="60">
@@ -2767,13 +2884,13 @@
         <v>32</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>205</v>
+        <v>221</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>206</v>
+        <v>222</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>132</v>
+        <v>148</v>
       </c>
       <c r="E6" s="9" t="s">
         <v>30</v>
@@ -2782,7 +2899,7 @@
         <v>31</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>207</v>
+        <v>223</v>
       </c>
     </row>
     <row r="7" ht="75">
@@ -2790,22 +2907,22 @@
         <v>36</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>208</v>
+        <v>224</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>209</v>
+        <v>225</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>159</v>
+        <v>175</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>210</v>
+        <v>226</v>
       </c>
       <c r="F7" s="12" t="s">
         <v>31</v>
       </c>
       <c r="G7" s="10" t="s">
-        <v>211</v>
+        <v>227</v>
       </c>
     </row>
     <row r="8" ht="60">
@@ -2813,10 +2930,10 @@
         <v>39</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>212</v>
+        <v>228</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>213</v>
+        <v>229</v>
       </c>
       <c r="D8" s="8" t="s">
         <v>29</v>
@@ -2828,7 +2945,7 @@
         <v>31</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>214</v>
+        <v>230</v>
       </c>
     </row>
     <row r="9" ht="60">
@@ -2836,13 +2953,13 @@
         <v>44</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>215</v>
+        <v>231</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>216</v>
+        <v>232</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>217</v>
+        <v>233</v>
       </c>
       <c r="E9" s="9" t="s">
         <v>30</v>
@@ -2851,7 +2968,7 @@
         <v>31</v>
       </c>
       <c r="G9" s="10" t="s">
-        <v>214</v>
+        <v>230</v>
       </c>
     </row>
     <row r="10" ht="75">
@@ -2859,10 +2976,10 @@
         <v>47</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>218</v>
+        <v>234</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>219</v>
+        <v>235</v>
       </c>
       <c r="D10" s="8" t="s">
         <v>29</v>
@@ -2874,7 +2991,7 @@
         <v>31</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>214</v>
+        <v>230</v>
       </c>
     </row>
     <row r="11" ht="90">
@@ -2882,16 +2999,16 @@
         <v>51</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>220</v>
+        <v>236</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>221</v>
+        <v>237</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>222</v>
+        <v>238</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>203</v>
+        <v>219</v>
       </c>
       <c r="F11" s="12" t="s">
         <v>31</v>
@@ -2905,22 +3022,22 @@
         <v>55</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>223</v>
+        <v>239</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>224</v>
+        <v>240</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>225</v>
+        <v>241</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>226</v>
+        <v>242</v>
       </c>
       <c r="F12" s="12" t="s">
-        <v>227</v>
+        <v>243</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>228</v>
+        <v>244</v>
       </c>
     </row>
     <row r="13" ht="45">
@@ -2928,13 +3045,13 @@
         <v>58</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>229</v>
+        <v>245</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>230</v>
+        <v>246</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>231</v>
+        <v>247</v>
       </c>
       <c r="E13" s="9" t="s">
         <v>30</v>
@@ -2943,24 +3060,24 @@
         <v>31</v>
       </c>
       <c r="G13" s="10" t="s">
-        <v>232</v>
+        <v>248</v>
       </c>
     </row>
     <row r="14" ht="75" customHeight="1">
       <c r="A14" s="6" t="s">
-        <v>233</v>
+        <v>249</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>234</v>
+        <v>250</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>235</v>
+        <v>251</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>236</v>
+        <v>252</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>203</v>
+        <v>219</v>
       </c>
       <c r="F14" s="12" t="s">
         <v>31</v>
@@ -2971,7 +3088,7 @@
     </row>
     <row r="16" ht="45" customHeight="1">
       <c r="B16" s="13" t="s">
-        <v>237</v>
+        <v>253</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Weryfikator 2069: scenariusz 8 (zmiana stopnia w trakcie zapisu historii) pozytywny po poprawce - test live 19.10.2026, 10/10
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018SWEtN1iMr88RMmUUHSCbE
</commit_message>
<xml_diff>
--- a/Weryfikatory czasu pracy/Scenariusze testowe weryfikatorow czasu pracy.xlsx
+++ b/Weryfikatory czasu pracy/Scenariusze testowe weryfikatorow czasu pracy.xlsx
@@ -807,10 +807,7 @@
     <t>Dla dnia (13.11.2026) zaplanowano czas (8:00), a pracownik bez zgody na pracę 8h (stopień niepełnosprawności Umiarkowany) może pracować maksymalnie 7:00 - (pracownik)</t>
   </si>
   <si>
-    <t>negatywny</t>
-  </si>
-  <si>
-    <t>Brak komunikatu. Przyczyna: weryfikator czyta stopień z historii pracownika (StopienNiepelnosp / PFRON), które w enova 2610 zwracają JEDNO orzeczenie obowiązujące w okresie zapisu historii – to z najpóźniejszą datą „Obowiązuje od” (tu lekki od 16.11). Okres tego orzeczenia nie obejmuje 13.11 → stopień „Brak”. Do poprawy: szukać orzeczenia obejmującego dany dzień w orzeczeniach PFRON i ZUS pracownika. (Ostrzeżenie o dobie pracowniczej i niedobór normy okresu – skutki danych testowych.)</t>
+    <t>Test 15.10.2026: negatywny (brak komunikatu - stopień czytany z historii pracownika, StopienNiepelnosp/PFRON, które w enova 2610 zwracają jedno orzeczenie z zapisu historii). Poprawka 19.10.2026: stopień z metody enova Pracownik.StopienNiepelnosprawnosciNaDzien (orzeczenia PFRON/ZUS obowiązujące w danym dniu). Powtórka 19.10.2026: komunikat jak oczekiwany - pozytywny. (Niedobór normy okresu - skutek danych testowych.)</t>
   </si>
   <si>
     <t>Zmiana stopnia w miesiącu – dzień po zmianie</t>
@@ -823,7 +820,7 @@
     <t>Brak błędu – od 16.11 stopień lekki</t>
   </si>
   <si>
-    <t>Niedobór normy okresu – skutek drugiego dnia testowego z planem 6:00.</t>
+    <t>Niedobór normy okresu - skutek drugiego dnia testowego z planem 6:00. Powtórka 19.10.2026 po poprawce: brak błędu tego weryfikatora - pozytywny.</t>
   </si>
   <si>
     <t>10</t>
@@ -3017,7 +3014,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" ht="300">
+    <row r="12" ht="270">
       <c r="A12" s="6" t="s">
         <v>55</v>
       </c>
@@ -3034,24 +3031,24 @@
         <v>242</v>
       </c>
       <c r="F12" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="G12" s="10" t="s">
         <v>243</v>
       </c>
-      <c r="G12" s="10" t="s">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="13" ht="45">
+    </row>
+    <row r="13" ht="90">
       <c r="A13" s="6" t="s">
         <v>58</v>
       </c>
       <c r="B13" s="7" t="s">
+        <v>244</v>
+      </c>
+      <c r="C13" s="7" t="s">
         <v>245</v>
       </c>
-      <c r="C13" s="7" t="s">
+      <c r="D13" s="11" t="s">
         <v>246</v>
-      </c>
-      <c r="D13" s="11" t="s">
-        <v>247</v>
       </c>
       <c r="E13" s="9" t="s">
         <v>30</v>
@@ -3060,21 +3057,21 @@
         <v>31</v>
       </c>
       <c r="G13" s="10" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="14" ht="75" customHeight="1">
       <c r="A14" s="6" t="s">
+        <v>248</v>
+      </c>
+      <c r="B14" s="7" t="s">
         <v>249</v>
       </c>
-      <c r="B14" s="7" t="s">
+      <c r="C14" s="7" t="s">
         <v>250</v>
       </c>
-      <c r="C14" s="7" t="s">
+      <c r="D14" s="8" t="s">
         <v>251</v>
-      </c>
-      <c r="D14" s="8" t="s">
-        <v>252</v>
       </c>
       <c r="E14" s="9" t="s">
         <v>219</v>
@@ -3088,7 +3085,7 @@
     </row>
     <row r="16" ht="45" customHeight="1">
       <c r="B16" s="13" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Weryfikator 2069: powtorka scenariuszy NP1-NP9 na kalendarzach klienta _N (19.10.2026) - 10/10 pozytywnie, norma okresu 37 liczy 7h i nie koliduje; XML danych testowych z kalendarzami _N
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018SWEtN1iMr88RMmUUHSCbE
</commit_message>
<xml_diff>
--- a/Weryfikatory czasu pracy/Scenariusze testowe weryfikatorow czasu pracy.xlsx
+++ b/Weryfikatory czasu pracy/Scenariusze testowe weryfikatorow czasu pracy.xlsx
@@ -718,86 +718,92 @@
     <t>Weryfikator: Brak zgody na pracę 8h</t>
   </si>
   <si>
-    <t>Weryfikator dnia planu pracy (Dzień planu), definicja „A1_Brak zgody na pracę 8h”. Pracownik ze stopniem umiarkowanym lub znacznym (orzeczenie PFRON albo ZUS), bez zaznaczonego na etacie pola „Zgoda na pracę 8h”, nie może mieć zaplanowanych więcej niż 7:00 na dobę. Na bazie testowej: kalendarze 3 miesięczny i Podstawowy system_1_8:16 – Błąd. Test 15.10.2026 na bazie Al, pracownicy NP1–NP9 (ImportyXML/Weryfikator brak zgody 8h - pracownicy i plan.xml; orzeczenia dodane w programie).</t>
+    <t>Weryfikator dnia planu pracy (Dzień planu), definicja „A1_Brak zgody na pracę 8h”. Pracownik ze stopniem umiarkowanym lub znacznym (orzeczenie PFRON albo ZUS), bez zaznaczonego na etacie pola „Zgoda na pracę 8h”, nie może mieć zaplanowanych więcej niż 7:00 na dobę. Podpięty jako Błąd do kalendarzy klienta, w tym wersji _N dla osób z niepełnosprawnością. Test 15.10.2026 na bazie Al, pracownicy NP1–NP9 (ImportyXML/Weryfikator brak zgody 8h - pracownicy i plan.xml; orzeczenia dodane w programie). Powtórka 19.10.2026 po poprawce odczytu stopnia (orzeczenie obowiązujące w danym dniu) i po podpięciu kalendarzy klienta _N: bez zgody - Podstawowy system_1_8:15_N (norma 7:00), ze zgodą / stopień lekki / bez orzeczenia - Podstawowy system_1_8:16_N (norma 8:00), system równoważny - Równoważny system_3_8:15_N (norma 7:00).</t>
   </si>
   <si>
     <t>Umiarkowany, bez zgody, plan 8:00</t>
   </si>
   <si>
-    <t>NP1: orzeczenie PFRON – umiarkowany 01.01–31.12.2026; „Zgoda na pracę 8h” niezaznaczona; kal. Podstawowy system_1_8:16.
+    <t>NP1: orzeczenie PFRON – umiarkowany 01.01–31.12.2026; „Zgoda na pracę 8h” niezaznaczona; kal. Podstawowy system_1_8:15_N (19.10; wcześniej Podstawowy system_1_8:16).
 Plan 02.11.2026: 8:00</t>
   </si>
   <si>
     <t>Dla dnia (2.11.2026) zaplanowano czas (8:00), a pracownik bez zgody na pracę 8h (stopień niepełnosprawności Umiarkowany) może pracować maksymalnie 7:00 - (pracownik)</t>
   </si>
   <si>
-    <t>Komunikat pojawia się już przy zmianie czasu strefy, przed zapisem.</t>
+    <t>Powtórka 19.10.2026 (kal. 8:15_N): komunikat jak oczekiwany. Razem z nim błąd normy dobowej (7:00) i niedobór normy okresu - norma okresu liczona już z 7h (140:00), bez podpowiedzi wydłużania dnia ponad 7:00.</t>
   </si>
   <si>
     <t>Umiarkowany, bez zgody, plan 7:00 (granica)</t>
   </si>
   <si>
-    <t>NP2: jak NP1.
-Plan 02.11.2026: 7:00 (dodatkowo sobota 07.11: 1:00, żeby nie wywołać niedoboru normy okresu)</t>
-  </si>
-  <si>
-    <t>Odezwał się tylko weryfikator dni wolnych – skutek pomocniczej soboty, nie tego weryfikatora.</t>
+    <t>NP2: jak NP1 (kal. Podstawowy system_1_8:15_N od 19.10).
+Plan 02.11.2026: 7:00 (dodatkowo sobota 07.11: 1:00 - pozostałość testu 15.10)</t>
+  </si>
+  <si>
+    <t>Powtórka 19.10.2026 (kal. 8:15_N): brak błędu tego weryfikatora. Pomocnicza sobota nie jest już potrzebna - jedyny komunikat to niedobór normy okresu (140:00) wynikający z danych testowych (2 dni planu).</t>
   </si>
   <si>
     <t>Znaczny, bez zgody, plan 7:30</t>
   </si>
   <si>
-    <t>NP3: orzeczenie PFRON – znaczny 01.01–31.12.2026; zgoda niezaznaczona; kal. Podstawowy system_1_8:16.
+    <t>NP3: orzeczenie PFRON – znaczny 01.01–31.12.2026; zgoda niezaznaczona; kal. Podstawowy system_1_8:15_N (19.10; wcześniej Podstawowy system_1_8:16).
 Plan 02.11.2026: 7:30</t>
   </si>
   <si>
     <t>Dla dnia (2.11.2026) zaplanowano czas (7:30), a pracownik bez zgody na pracę 8h (stopień niepełnosprawności Znaczny) może pracować maksymalnie 7:00 - (pracownik)</t>
   </si>
   <si>
-    <t>Jednocześnie norma okresu rozliczeniowego żąda 160:00 i podpowiada „Wydłuż plan dni: 02.11 (+0:30)” – patrz uwaga pod tabelą.</t>
+    <t>Powtórka 19.10.2026 (kal. 8:15_N): komunikat jak oczekiwany, razem z błędem normy dobowej (7:00). Norma okresu 140:00, bez podpowiedzi wydłużania dnia - konflikt z normą okresu ustąpił.</t>
   </si>
   <si>
     <t>Umiarkowany, ze zgodą na pracę 8h</t>
   </si>
   <si>
-    <t>NP4: orzeczenie PFRON – umiarkowany; „Zgoda na pracę 8h” zaznaczona; kal. Podstawowy system_1_8:16.
+    <t>NP4: orzeczenie PFRON – umiarkowany; „Zgoda na pracę 8h” zaznaczona; kal. Podstawowy system_1_8:16_N (19.10; wcześniej Podstawowy system_1_8:16).
 Plan 02.11.2026: 8:00</t>
   </si>
   <si>
-    <t>Dzień zapisany.</t>
+    <t>Powtórka 19.10.2026 (kal. 8:16_N): brak błędu tego weryfikatora i normy dobowej; tylko niedobór normy okresu (160:00) - skutek danych testowych.</t>
   </si>
   <si>
     <t>Stopień lekki, bez zgody</t>
   </si>
   <si>
-    <t>NP5: orzeczenie PFRON – lekki; zgoda niezaznaczona; kal. Podstawowy system_1_8:16.
+    <t>NP5: orzeczenie PFRON – lekki; zgoda niezaznaczona; kal. Podstawowy system_1_8:16_N (19.10; wcześniej Podstawowy system_1_8:16).
 Plan 02.11.2026: 8:00</t>
   </si>
   <si>
     <t>Brak błędu – stopień lekki nie jest objęty limitem 7h</t>
   </si>
   <si>
+    <t>Powtórka 19.10.2026 (kal. 8:16_N): brak błędu tego weryfikatora; tylko niedobór normy okresu - skutek danych testowych.</t>
+  </si>
+  <si>
     <t>Bez orzeczenia</t>
   </si>
   <si>
-    <t>NP6: brak orzeczeń; zgoda niezaznaczona (pole jest puste także u osób bez niepełnosprawności); kal. Podstawowy system_1_8:16.
+    <t>NP6: brak orzeczeń; zgoda niezaznaczona (pole jest puste także u osób bez niepełnosprawności); kal. Podstawowy system_1_8:16_N (19.10; wcześniej Podstawowy system_1_8:16).
 Plan 02.11.2026: 8:00</t>
   </si>
   <si>
     <t>Orzeczenie ZUS zamiast PFRON</t>
   </si>
   <si>
-    <t>NP7: orzeczenie ZUS – całkowita niezdolność do pracy 01.01–31.12.2026 (odpowiadający stopień: umiarkowany), brak orzeczenia PFRON; zgoda niezaznaczona; kal. Podstawowy system_1_8:16.
+    <t>NP7: orzeczenie ZUS – całkowita niezdolność do pracy 01.01–31.12.2026 (odpowiadający stopień: umiarkowany), brak orzeczenia PFRON; zgoda niezaznaczona; kal. Podstawowy system_1_8:15_N (19.10; wcześniej Podstawowy system_1_8:16).
 Plan 02.11.2026: 8:00</t>
   </si>
   <si>
     <t>Błąd – stopień z orzeczenia ZUS też się liczy</t>
   </si>
   <si>
+    <t>Powtórka 19.10.2026 (kal. 8:15_N): komunikat jak oczekiwany, razem z błędem normy dobowej (7:00).</t>
+  </si>
+  <si>
     <t>Zmiana stopnia w miesiącu – dzień przed zmianą</t>
   </si>
   <si>
-    <t>NP8: orzeczenia PFRON – umiarkowany 01.01–15.11.2026, lekki 16.11–31.12.2026; zgoda niezaznaczona; kal. Podstawowy system_1_8:16.
+    <t>NP8: orzeczenia PFRON – umiarkowany 01.01–15.11.2026, lekki 16.11–31.12.2026; zgoda niezaznaczona; kal. Podstawowy system_1_8:15_N (19.10; wcześniej Podstawowy system_1_8:16).
 Plan 13.11.2026: 8:00</t>
   </si>
   <si>
@@ -807,7 +813,7 @@
     <t>Dla dnia (13.11.2026) zaplanowano czas (8:00), a pracownik bez zgody na pracę 8h (stopień niepełnosprawności Umiarkowany) może pracować maksymalnie 7:00 - (pracownik)</t>
   </si>
   <si>
-    <t>Test 15.10.2026: negatywny (brak komunikatu - stopień czytany z historii pracownika, StopienNiepelnosp/PFRON, które w enova 2610 zwracają jedno orzeczenie z zapisu historii). Poprawka 19.10.2026: stopień z metody enova Pracownik.StopienNiepelnosprawnosciNaDzien (orzeczenia PFRON/ZUS obowiązujące w danym dniu). Powtórka 19.10.2026: komunikat jak oczekiwany - pozytywny. (Niedobór normy okresu - skutek danych testowych.)</t>
+    <t>Test 15.10.2026: negatywny (brak komunikatu - stopień czytany z historii pracownika, które w enova 2610 zwracają jedno orzeczenie z zapisu historii). Poprawka 19.10.2026: stopień z metody enova Pracownik.StopienNiepelnosprawnosciNaDzien. Powtórka 19.10.2026 (kal. 8:15_N): komunikat jak oczekiwany, razem z błędem normy dobowej (7:00).</t>
   </si>
   <si>
     <t>Zmiana stopnia w miesiącu – dzień po zmianie</t>
@@ -820,7 +826,7 @@
     <t>Brak błędu – od 16.11 stopień lekki</t>
   </si>
   <si>
-    <t>Niedobór normy okresu - skutek drugiego dnia testowego z planem 6:00. Powtórka 19.10.2026 po poprawce: brak błędu tego weryfikatora - pozytywny.</t>
+    <t>Powtórka 19.10.2026 (kal. 8:15_N): brak błędu tego weryfikatora. Odzywa się norma dobowa (7:00), bo w danych testowych pracownik ma kalendarz 8:15_N przez cały okres; w praktyce po zmianie stopnia na lekki kalendarz zmienia się aktualizacją historii.</t>
   </si>
   <si>
     <t>10</t>
@@ -829,14 +835,17 @@
     <t>System równoważny</t>
   </si>
   <si>
-    <t>NP9: orzeczenie PFRON – umiarkowany; zgoda niezaznaczona; kal. 3 miesięczny (równoważny).
+    <t>NP9: orzeczenie PFRON – umiarkowany; zgoda niezaznaczona; kal. Równoważny system_3_8:15_N (19.10; wcześniej 3 miesięczny).
 Plan 02.11.2026: 8:00</t>
   </si>
   <si>
     <t>Błąd – weryfikator podpięty także do kalendarza 3 miesięczny</t>
   </si>
   <si>
-    <t>Uwaga z testu (poza zakresem tego weryfikatora): weryfikator normy okresu rozliczeniowego liczy normę ogólną (np. 160:00 w 11.2026) także dla osób ze stopniem umiarkowanym/znacznym bez zgody, którym przysługuje norma 7h/dobę i 35h/tydzień. Dla takiej osoby oba weryfikatory wykluczają się: niedobór normy okresu podpowiada wydłużenie dnia do 8:00, a ten weryfikator blokuje więcej niż 7:00.</t>
+    <t>Powtórka 19.10.2026 (kal. Równoważny system_3_8:15_N): komunikat jak oczekiwany. Norma okresu 448:00 (IX-XI, 7h/dzień); podpowiedź normy okresu proponuje wydłużenie dnia o 4:00 (do 12h w systemie równoważnym), czego ten weryfikator nie przepuści - znana niespójność podpowiedzi, niezmieniana.</t>
+  </si>
+  <si>
+    <t>Uwaga z testu (poza zakresem tego weryfikatora): weryfikator normy okresu rozliczeniowego liczy normę ogólną (np. 160:00 w 11.2026) także dla osób ze stopniem umiarkowanym/znacznym bez zgody, którym przysługuje norma 7h/dobę i 35h/tydzień. Dla takiej osoby oba weryfikatory wykluczają się: niedobór normy okresu podpowiada wydłużenie dnia do 8:00, a ten weryfikator blokuje więcej niż 7:00. Decyzja 19.10.2026: bez zmian w kodzie - osoby bez zgody mają kalendarz klienta 8:15_N (norma 7:00), na którym norma okresu liczy 7h/dzień i konflikt nie występuje (potwierdzone w powtórce).</t>
   </si>
 </sst>
 </file>
@@ -2853,7 +2862,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" ht="75">
+    <row r="5" ht="120">
       <c r="A5" s="6" t="s">
         <v>26</v>
       </c>
@@ -2876,7 +2885,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="6" ht="60">
+    <row r="6" ht="120">
       <c r="A6" s="6" t="s">
         <v>32</v>
       </c>
@@ -2899,7 +2908,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="7" ht="75">
+    <row r="7" ht="120">
       <c r="A7" s="6" t="s">
         <v>36</v>
       </c>
@@ -2922,7 +2931,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="8" ht="60">
+    <row r="8" ht="90">
       <c r="A8" s="6" t="s">
         <v>39</v>
       </c>
@@ -2945,7 +2954,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="9" ht="60">
+    <row r="9" ht="75">
       <c r="A9" s="6" t="s">
         <v>44</v>
       </c>
@@ -2965,18 +2974,18 @@
         <v>31</v>
       </c>
       <c r="G9" s="10" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="10" ht="75">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="10" ht="90">
       <c r="A10" s="6" t="s">
         <v>47</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D10" s="8" t="s">
         <v>29</v>
@@ -2988,21 +2997,21 @@
         <v>31</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="11" ht="90">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="11" ht="105">
       <c r="A11" s="6" t="s">
         <v>51</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="E11" s="9" t="s">
         <v>219</v>
@@ -3011,44 +3020,44 @@
         <v>31</v>
       </c>
       <c r="G11" s="10" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="12" ht="270">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="12" ht="210">
       <c r="A12" s="6" t="s">
         <v>55</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="F12" s="12" t="s">
         <v>31</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="13" ht="90">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="13" ht="150">
       <c r="A13" s="6" t="s">
         <v>58</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="E13" s="9" t="s">
         <v>30</v>
@@ -3057,21 +3066,21 @@
         <v>31</v>
       </c>
       <c r="G13" s="10" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
     </row>
     <row r="14" ht="75" customHeight="1">
       <c r="A14" s="6" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="E14" s="9" t="s">
         <v>219</v>
@@ -3080,12 +3089,12 @@
         <v>31</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>2</v>
+        <v>254</v>
       </c>
     </row>
     <row r="16" ht="45" customHeight="1">
       <c r="B16" s="13" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Weryfikatory zgod niepelnosprawnych 2070-2072: test live 14/14 (baza Al), arkusz 'Zgody nadgodziny i noc', XML dni pracy NP1-NP6
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018SWEtN1iMr88RMmUUHSCbE
</commit_message>
<xml_diff>
--- a/Weryfikatory czasu pracy/Scenariusze testowe weryfikatorow czasu pracy.xlsx
+++ b/Weryfikatory czasu pracy/Scenariusze testowe weryfikatorow czasu pracy.xlsx
@@ -8,7 +8,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" firstSheet="2" activeTab="7"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" firstSheet="2" activeTab="8"/>
   </bookViews>
   <sheets>
     <sheet name="Informacje" sheetId="1" r:id="rId1"/>
@@ -19,6 +19,7 @@
     <sheet name="Praca w normie wg planu" sheetId="9" r:id="rId6"/>
     <sheet name="Magazyn nadgodzin - umowy" sheetId="11" r:id="rId7"/>
     <sheet name="Brak zgody 8h" sheetId="12" r:id="rId8"/>
+    <sheet name="Zgody nadgodziny i noc" sheetId="13" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Okres zatrudnienia'!$A$4:$G$13</definedName>
@@ -28,6 +29,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Praca w normie wg planu'!$A$4:$G$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Magazyn nadgodzin - umowy'!$A$4:$G$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Brak zgody 8h'!$A$4:$G$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Zgody nadgodziny i noc'!$A$4:$G$14</definedName>
   </definedNames>
   <calcPr/>
 </workbook>
@@ -847,12 +849,190 @@
   <si>
     <t>Uwaga z testu (poza zakresem tego weryfikatora): weryfikator normy okresu rozliczeniowego liczy normę ogólną (np. 160:00 w 11.2026) także dla osób ze stopniem umiarkowanym/znacznym bez zgody, którym przysługuje norma 7h/dobę i 35h/tydzień. Dla takiej osoby oba weryfikatory wykluczają się: niedobór normy okresu podpowiada wydłużenie dnia do 8:00, a ten weryfikator blokuje więcej niż 7:00. Decyzja 19.10.2026: bez zmian w kodzie - osoby bez zgody mają kalendarz klienta 8:15_N (norma 7:00), na którym norma okresu liczy 7h/dzień i konflikt nie występuje (potwierdzone w powtórce).</t>
   </si>
+  <si>
+    <t>Weryfikatory: Brak zgody na nadgodziny / Brak zgody na pracę w nocy</t>
+  </si>
+  <si>
+    <t>Trzy weryfikatory zgód osoby z niepełnosprawnością (każdy stopień - orzeczenie PFRON albo ZUS obowiązujące w dniu), zgody czytane z etatu w zapisie historii obowiązującym w dniu: „A1_Brak zgody na pracę w nocy (plan)” (Dzień planu, Błąd) - praca zaplanowana w porze nocnej bez zgody na pracę w porze nocnej; „A1_Brak zgody na pracę w nocy (czas)” (Dzień pracy, Ostrzeżenie) - praca w porze nocnej wpisana w czasie pracy; „A1_Brak zgody na nadgodziny” (Dzień pracy, Ostrzeżenie) - czas pracy dnia ponad większą z wartości: plan dnia i norma dobowa z etatu (w dniu wolnym wg planu - każda praca). Pora nocna z kalendarza etatu (w kalendarzach klienta _N: 22:00-6:00). Test 19.10.2026 na bazie Al, pracownicy NP1-NP6 (kalendarze _N; NP4 ma zgody na nadgodziny i pracę w nocy); dni pracy: ImportyXML/Weryfikatory zgod niepelnosprawnych - dni pracy.xml. Zmiany wpisywane w programie i wycofywane bez zapisu.</t>
+  </si>
+  <si>
+    <t>Plan w nocy - umiarkowany, bez zgody</t>
+  </si>
+  <si>
+    <t>NP1: orzeczenie PFRON umiarkowany; zgoda na pracę w nocy niezaznaczona; kal. Podstawowy system_1_8:15_N (norma 7:00, pora nocna 22:00-6:00).
+Plan 02.11.2026: 22:00, 6:00</t>
+  </si>
+  <si>
+    <t>Błąd - zapis zablokowany</t>
+  </si>
+  <si>
+    <t>Dla dnia (2.11.2026) zaplanowano pracę w porze nocnej (6:00), a pracownik z niepełnosprawnością (stopień Umiarkowany) nie ma na etacie zgody na pracę w porze nocnej - (pracownik)</t>
+  </si>
+  <si>
+    <t>Dodatkowo niedobór normy okresu - skutek danych testowych (1 dzień planu).</t>
+  </si>
+  <si>
+    <t>Plan tuż przed porą nocną (granica)</t>
+  </si>
+  <si>
+    <t>NP1: jak wyżej.
+Plan 02.11.2026: 16:00-22:00</t>
+  </si>
+  <si>
+    <t>Praca kończy się z początkiem pory nocnej - nie jest liczona.</t>
+  </si>
+  <si>
+    <t>Plan częściowo w porze nocnej (wieczór)</t>
+  </si>
+  <si>
+    <t>NP1: jak wyżej.
+Plan 02.11.2026: 16:30-22:30</t>
+  </si>
+  <si>
+    <t>…zaplanowano pracę w porze nocnej (0:30)…</t>
+  </si>
+  <si>
+    <t>Plan częściowo w porze nocnej (rano)</t>
+  </si>
+  <si>
+    <t>NP1: jak wyżej.
+Plan 02.11.2026: 5:00-11:00</t>
+  </si>
+  <si>
+    <t>…zaplanowano pracę w porze nocnej (1:00)…</t>
+  </si>
+  <si>
+    <t>Plan w nocy - stopień lekki, bez zgody</t>
+  </si>
+  <si>
+    <t>NP5: orzeczenie PFRON lekki; zgody niezaznaczone; kal. Podstawowy system_1_8:16_N (norma 8:00, pora nocna 22:00-6:00).
+Plan 02.11.2026: 22:00, 8:00</t>
+  </si>
+  <si>
+    <t>Błąd - weryfikator obejmuje każdy stopień</t>
+  </si>
+  <si>
+    <t>…zaplanowano pracę w porze nocnej (8:00), a pracownik z niepełnosprawnością (stopień Lekki)…</t>
+  </si>
+  <si>
+    <t>Plan w nocy - bez orzeczenia</t>
+  </si>
+  <si>
+    <t>NP6: brak orzeczeń; kal. Podstawowy system_1_8:16_N (norma 8:00, pora nocna 22:00-6:00).
+Plan 02.11.2026: 22:00, 8:00</t>
+  </si>
+  <si>
+    <t>Plan w nocy - ze zgodą</t>
+  </si>
+  <si>
+    <t>NP4: orzeczenie PFRON umiarkowany; zaznaczone zgody na pracę 8h, w nadgodzinach i w porze nocnej; kal. Podstawowy system_1_8:16_N (norma 8:00, pora nocna 22:00-6:00).
+Plan 02.11.2026: 22:00, 8:00</t>
+  </si>
+  <si>
+    <t>Czas pracy w nocy - bez zgody</t>
+  </si>
+  <si>
+    <t>NP1: jak w scen. 1. Dzień pracy 02.11.2026: Praca w normie 22:00, 6:00</t>
+  </si>
+  <si>
+    <t>Ostrzeżenie - zapis możliwy</t>
+  </si>
+  <si>
+    <t>Dla dnia (2.11.2026) wpisano pracę w porze nocnej (6:00), a pracownik z niepełnosprawnością (stopień Umiarkowany) nie ma na etacie zgody na pracę w porze nocnej - (pracownik)</t>
+  </si>
+  <si>
+    <t>Komunikat typu ostrzeżenie (nie błąd).</t>
+  </si>
+  <si>
+    <t>Czas pracy równy normie dobowej (granica)</t>
+  </si>
+  <si>
+    <t>NP2: orzeczenie PFRON umiarkowany; zgody niezaznaczone; kal. Podstawowy system_1_8:15_N (norma 7:00, pora nocna 22:00-6:00); plan 02.11: 6:00.
+Dzień pracy 02.11.2026: Praca w normie 7:00-13:00 + Praca poza normą 13:00-14:00 (razem 7:00)</t>
+  </si>
+  <si>
+    <t>Brak ostrzeżenia</t>
+  </si>
+  <si>
+    <t>brak</t>
+  </si>
+  <si>
+    <t>Limit dnia = większa z wartości: plan (6:00) i norma dobowa (7:00).</t>
+  </si>
+  <si>
+    <t>Nadgodziny - bez zgody</t>
+  </si>
+  <si>
+    <t>NP2: jak wyżej.
+Dzień pracy 02.11.2026: Praca w normie 6:00 + Praca poza normą 2:00 (razem 8:00)</t>
+  </si>
+  <si>
+    <t>Dla dnia (2.11.2026) wpisano pracę w godzinach nadliczbowych (1:00; czas pracy 8:00, limit dnia 7:00), a pracownik z niepełnosprawnością (stopień Umiarkowany) nie ma na etacie zgody na pracę w nadgodzinach - (pracownik)</t>
+  </si>
+  <si>
+    <t>11</t>
+  </si>
+  <si>
+    <t>Praca w dniu wolnym - bez zgody</t>
+  </si>
+  <si>
+    <t>NP3: orzeczenie PFRON znaczny; zgody niezaznaczone; kal. Podstawowy system_1_8:15_N (norma 7:00, pora nocna 22:00-6:00).
+Dzień pracy 07.11.2026 (sobota, wolny wg planu): Praca poza normą 8:00-12:00</t>
+  </si>
+  <si>
+    <t>Ostrzeżenie - każda praca w dniu wolnym</t>
+  </si>
+  <si>
+    <t>…wpisano pracę w godzinach nadliczbowych (4:00; czas pracy 4:00, limit dnia 0:00)… (stopień Znaczny)…</t>
+  </si>
+  <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>Nadgodziny - stopień lekki</t>
+  </si>
+  <si>
+    <t>NP5: jak w scen. 5; plan 02.11: 8:00.
+Dzień pracy 02.11.2026: Praca w normie 8:00 + Praca poza normą 1:00</t>
+  </si>
+  <si>
+    <t>Ostrzeżenie</t>
+  </si>
+  <si>
+    <t>…(1:00; czas pracy 9:00, limit dnia 8:00)… (stopień Lekki)…</t>
+  </si>
+  <si>
+    <t>13</t>
+  </si>
+  <si>
+    <t>Nadgodziny i noc - ze zgodami</t>
+  </si>
+  <si>
+    <t>NP4: jak w scen. 7.
+Dzień pracy 02.11.2026: Praca w normie 21:00-5:00 + Praca poza normą 5:00-6:00</t>
+  </si>
+  <si>
+    <t>Brak ostrzeżeń</t>
+  </si>
+  <si>
+    <t>14</t>
+  </si>
+  <si>
+    <t>Nadgodziny i noc - bez orzeczenia</t>
+  </si>
+  <si>
+    <t>NP6: jak w scen. 6.
+Dzień pracy 02.11.2026: jak w scen. 13</t>
+  </si>
+  <si>
+    <t>Uwagi: 1) Weryfikatory dnia pracy nie blokują zapisu (ostrzeżenie); w teście sprawdzono typ komunikatu, dni nie były zapisywane. 2) Nadwyżkę wpisano jako „Praca poza normą”, bo „Praca w normie” ponad plan blokuje weryfikator „A1_Praca w normie nie ponad plan”. 3) Na kalendarzach 8:15_N przy planie &gt; 7:00 odzywa się też „A1_Norma dobowa”.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -896,8 +1076,14 @@
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C5700"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -924,6 +1110,11 @@
         <fgColor rgb="FFFFC7CE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border/>
@@ -945,7 +1136,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -976,6 +1167,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3103,4 +3297,385 @@
     <mergeCell ref="B16:G16"/>
   </mergeCells>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="5.7109375" customWidth="1"/>
+    <col min="2" max="2" width="34.710938" customWidth="1"/>
+    <col min="3" max="3" width="40.710938" customWidth="1"/>
+    <col min="4" max="4" width="44.710938" customWidth="1"/>
+    <col min="5" max="5" width="46.710938" customWidth="1"/>
+    <col min="6" max="6" width="18.710938" customWidth="1"/>
+    <col min="7" max="7" width="26.710938" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="17.25">
+      <c r="A1" s="3" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" ht="75">
+      <c r="A5" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>258</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>259</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>260</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>261</v>
+      </c>
+      <c r="F5" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="G5" s="10" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="6" ht="45">
+      <c r="A6" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>263</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>264</v>
+      </c>
+      <c r="D6" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="E6" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="F6" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="G6" s="10" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="7" ht="30">
+      <c r="A7" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>266</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>267</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>260</v>
+      </c>
+      <c r="E7" s="9" t="s">
+        <v>268</v>
+      </c>
+      <c r="F7" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="G7" s="10" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" ht="30">
+      <c r="A8" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>269</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>270</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>260</v>
+      </c>
+      <c r="E8" s="9" t="s">
+        <v>271</v>
+      </c>
+      <c r="F8" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="G8" s="10" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9" ht="75">
+      <c r="A9" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>272</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>273</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>274</v>
+      </c>
+      <c r="E9" s="9" t="s">
+        <v>275</v>
+      </c>
+      <c r="F9" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="G9" s="10" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" ht="60">
+      <c r="A10" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>277</v>
+      </c>
+      <c r="D10" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="E10" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="F10" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="G10" s="10" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" ht="90">
+      <c r="A11" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>278</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>279</v>
+      </c>
+      <c r="D11" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="E11" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="F11" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="G11" s="10" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" ht="48">
+      <c r="A12" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="D12" s="14" t="s">
+        <v>282</v>
+      </c>
+      <c r="E12" s="9" t="s">
+        <v>283</v>
+      </c>
+      <c r="F12" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="G12" s="10" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="13" ht="105">
+      <c r="A13" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>285</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>286</v>
+      </c>
+      <c r="D13" s="11" t="s">
+        <v>287</v>
+      </c>
+      <c r="E13" s="9" t="s">
+        <v>288</v>
+      </c>
+      <c r="F13" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="G13" s="10" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="14" ht="75" customHeight="1">
+      <c r="A14" s="6" t="s">
+        <v>250</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>290</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>291</v>
+      </c>
+      <c r="D14" s="14" t="s">
+        <v>282</v>
+      </c>
+      <c r="E14" s="9" t="s">
+        <v>292</v>
+      </c>
+      <c r="F14" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="G14" s="10" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" ht="90">
+      <c r="A15" s="6" t="s">
+        <v>293</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>294</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>295</v>
+      </c>
+      <c r="D15" s="14" t="s">
+        <v>296</v>
+      </c>
+      <c r="E15" s="9" t="s">
+        <v>297</v>
+      </c>
+      <c r="F15" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="G15" s="10" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16" ht="45" customHeight="1">
+      <c r="A16" s="6" t="s">
+        <v>298</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>299</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>300</v>
+      </c>
+      <c r="D16" s="14" t="s">
+        <v>301</v>
+      </c>
+      <c r="E16" s="9" t="s">
+        <v>302</v>
+      </c>
+      <c r="F16" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="G16" s="10" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17" ht="45">
+      <c r="A17" s="6" t="s">
+        <v>303</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>304</v>
+      </c>
+      <c r="C17" s="7" t="s">
+        <v>305</v>
+      </c>
+      <c r="D17" s="11" t="s">
+        <v>306</v>
+      </c>
+      <c r="E17" s="9" t="s">
+        <v>288</v>
+      </c>
+      <c r="F17" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="G17" s="10" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" ht="30">
+      <c r="A18" s="6" t="s">
+        <v>307</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>308</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>309</v>
+      </c>
+      <c r="D18" s="11" t="s">
+        <v>306</v>
+      </c>
+      <c r="E18" s="9" t="s">
+        <v>288</v>
+      </c>
+      <c r="F18" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="G18" s="10" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="13" t="s">
+        <v>310</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:G14"/>
+  <mergeCells count="1">
+    <mergeCell ref="B20:G20"/>
+  </mergeCells>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Weryfikatory 3070/3071 (Al): test live 19.10.2026 - wszystkie scenariusze pozytywne; arkusz 'Norma tygodniowa 35-40h', sekcje w Instrukcja_Weryfikatory.docx (opis, konfiguracja, komunikaty, scenariusze); decyzja: Blad przy kalendarzu podstawowym
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JXMhWf2ag4PGnQHt13HR9W
</commit_message>
<xml_diff>
--- a/Weryfikatory czasu pracy/Scenariusze testowe weryfikatorow czasu pracy.xlsx
+++ b/Weryfikatory czasu pracy/Scenariusze testowe weryfikatorow czasu pracy.xlsx
@@ -8,7 +8,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" firstSheet="2" activeTab="8"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" firstSheet="2" activeTab="9"/>
   </bookViews>
   <sheets>
     <sheet name="Informacje" sheetId="1" r:id="rId1"/>
@@ -20,6 +20,7 @@
     <sheet name="Magazyn nadgodzin - umowy" sheetId="11" r:id="rId7"/>
     <sheet name="Brak zgody 8h" sheetId="12" r:id="rId8"/>
     <sheet name="Zgody nadgodziny i noc" sheetId="13" r:id="rId9"/>
+    <sheet name="Norma tygodniowa 35-40h" sheetId="14" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Okres zatrudnienia'!$A$4:$G$13</definedName>
@@ -30,6 +31,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Magazyn nadgodzin - umowy'!$A$4:$G$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Brak zgody 8h'!$A$4:$G$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Zgody nadgodziny i noc'!$A$4:$G$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Norma tygodniowa 35-40h'!$A$4:$G$14</definedName>
   </definedNames>
   <calcPr/>
 </workbook>
@@ -1026,6 +1028,163 @@
   </si>
   <si>
     <t>Uwagi: 1) Weryfikatory dnia pracy nie blokują zapisu (ostrzeżenie); w teście sprawdzono typ komunikatu, dni nie były zapisywane. 2) Nadwyżkę wpisano jako „Praca poza normą”, bo „Praca w normie” ponad plan blokuje weryfikator „A1_Praca w normie nie ponad plan”. 3) Na kalendarzach 8:15_N przy planie &gt; 7:00 odzywa się też „A1_Norma dobowa”.</t>
+  </si>
+  <si>
+    <t>Weryfikatory: A1_Norma tygodniowa niepełnosprawnych / A1_Doba niepełnosprawnych (równoważny)</t>
+  </si>
+  <si>
+    <t>„A1_Norma tygodniowa niepełnosprawnych” (Plan pracy, Błąd): osoba z niepełnosprawnością - umiarkowany/znaczny bez zgody na pracę 8h: 35h/tydz. (7h/doba), lekki albo zgoda na pracę 8h: 40h/tydz. (8h/doba). Tygodnie = 7 kolejnych dni od pierwszego dnia okresu rozliczeniowego. Kalendarz podstawowy: każdy tydzień sztywno ≤ W oraz okres ≤ wymiar; kalendarz równoważny: okres ≤ wymiar (art. 130 KP z normą 7h/8h: W × pełne tygodnie + d × dni pon-pt niepełnego tygodnia - d × święta poza niedzielą). „A1_Doba niepełnosprawnych (równoważny)” (Dzień planu, Ostrzeżenie): dzień planu dłuższy niż 7h/8h na kalendarzu równoważnym. Test 19.10.2026 na bazie Al, pracownicy NP1-NP9; plan: ImportyXML/Weryfikator norma tygodniowa niepelnosprawnych - plan.xml. Zmiany wpisywane w programie i wycofywane bez zapisu.</t>
+  </si>
+  <si>
+    <t>Podstawowy, 35h - każdy tydzień 35h</t>
+  </si>
+  <si>
+    <t>NP1: PFRON umiarkowany, bez zgody 8h; kal. Podstawowy system_1_8:15_N (okres 1 mies.).
+Plan X.2026 pon-pt 7:00 (1.10: 6:00 → 7:00), razem 154:00</t>
+  </si>
+  <si>
+    <t>brak komunikatu</t>
+  </si>
+  <si>
+    <t>Podstawowy, 35h - tydzień 36h, okres ≤ wymiar</t>
+  </si>
+  <si>
+    <t>NP2: jak NP1.
+Tydzień 8-14.10: czw-śr 7:00, sob 10.10 1:00, pt 9.10 6:00 → 7:00 (36:00); 1.10 6:00 - okres 154:00</t>
+  </si>
+  <si>
+    <t>Przekroczono tygodniową normę (35:00) osoby z niepełnosprawnością w tygodniu (8...14.10.2026) okresu rozliczeniowego - zaplanowano (36:00) - (pracownik)</t>
+  </si>
+  <si>
+    <t>Dodatkowo „za mało dni wolnych” (sobota pracująca).</t>
+  </si>
+  <si>
+    <t>Podstawowy, okres 3-mies. - tygodnie przez granicę miesięcy</t>
+  </si>
+  <si>
+    <t>NP3: PFRON znaczny; kal. testowy TEST Podstawowy_3_8:15_N (okres IX-XI od 1.09 - wtorek).
+Tydzień 29.09-5.10 (wt-pn): sob 3.10 1:00, pt 2.10 6:00 → 7:00</t>
+  </si>
+  <si>
+    <t>Przekroczono tygodniową normę (35:00) … w tygodniu (29.09.2026...5.10.2026) … zaplanowano (36:00)</t>
+  </si>
+  <si>
+    <t>Tydzień nie zaczyna się od nowa 1.10.</t>
+  </si>
+  <si>
+    <t>Okres od czwartku - tydzień czw-śr, nie pon-nd</t>
+  </si>
+  <si>
+    <t>NP7: ZUS (umiarkowany); kal. Podstawowy system_1_8:15_N (okres 1 mies.).
+sob 17.10 6:00 → 7:00, pon 19.10 wolny: tydzień 15-21.10 (czw-śr) = 35:00, pon-nd 12-18.10 = 42:00</t>
+  </si>
+  <si>
+    <t>Równoważny, 35h - tydzień 42h, okres = wymiar</t>
+  </si>
+  <si>
+    <t>NP9: PFRON umiarkowany; kal. Równoważny system_3_8:15_N (IX-XI).
+Tydzień 1-7.09 = 42:00 (sob 5.09 7:00); 9.09 6:00 → 5:00 - okres 447:00 (wymiar 448:00)</t>
+  </si>
+  <si>
+    <t>Brak błędu 3070</t>
+  </si>
+  <si>
+    <t>brak komunikatu 3070</t>
+  </si>
+  <si>
+    <t>Odzywa się niedobór normy okresu (37) i dni wolnych (1036).</t>
+  </si>
+  <si>
+    <t>Równoważny, 35h - okres ponad wymiar</t>
+  </si>
+  <si>
+    <t>NP9: jak wyżej; 9.09 → 7:00 - okres 449:00</t>
+  </si>
+  <si>
+    <t>Zaplanowany czas pracy (449:00) przekracza wymiar (448:00) osoby z niepełnosprawnością o (1:00) w okresie rozliczeniowym (1.09.2026...30.11.2026) - (pracownik)</t>
+  </si>
+  <si>
+    <t>Święto w dniu roboczym pomniejsza wymiar</t>
+  </si>
+  <si>
+    <t>NP9: okres IX-XI = 13 pełnych tygodni; 11.11.2026 (środa) święto</t>
+  </si>
+  <si>
+    <t>Wymiar 13 × 35 - 7 = 448:00</t>
+  </si>
+  <si>
+    <t>wymiar (448:00) w komunikacie scen. 6</t>
+  </si>
+  <si>
+    <t>Bez święta wymiar wyniósłby 455:00.</t>
+  </si>
+  <si>
+    <t>Stopień lekki - normy 40/8</t>
+  </si>
+  <si>
+    <t>NP5: PFRON lekki; kal. Podstawowy system_1_8:16_N.
+Tydzień 8-14.10: sob 10.10 1:00, pt 9.10 7:00 → 8:00 (41:00)</t>
+  </si>
+  <si>
+    <t>Przekroczono tygodniową normę (40:00) … w tygodniu (8...14.10.2026) … zaplanowano (41:00)</t>
+  </si>
+  <si>
+    <t>8a</t>
+  </si>
+  <si>
+    <t>Zgoda na pracę 8h - normy 40/8, równoważny</t>
+  </si>
+  <si>
+    <t>NP4: PFRON umiarkowany ze zgodą 8h; kal. Równoważny system_1_8:16_N.
+2.10 8:00 → 9:00 - okres 177:00</t>
+  </si>
+  <si>
+    <t>Błąd + Ostrzeżenie</t>
+  </si>
+  <si>
+    <t>Błąd: Zaplanowany czas pracy (177:00) przekracza wymiar (176:00) … o (1:00) …; Ostrzeżenie: Dla dnia (2.10.2026) zaplanowano czas (9:00) dłuższy niż norma dobowa (8:00) osoby z niepełnosprawnością w równoważnym systemie czasu pracy</t>
+  </si>
+  <si>
+    <t>Ostrzeżenie = definicja „A1_Doba niepełnosprawnych (równoważny)”.</t>
+  </si>
+  <si>
+    <t>Bez orzeczenia - brak weryfikacji</t>
+  </si>
+  <si>
+    <t>NP6: brak orzeczeń; kal. Podstawowy system_1_8:16_N.
+Tydzień 8-14.10: sob 10.10 8:00, pt 9.10 7:00 → 8:00 (48:00)</t>
+  </si>
+  <si>
+    <t>Odzywają się ogólne: limit godzin okresu (37) i dni wolne (1036).</t>
+  </si>
+  <si>
+    <t>10a</t>
+  </si>
+  <si>
+    <t>Zmiana orzeczenia w okresie - po zmianie 40h</t>
+  </si>
+  <si>
+    <t>NP8: PFRON umiarkowany do 15.11, lekki od 16.11; kal. Podstawowy system_1_8:15_N (okres 1 mies.).
+Tydzień 15-21.11 = 40:00 (16-20.11 po 8:00); 30.11 7:00 → 8:00 - okres 151:00 = wymiar (35+28+40+40+8)</t>
+  </si>
+  <si>
+    <t>Odzywa się „A1_Norma dobowa” i limit okresu (37) - kalendarz 7h przy stopniu lekkim (dane testowe).</t>
+  </si>
+  <si>
+    <t>10b</t>
+  </si>
+  <si>
+    <t>Zmiana orzeczenia w okresie - przed zmianą 35h</t>
+  </si>
+  <si>
+    <t>NP8: jak wyżej.
+Tydzień 1-7.11: sob 7.11 1:00, pt 6.11 6:00 → 7:00 (36:00)</t>
+  </si>
+  <si>
+    <t>Przekroczono tygodniową normę (35:00) … w tygodniu (1...7.11.2026) … zaplanowano (36:00)</t>
+  </si>
+  <si>
+    <t>Uwagi: 1) Kalendarze klienta _N nie generują planu z definicji kalendarza - w danych testowych każdy dzień roboczy ma jawny plan. 2) Poziom Błąd/Ostrzeżenie ustawia się na zakładce Weryfikatory kalendarza (podpięcie), bez zmian w kodzie. 3) Weryfikator nie uruchamia się przy zmianie kalendarza na etacie ani orzeczenia - dopiero przy edycji planu.</t>
   </si>
 </sst>
 </file>
@@ -1579,6 +1738,341 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="5.7109375" customWidth="1"/>
+    <col min="2" max="2" width="34.710938" customWidth="1"/>
+    <col min="3" max="3" width="40.710938" customWidth="1"/>
+    <col min="4" max="4" width="44.710938" customWidth="1"/>
+    <col min="5" max="5" width="46.710938" customWidth="1"/>
+    <col min="6" max="6" width="18.710938" customWidth="1"/>
+    <col min="7" max="7" width="26.710938" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="17.25">
+      <c r="A1" s="3" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" ht="75">
+      <c r="A5" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>313</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>314</v>
+      </c>
+      <c r="D5" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>315</v>
+      </c>
+      <c r="F5" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="G5" s="10" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" ht="60">
+      <c r="A6" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>316</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>317</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>260</v>
+      </c>
+      <c r="E6" s="9" t="s">
+        <v>318</v>
+      </c>
+      <c r="F6" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="G6" s="10" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="7" ht="75">
+      <c r="A7" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>320</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>321</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>260</v>
+      </c>
+      <c r="E7" s="9" t="s">
+        <v>322</v>
+      </c>
+      <c r="F7" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="G7" s="10" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="8" ht="75">
+      <c r="A8" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>324</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>325</v>
+      </c>
+      <c r="D8" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="E8" s="9" t="s">
+        <v>315</v>
+      </c>
+      <c r="F8" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="G8" s="10" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9" ht="60">
+      <c r="A9" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>326</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>327</v>
+      </c>
+      <c r="D9" s="11" t="s">
+        <v>328</v>
+      </c>
+      <c r="E9" s="9" t="s">
+        <v>329</v>
+      </c>
+      <c r="F9" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="G9" s="10" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="10" ht="36">
+      <c r="A10" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>331</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>332</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>260</v>
+      </c>
+      <c r="E10" s="9" t="s">
+        <v>333</v>
+      </c>
+      <c r="F10" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="G10" s="10" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" ht="30">
+      <c r="A11" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>334</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>335</v>
+      </c>
+      <c r="D11" s="11" t="s">
+        <v>336</v>
+      </c>
+      <c r="E11" s="9" t="s">
+        <v>337</v>
+      </c>
+      <c r="F11" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="G11" s="10" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="12" ht="60">
+      <c r="A12" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>339</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>340</v>
+      </c>
+      <c r="D12" s="8" t="s">
+        <v>260</v>
+      </c>
+      <c r="E12" s="9" t="s">
+        <v>341</v>
+      </c>
+      <c r="F12" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="G12" s="10" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" ht="60">
+      <c r="A13" s="6" t="s">
+        <v>342</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>343</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>344</v>
+      </c>
+      <c r="D13" s="8" t="s">
+        <v>345</v>
+      </c>
+      <c r="E13" s="9" t="s">
+        <v>346</v>
+      </c>
+      <c r="F13" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="G13" s="10" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="14" ht="75" customHeight="1">
+      <c r="A14" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>348</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>349</v>
+      </c>
+      <c r="D14" s="11" t="s">
+        <v>328</v>
+      </c>
+      <c r="E14" s="9" t="s">
+        <v>329</v>
+      </c>
+      <c r="F14" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="G14" s="10" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="15" ht="90">
+      <c r="A15" s="6" t="s">
+        <v>351</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>352</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>353</v>
+      </c>
+      <c r="D15" s="11" t="s">
+        <v>328</v>
+      </c>
+      <c r="E15" s="9" t="s">
+        <v>329</v>
+      </c>
+      <c r="F15" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="G15" s="10" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="16" ht="45" customHeight="1">
+      <c r="A16" s="6" t="s">
+        <v>355</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>356</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>357</v>
+      </c>
+      <c r="D16" s="8" t="s">
+        <v>260</v>
+      </c>
+      <c r="E16" s="9" t="s">
+        <v>358</v>
+      </c>
+      <c r="F16" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="G16" s="10" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="13" t="s">
+        <v>359</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:G14"/>
+  <mergeCells count="1">
+    <mergeCell ref="B18:G18"/>
+  </mergeCells>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetFormatPr defaultRowHeight="15"/>

</xml_diff>

<commit_message>
Weryfikatory niepelnosprawnych: zgodnosc z enova 2512.10.12 klienta - stopien z zapisu historii (A1StopienNiepelnosprawnosciNaDzien: StopienNiepelnosp/PFRON, OkresExt) zamiast Pracownik.StopienNiepelnosprawnosciNaDzien z 2610; kompilacja 2512.10.12 0/0, Al 2610 0 bledow; docx/xlsx: zrodlo stopnia
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016Sk1XN31K2XRRWhL9D8Qkd
</commit_message>
<xml_diff>
--- a/Weryfikatory czasu pracy/Scenariusze testowe weryfikatorow czasu pracy.xlsx
+++ b/Weryfikatory czasu pracy/Scenariusze testowe weryfikatorow czasu pracy.xlsx
@@ -722,7 +722,7 @@
     <t>Weryfikator: Brak zgody na pracę 8h</t>
   </si>
   <si>
-    <t>Weryfikator dnia planu pracy (Dzień planu), definicja „A1_Brak zgody na pracę 8h”. Pracownik ze stopniem umiarkowanym lub znacznym (orzeczenie PFRON albo ZUS), bez zaznaczonego na etacie pola „Zgoda na pracę 8h”, nie może mieć zaplanowanych więcej niż 7:00 na dobę. Podpięty jako Błąd do kalendarzy klienta, w tym wersji _N dla osób z niepełnosprawnością. Test 15.10.2026 na bazie Al, pracownicy NP1–NP9 (ImportyXML/Weryfikator brak zgody 8h - pracownicy i plan.xml; orzeczenia dodane w programie). Powtórka 19.10.2026 po poprawce odczytu stopnia (orzeczenie obowiązujące w danym dniu) i po podpięciu kalendarzy klienta _N: bez zgody - Podstawowy system_1_8:15_N (norma 7:00), ze zgodą / stopień lekki / bez orzeczenia - Podstawowy system_1_8:16_N (norma 8:00), system równoważny - Równoważny system_3_8:15_N (norma 7:00).</t>
+    <t>Weryfikator dnia planu pracy (Dzień planu), definicja „A1_Brak zgody na pracę 8h”. Pracownik ze stopniem umiarkowanym lub znacznym (z danych ubezpieczeniowych albo PFRON), bez zaznaczonego na etacie pola „Zgoda na pracę 8h”, nie może mieć zaplanowanych więcej niż 7:00 na dobę. Podpięty jako Błąd do kalendarzy klienta, w tym wersji _N dla osób z niepełnosprawnością. Test 15.10.2026 na bazie Al, pracownicy NP1–NP9 (ImportyXML/Weryfikator brak zgody 8h - pracownicy i plan.xml; orzeczenia dodane w programie). Powtórka 19.10.2026 po poprawce odczytu stopnia (orzeczenie obowiązujące w danym dniu) i po podpięciu kalendarzy klienta _N: bez zgody - Podstawowy system_1_8:15_N (norma 7:00), ze zgodą / stopień lekki / bez orzeczenia - Podstawowy system_1_8:16_N (norma 8:00), system równoważny - Równoważny system_3_8:15_N (norma 7:00).</t>
   </si>
   <si>
     <t>Umiarkowany, bez zgody, plan 8:00</t>
@@ -817,7 +817,7 @@
     <t>Dla dnia (13.11.2026) zaplanowano czas (8:00), a pracownik bez zgody na pracę 8h (stopień niepełnosprawności Umiarkowany) może pracować maksymalnie 7:00 - (pracownik)</t>
   </si>
   <si>
-    <t>Test 15.10.2026: negatywny (brak komunikatu - stopień czytany z historii pracownika, które w enova 2610 zwracają jedno orzeczenie z zapisu historii). Poprawka 19.10.2026: stopień z metody enova Pracownik.StopienNiepelnosprawnosciNaDzien. Powtórka 19.10.2026 (kal. 8:15_N): komunikat jak oczekiwany, razem z błędem normy dobowej (7:00).</t>
+    <t>Test 15.10.2026: negatywny (brak komunikatu - stopień czytany z historii pracownika, które w enova 2610 zwracają jedno orzeczenie z zapisu historii). Poprawka 19.10.2026: stopień z metody enova Pracownik.StopienNiepelnosprawnosciNaDzien. 20.10.2026: klient ma enova 2512.10.12, w której tej metody nie ma - stopień znowu z zapisu historii obowiązującego w dniu (w 2512 każdy zapis historii ma własne dane o niepełnosprawności, więc problem z 2610 nie występuje; w bazie testowej 2610 scenariusz pozostaje negatywny). Powtórka 19.10.2026 (kal. 8:15_N): komunikat jak oczekiwany, razem z błędem normy dobowej (7:00).</t>
   </si>
   <si>
     <t>Zmiana stopnia w miesiącu – dzień po zmianie</t>
@@ -855,7 +855,7 @@
     <t>Weryfikatory: Brak zgody na nadgodziny / Brak zgody na pracę w nocy</t>
   </si>
   <si>
-    <t>Trzy weryfikatory zgód osoby z niepełnosprawnością (każdy stopień - orzeczenie PFRON albo ZUS obowiązujące w dniu), zgody czytane z etatu w zapisie historii obowiązującym w dniu: „A1_Brak zgody na pracę w nocy (plan)” (Dzień planu, Błąd) - praca zaplanowana w porze nocnej bez zgody na pracę w porze nocnej; „A1_Brak zgody na pracę w nocy (czas)” (Dzień pracy, Ostrzeżenie) - praca w porze nocnej wpisana w czasie pracy; „A1_Brak zgody na nadgodziny” (Dzień pracy, Ostrzeżenie) - czas pracy dnia ponad większą z wartości: plan dnia i norma dobowa z etatu (w dniu wolnym wg planu - każda praca). Pora nocna z kalendarza etatu (w kalendarzach klienta _N: 22:00-6:00). Test 19.10.2026 na bazie Al, pracownicy NP1-NP6 (kalendarze _N; NP4 ma zgody na nadgodziny i pracę w nocy); dni pracy: ImportyXML/Weryfikatory zgod niepelnosprawnych - dni pracy.xml. Zmiany wpisywane w programie i wycofywane bez zapisu.</t>
+    <t>Trzy weryfikatory zgód osoby z niepełnosprawnością (każdy stopień - z danych ubezpieczeniowych albo PFRON obowiązujących w dniu), zgody czytane z etatu w zapisie historii obowiązującym w dniu: „A1_Brak zgody na pracę w nocy (plan)” (Dzień planu, Błąd) - praca zaplanowana w porze nocnej bez zgody na pracę w porze nocnej; „A1_Brak zgody na pracę w nocy (czas)” (Dzień pracy, Ostrzeżenie) - praca w porze nocnej wpisana w czasie pracy; „A1_Brak zgody na nadgodziny” (Dzień pracy, Ostrzeżenie) - czas pracy dnia ponad większą z wartości: plan dnia i norma dobowa z etatu (w dniu wolnym wg planu - każda praca). Pora nocna z kalendarza etatu (w kalendarzach klienta _N: 22:00-6:00). Test 19.10.2026 na bazie Al, pracownicy NP1-NP6 (kalendarze _N; NP4 ma zgody na nadgodziny i pracę w nocy); dni pracy: ImportyXML/Weryfikatory zgod niepelnosprawnych - dni pracy.xml. Zmiany wpisywane w programie i wycofywane bez zapisu.</t>
   </si>
   <si>
     <t>Plan w nocy - umiarkowany, bez zgody</t>

</xml_diff>

<commit_message>
Weryfikatory czasu pracy: sekcje i arkusze niepelnosprawnych usuniete ze wspolnej instrukcji i arkusza (odsylacz do Niepelnosprawni)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01H918m5sg9GbnyH8qFXz1MS
</commit_message>
<xml_diff>
--- a/Weryfikatory czasu pracy/Scenariusze testowe weryfikatorow czasu pracy.xlsx
+++ b/Weryfikatory czasu pracy/Scenariusze testowe weryfikatorow czasu pracy.xlsx
@@ -8,7 +8,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" firstSheet="2" activeTab="9"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Informacje" sheetId="1" r:id="rId1"/>
@@ -18,9 +18,6 @@
     <sheet name="Norma dobowa" sheetId="5" r:id="rId5"/>
     <sheet name="Praca w normie wg planu" sheetId="9" r:id="rId6"/>
     <sheet name="Magazyn nadgodzin - umowy" sheetId="11" r:id="rId7"/>
-    <sheet name="Brak zgody 8h" sheetId="12" r:id="rId8"/>
-    <sheet name="Zgody nadgodziny i noc" sheetId="13" r:id="rId9"/>
-    <sheet name="Norma tygodniowa 35-40h" sheetId="14" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Okres zatrudnienia'!$A$4:$G$13</definedName>
@@ -29,16 +26,13 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Norma dobowa'!$A$4:$G$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Praca w normie wg planu'!$A$4:$G$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Magazyn nadgodzin - umowy'!$A$4:$G$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Brak zgody 8h'!$A$4:$G$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Zgody nadgodziny i noc'!$A$4:$G$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Norma tygodniowa 35-40h'!$A$4:$G$14</definedName>
   </definedNames>
   <calcPr/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="362">
   <si>
     <t>Scenariusze testowe – weryfikatory czasu pracy</t>
   </si>
@@ -1185,6 +1179,12 @@
   </si>
   <si>
     <t>Uwagi: 1) Kalendarze klienta _N nie generują planu z definicji kalendarza - w danych testowych każdy dzień roboczy ma jawny plan. 2) Poziom Błąd/Ostrzeżenie ustawia się na zakładce Weryfikatory kalendarza (podpięcie), bez zmian w kodzie. 3) Weryfikator nie uruchamia się przy zmianie kalendarza na etacie ani orzeczenia - dopiero przy edycji planu.</t>
+  </si>
+  <si>
+    <t>Zakres: sześć weryfikatorów z folderu „Weryfikatory czasu pracy”, każdy na osobnym arkuszu.</t>
+  </si>
+  <si>
+    <t>• Weryfikatory osób z niepełnosprawnością – osobny plik: Niepelnosprawni\Scenariusze testowe weryfikatorow niepelnosprawnych.xlsx.</t>
   </si>
 </sst>
 </file>
@@ -1641,7 +1641,7 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>1</v>
+        <v>360</v>
       </c>
     </row>
     <row r="4">
@@ -1686,7 +1686,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>10</v>
+        <v>361</v>
       </c>
     </row>
     <row r="13">
@@ -1735,341 +1735,6 @@
       </c>
     </row>
   </sheetData>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="5.7109375" customWidth="1"/>
-    <col min="2" max="2" width="34.710938" customWidth="1"/>
-    <col min="3" max="3" width="40.710938" customWidth="1"/>
-    <col min="4" max="4" width="44.710938" customWidth="1"/>
-    <col min="5" max="5" width="46.710938" customWidth="1"/>
-    <col min="6" max="6" width="18.710938" customWidth="1"/>
-    <col min="7" max="7" width="26.710938" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="17.25">
-      <c r="A1" s="3" t="s">
-        <v>311</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="s">
-        <v>312</v>
-      </c>
-    </row>
-    <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="5" ht="75">
-      <c r="A5" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="B5" s="7" t="s">
-        <v>313</v>
-      </c>
-      <c r="C5" s="7" t="s">
-        <v>314</v>
-      </c>
-      <c r="D5" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="E5" s="9" t="s">
-        <v>315</v>
-      </c>
-      <c r="F5" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="G5" s="10" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6" ht="60">
-      <c r="A6" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="B6" s="7" t="s">
-        <v>316</v>
-      </c>
-      <c r="C6" s="7" t="s">
-        <v>317</v>
-      </c>
-      <c r="D6" s="8" t="s">
-        <v>260</v>
-      </c>
-      <c r="E6" s="9" t="s">
-        <v>318</v>
-      </c>
-      <c r="F6" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="G6" s="10" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="7" ht="75">
-      <c r="A7" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="B7" s="7" t="s">
-        <v>320</v>
-      </c>
-      <c r="C7" s="7" t="s">
-        <v>321</v>
-      </c>
-      <c r="D7" s="8" t="s">
-        <v>260</v>
-      </c>
-      <c r="E7" s="9" t="s">
-        <v>322</v>
-      </c>
-      <c r="F7" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="G7" s="10" t="s">
-        <v>323</v>
-      </c>
-    </row>
-    <row r="8" ht="75">
-      <c r="A8" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="B8" s="7" t="s">
-        <v>324</v>
-      </c>
-      <c r="C8" s="7" t="s">
-        <v>325</v>
-      </c>
-      <c r="D8" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="E8" s="9" t="s">
-        <v>315</v>
-      </c>
-      <c r="F8" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="G8" s="10" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="9" ht="60">
-      <c r="A9" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="B9" s="7" t="s">
-        <v>326</v>
-      </c>
-      <c r="C9" s="7" t="s">
-        <v>327</v>
-      </c>
-      <c r="D9" s="11" t="s">
-        <v>328</v>
-      </c>
-      <c r="E9" s="9" t="s">
-        <v>329</v>
-      </c>
-      <c r="F9" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="G9" s="10" t="s">
-        <v>330</v>
-      </c>
-    </row>
-    <row r="10" ht="36">
-      <c r="A10" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="B10" s="7" t="s">
-        <v>331</v>
-      </c>
-      <c r="C10" s="7" t="s">
-        <v>332</v>
-      </c>
-      <c r="D10" s="8" t="s">
-        <v>260</v>
-      </c>
-      <c r="E10" s="9" t="s">
-        <v>333</v>
-      </c>
-      <c r="F10" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="G10" s="10" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="11" ht="30">
-      <c r="A11" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="B11" s="7" t="s">
-        <v>334</v>
-      </c>
-      <c r="C11" s="7" t="s">
-        <v>335</v>
-      </c>
-      <c r="D11" s="11" t="s">
-        <v>336</v>
-      </c>
-      <c r="E11" s="9" t="s">
-        <v>337</v>
-      </c>
-      <c r="F11" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="G11" s="10" t="s">
-        <v>338</v>
-      </c>
-    </row>
-    <row r="12" ht="60">
-      <c r="A12" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="B12" s="7" t="s">
-        <v>339</v>
-      </c>
-      <c r="C12" s="7" t="s">
-        <v>340</v>
-      </c>
-      <c r="D12" s="8" t="s">
-        <v>260</v>
-      </c>
-      <c r="E12" s="9" t="s">
-        <v>341</v>
-      </c>
-      <c r="F12" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="G12" s="10" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="13" ht="60">
-      <c r="A13" s="6" t="s">
-        <v>342</v>
-      </c>
-      <c r="B13" s="7" t="s">
-        <v>343</v>
-      </c>
-      <c r="C13" s="7" t="s">
-        <v>344</v>
-      </c>
-      <c r="D13" s="8" t="s">
-        <v>345</v>
-      </c>
-      <c r="E13" s="9" t="s">
-        <v>346</v>
-      </c>
-      <c r="F13" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="G13" s="10" t="s">
-        <v>347</v>
-      </c>
-    </row>
-    <row r="14" ht="75" customHeight="1">
-      <c r="A14" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="B14" s="7" t="s">
-        <v>348</v>
-      </c>
-      <c r="C14" s="7" t="s">
-        <v>349</v>
-      </c>
-      <c r="D14" s="11" t="s">
-        <v>328</v>
-      </c>
-      <c r="E14" s="9" t="s">
-        <v>329</v>
-      </c>
-      <c r="F14" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="G14" s="10" t="s">
-        <v>350</v>
-      </c>
-    </row>
-    <row r="15" ht="90">
-      <c r="A15" s="6" t="s">
-        <v>351</v>
-      </c>
-      <c r="B15" s="7" t="s">
-        <v>352</v>
-      </c>
-      <c r="C15" s="7" t="s">
-        <v>353</v>
-      </c>
-      <c r="D15" s="11" t="s">
-        <v>328</v>
-      </c>
-      <c r="E15" s="9" t="s">
-        <v>329</v>
-      </c>
-      <c r="F15" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="G15" s="10" t="s">
-        <v>354</v>
-      </c>
-    </row>
-    <row r="16" ht="45" customHeight="1">
-      <c r="A16" s="6" t="s">
-        <v>355</v>
-      </c>
-      <c r="B16" s="7" t="s">
-        <v>356</v>
-      </c>
-      <c r="C16" s="7" t="s">
-        <v>357</v>
-      </c>
-      <c r="D16" s="8" t="s">
-        <v>260</v>
-      </c>
-      <c r="E16" s="9" t="s">
-        <v>358</v>
-      </c>
-      <c r="F16" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="G16" s="10" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="B18" s="13" t="s">
-        <v>359</v>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A4:G14"/>
-  <mergeCells count="1">
-    <mergeCell ref="B18:G18"/>
-  </mergeCells>
 </worksheet>
 </file>
 
@@ -3502,674 +3167,4 @@
   </sheetData>
   <autoFilter ref="A4:G13"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="5.7109375" customWidth="1"/>
-    <col min="2" max="2" width="34.710938" customWidth="1"/>
-    <col min="3" max="3" width="40.710938" customWidth="1"/>
-    <col min="4" max="4" width="44.710938" customWidth="1"/>
-    <col min="5" max="5" width="46.710938" customWidth="1"/>
-    <col min="6" max="6" width="18.710938" customWidth="1"/>
-    <col min="7" max="7" width="26.710938" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="17.25">
-      <c r="A1" s="3" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="5" ht="120">
-      <c r="A5" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="B5" s="7" t="s">
-        <v>217</v>
-      </c>
-      <c r="C5" s="7" t="s">
-        <v>218</v>
-      </c>
-      <c r="D5" s="8" t="s">
-        <v>175</v>
-      </c>
-      <c r="E5" s="9" t="s">
-        <v>219</v>
-      </c>
-      <c r="F5" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="G5" s="10" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="6" ht="120">
-      <c r="A6" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="B6" s="7" t="s">
-        <v>221</v>
-      </c>
-      <c r="C6" s="7" t="s">
-        <v>222</v>
-      </c>
-      <c r="D6" s="11" t="s">
-        <v>148</v>
-      </c>
-      <c r="E6" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="F6" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="G6" s="10" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="7" ht="120">
-      <c r="A7" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="B7" s="7" t="s">
-        <v>224</v>
-      </c>
-      <c r="C7" s="7" t="s">
-        <v>225</v>
-      </c>
-      <c r="D7" s="11" t="s">
-        <v>175</v>
-      </c>
-      <c r="E7" s="9" t="s">
-        <v>226</v>
-      </c>
-      <c r="F7" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="G7" s="10" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="8" ht="90">
-      <c r="A8" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="B8" s="7" t="s">
-        <v>228</v>
-      </c>
-      <c r="C8" s="7" t="s">
-        <v>229</v>
-      </c>
-      <c r="D8" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="E8" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="F8" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="G8" s="10" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="9" ht="75">
-      <c r="A9" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="B9" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="C9" s="7" t="s">
-        <v>232</v>
-      </c>
-      <c r="D9" s="8" t="s">
-        <v>233</v>
-      </c>
-      <c r="E9" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="F9" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="G9" s="10" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="10" ht="90">
-      <c r="A10" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="B10" s="7" t="s">
-        <v>235</v>
-      </c>
-      <c r="C10" s="7" t="s">
-        <v>236</v>
-      </c>
-      <c r="D10" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="E10" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="F10" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="G10" s="10" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="11" ht="105">
-      <c r="A11" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="B11" s="7" t="s">
-        <v>237</v>
-      </c>
-      <c r="C11" s="7" t="s">
-        <v>238</v>
-      </c>
-      <c r="D11" s="11" t="s">
-        <v>239</v>
-      </c>
-      <c r="E11" s="9" t="s">
-        <v>219</v>
-      </c>
-      <c r="F11" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="G11" s="10" t="s">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="12" ht="210">
-      <c r="A12" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="B12" s="7" t="s">
-        <v>241</v>
-      </c>
-      <c r="C12" s="7" t="s">
-        <v>242</v>
-      </c>
-      <c r="D12" s="8" t="s">
-        <v>243</v>
-      </c>
-      <c r="E12" s="9" t="s">
-        <v>244</v>
-      </c>
-      <c r="F12" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="G12" s="10" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="13" ht="150">
-      <c r="A13" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="B13" s="7" t="s">
-        <v>246</v>
-      </c>
-      <c r="C13" s="7" t="s">
-        <v>247</v>
-      </c>
-      <c r="D13" s="11" t="s">
-        <v>248</v>
-      </c>
-      <c r="E13" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="F13" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="G13" s="10" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="14" ht="75" customHeight="1">
-      <c r="A14" s="6" t="s">
-        <v>250</v>
-      </c>
-      <c r="B14" s="7" t="s">
-        <v>251</v>
-      </c>
-      <c r="C14" s="7" t="s">
-        <v>252</v>
-      </c>
-      <c r="D14" s="8" t="s">
-        <v>253</v>
-      </c>
-      <c r="E14" s="9" t="s">
-        <v>219</v>
-      </c>
-      <c r="F14" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="G14" s="10" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="16" ht="45" customHeight="1">
-      <c r="B16" s="13" t="s">
-        <v>255</v>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A4:G14"/>
-  <mergeCells count="1">
-    <mergeCell ref="B16:G16"/>
-  </mergeCells>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="5.7109375" customWidth="1"/>
-    <col min="2" max="2" width="34.710938" customWidth="1"/>
-    <col min="3" max="3" width="40.710938" customWidth="1"/>
-    <col min="4" max="4" width="44.710938" customWidth="1"/>
-    <col min="5" max="5" width="46.710938" customWidth="1"/>
-    <col min="6" max="6" width="18.710938" customWidth="1"/>
-    <col min="7" max="7" width="26.710938" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="17.25">
-      <c r="A1" s="3" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="s">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="5" ht="75">
-      <c r="A5" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="B5" s="7" t="s">
-        <v>258</v>
-      </c>
-      <c r="C5" s="7" t="s">
-        <v>259</v>
-      </c>
-      <c r="D5" s="8" t="s">
-        <v>260</v>
-      </c>
-      <c r="E5" s="9" t="s">
-        <v>261</v>
-      </c>
-      <c r="F5" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="G5" s="10" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="6" ht="45">
-      <c r="A6" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="B6" s="7" t="s">
-        <v>263</v>
-      </c>
-      <c r="C6" s="7" t="s">
-        <v>264</v>
-      </c>
-      <c r="D6" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="E6" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="F6" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="G6" s="10" t="s">
-        <v>265</v>
-      </c>
-    </row>
-    <row r="7" ht="30">
-      <c r="A7" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="B7" s="7" t="s">
-        <v>266</v>
-      </c>
-      <c r="C7" s="7" t="s">
-        <v>267</v>
-      </c>
-      <c r="D7" s="8" t="s">
-        <v>260</v>
-      </c>
-      <c r="E7" s="9" t="s">
-        <v>268</v>
-      </c>
-      <c r="F7" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="G7" s="10" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="8" ht="30">
-      <c r="A8" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="B8" s="7" t="s">
-        <v>269</v>
-      </c>
-      <c r="C8" s="7" t="s">
-        <v>270</v>
-      </c>
-      <c r="D8" s="8" t="s">
-        <v>260</v>
-      </c>
-      <c r="E8" s="9" t="s">
-        <v>271</v>
-      </c>
-      <c r="F8" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="G8" s="10" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="9" ht="75">
-      <c r="A9" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="B9" s="7" t="s">
-        <v>272</v>
-      </c>
-      <c r="C9" s="7" t="s">
-        <v>273</v>
-      </c>
-      <c r="D9" s="8" t="s">
-        <v>274</v>
-      </c>
-      <c r="E9" s="9" t="s">
-        <v>275</v>
-      </c>
-      <c r="F9" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="G9" s="10" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="10" ht="60">
-      <c r="A10" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="B10" s="7" t="s">
-        <v>276</v>
-      </c>
-      <c r="C10" s="7" t="s">
-        <v>277</v>
-      </c>
-      <c r="D10" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="E10" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="F10" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="G10" s="10" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="11" ht="90">
-      <c r="A11" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="B11" s="7" t="s">
-        <v>278</v>
-      </c>
-      <c r="C11" s="7" t="s">
-        <v>279</v>
-      </c>
-      <c r="D11" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="E11" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="F11" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="G11" s="10" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="12" ht="48">
-      <c r="A12" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="B12" s="7" t="s">
-        <v>280</v>
-      </c>
-      <c r="C12" s="7" t="s">
-        <v>281</v>
-      </c>
-      <c r="D12" s="14" t="s">
-        <v>282</v>
-      </c>
-      <c r="E12" s="9" t="s">
-        <v>283</v>
-      </c>
-      <c r="F12" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="G12" s="10" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="13" ht="105">
-      <c r="A13" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="B13" s="7" t="s">
-        <v>285</v>
-      </c>
-      <c r="C13" s="7" t="s">
-        <v>286</v>
-      </c>
-      <c r="D13" s="11" t="s">
-        <v>287</v>
-      </c>
-      <c r="E13" s="9" t="s">
-        <v>288</v>
-      </c>
-      <c r="F13" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="G13" s="10" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="14" ht="75" customHeight="1">
-      <c r="A14" s="6" t="s">
-        <v>250</v>
-      </c>
-      <c r="B14" s="7" t="s">
-        <v>290</v>
-      </c>
-      <c r="C14" s="7" t="s">
-        <v>291</v>
-      </c>
-      <c r="D14" s="14" t="s">
-        <v>282</v>
-      </c>
-      <c r="E14" s="9" t="s">
-        <v>292</v>
-      </c>
-      <c r="F14" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="G14" s="10" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="15" ht="90">
-      <c r="A15" s="6" t="s">
-        <v>293</v>
-      </c>
-      <c r="B15" s="7" t="s">
-        <v>294</v>
-      </c>
-      <c r="C15" s="7" t="s">
-        <v>295</v>
-      </c>
-      <c r="D15" s="14" t="s">
-        <v>296</v>
-      </c>
-      <c r="E15" s="9" t="s">
-        <v>297</v>
-      </c>
-      <c r="F15" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="G15" s="10" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="16" ht="45" customHeight="1">
-      <c r="A16" s="6" t="s">
-        <v>298</v>
-      </c>
-      <c r="B16" s="7" t="s">
-        <v>299</v>
-      </c>
-      <c r="C16" s="7" t="s">
-        <v>300</v>
-      </c>
-      <c r="D16" s="14" t="s">
-        <v>301</v>
-      </c>
-      <c r="E16" s="9" t="s">
-        <v>302</v>
-      </c>
-      <c r="F16" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="G16" s="10" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="17" ht="45">
-      <c r="A17" s="6" t="s">
-        <v>303</v>
-      </c>
-      <c r="B17" s="7" t="s">
-        <v>304</v>
-      </c>
-      <c r="C17" s="7" t="s">
-        <v>305</v>
-      </c>
-      <c r="D17" s="11" t="s">
-        <v>306</v>
-      </c>
-      <c r="E17" s="9" t="s">
-        <v>288</v>
-      </c>
-      <c r="F17" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="G17" s="10" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="18" ht="30">
-      <c r="A18" s="6" t="s">
-        <v>307</v>
-      </c>
-      <c r="B18" s="7" t="s">
-        <v>308</v>
-      </c>
-      <c r="C18" s="7" t="s">
-        <v>309</v>
-      </c>
-      <c r="D18" s="11" t="s">
-        <v>306</v>
-      </c>
-      <c r="E18" s="9" t="s">
-        <v>288</v>
-      </c>
-      <c r="F18" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="G18" s="10" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="B20" s="13" t="s">
-        <v>310</v>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A4:G14"/>
-  <mergeCells count="1">
-    <mergeCell ref="B20:G20"/>
-  </mergeCells>
-</worksheet>
 </file>
</xml_diff>